<commit_message>
state: bot run 2026-09-08T08:04 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_india.xlsx
+++ b/data/trade_log_india.xlsx
@@ -431,61 +431,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K353"/>
+  <dimension ref="A1:K453"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Close</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>SMA20</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Upper_Band</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>EMA9</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>EMA21</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Vol_Ratio</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Qualifies</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Rejection_Or_Status</t>
         </is>
@@ -15604,6 +15604,4306 @@
         <v>0</v>
       </c>
       <c r="K353" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1156.90 &lt;= Upper 1209.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+      <c r="D354" t="n">
+        <v>7410</v>
+      </c>
+      <c r="E354" t="n">
+        <v>7758.99</v>
+      </c>
+      <c r="F354" t="n">
+        <v>7758.99</v>
+      </c>
+      <c r="G354" t="n">
+        <v>7476.85</v>
+      </c>
+      <c r="H354" t="n">
+        <v>7484.06</v>
+      </c>
+      <c r="I354" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="J354" t="b">
+        <v>0</v>
+      </c>
+      <c r="K354" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7476.85 &lt;= EMA21 7484.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="D355" t="n">
+        <v>1390.4</v>
+      </c>
+      <c r="E355" t="n">
+        <v>1708.69</v>
+      </c>
+      <c r="F355" t="n">
+        <v>1708.69</v>
+      </c>
+      <c r="G355" t="n">
+        <v>1445.34</v>
+      </c>
+      <c r="H355" t="n">
+        <v>1510.18</v>
+      </c>
+      <c r="I355" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="J355" t="b">
+        <v>0</v>
+      </c>
+      <c r="K355" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1445.34 &lt;= EMA21 1510.18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>ADANIENT</t>
+        </is>
+      </c>
+      <c r="D356" t="n">
+        <v>2950</v>
+      </c>
+      <c r="E356" t="n">
+        <v>3174.75</v>
+      </c>
+      <c r="F356" t="n">
+        <v>3174.75</v>
+      </c>
+      <c r="G356" t="n">
+        <v>2958.78</v>
+      </c>
+      <c r="H356" t="n">
+        <v>2992.12</v>
+      </c>
+      <c r="I356" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J356" t="b">
+        <v>0</v>
+      </c>
+      <c r="K356" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2958.78 &lt;= EMA21 2992.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>ADANIGREEN</t>
+        </is>
+      </c>
+      <c r="D357" t="n">
+        <v>1288</v>
+      </c>
+      <c r="E357" t="n">
+        <v>1370.67</v>
+      </c>
+      <c r="F357" t="n">
+        <v>1370.67</v>
+      </c>
+      <c r="G357" t="n">
+        <v>1291.88</v>
+      </c>
+      <c r="H357" t="n">
+        <v>1315.87</v>
+      </c>
+      <c r="I357" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="J357" t="b">
+        <v>0</v>
+      </c>
+      <c r="K357" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1291.88 &lt;= EMA21 1315.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="D358" t="n">
+        <v>1707.3</v>
+      </c>
+      <c r="E358" t="n">
+        <v>1737.54</v>
+      </c>
+      <c r="F358" t="n">
+        <v>1737.54</v>
+      </c>
+      <c r="G358" t="n">
+        <v>1684.09</v>
+      </c>
+      <c r="H358" t="n">
+        <v>1692.4</v>
+      </c>
+      <c r="I358" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J358" t="b">
+        <v>0</v>
+      </c>
+      <c r="K358" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1684.09 &lt;= EMA21 1692.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="D359" t="n">
+        <v>204.49</v>
+      </c>
+      <c r="E359" t="n">
+        <v>213.26</v>
+      </c>
+      <c r="F359" t="n">
+        <v>213.26</v>
+      </c>
+      <c r="G359" t="n">
+        <v>206.4</v>
+      </c>
+      <c r="H359" t="n">
+        <v>207.39</v>
+      </c>
+      <c r="I359" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="J359" t="b">
+        <v>0</v>
+      </c>
+      <c r="K359" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 206.40 &lt;= EMA21 207.39)</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>AMBUJACEM</t>
+        </is>
+      </c>
+      <c r="D360" t="n">
+        <v>398.6</v>
+      </c>
+      <c r="E360" t="n">
+        <v>425.38</v>
+      </c>
+      <c r="F360" t="n">
+        <v>425.38</v>
+      </c>
+      <c r="G360" t="n">
+        <v>405.41</v>
+      </c>
+      <c r="H360" t="n">
+        <v>411.83</v>
+      </c>
+      <c r="I360" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="J360" t="b">
+        <v>0</v>
+      </c>
+      <c r="K360" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 405.41 &lt;= EMA21 411.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="D361" t="n">
+        <v>8650</v>
+      </c>
+      <c r="E361" t="n">
+        <v>8959.780000000001</v>
+      </c>
+      <c r="F361" t="n">
+        <v>8959.780000000001</v>
+      </c>
+      <c r="G361" t="n">
+        <v>8743.82</v>
+      </c>
+      <c r="H361" t="n">
+        <v>8774.309999999999</v>
+      </c>
+      <c r="I361" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J361" t="b">
+        <v>0</v>
+      </c>
+      <c r="K361" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 8743.82 &lt;= EMA21 8774.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="D362" t="n">
+        <v>2500.9</v>
+      </c>
+      <c r="E362" t="n">
+        <v>2773.19</v>
+      </c>
+      <c r="F362" t="n">
+        <v>2773.19</v>
+      </c>
+      <c r="G362" t="n">
+        <v>2565.82</v>
+      </c>
+      <c r="H362" t="n">
+        <v>2616.42</v>
+      </c>
+      <c r="I362" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J362" t="b">
+        <v>0</v>
+      </c>
+      <c r="K362" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2565.82 &lt;= EMA21 2616.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="D363" t="n">
+        <v>3710</v>
+      </c>
+      <c r="E363" t="n">
+        <v>4123.46</v>
+      </c>
+      <c r="F363" t="n">
+        <v>4123.46</v>
+      </c>
+      <c r="G363" t="n">
+        <v>3807.79</v>
+      </c>
+      <c r="H363" t="n">
+        <v>3875.23</v>
+      </c>
+      <c r="I363" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J363" t="b">
+        <v>0</v>
+      </c>
+      <c r="K363" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3807.79 &lt;= EMA21 3875.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="D364" t="n">
+        <v>1273</v>
+      </c>
+      <c r="E364" t="n">
+        <v>1286.96</v>
+      </c>
+      <c r="F364" t="n">
+        <v>1286.96</v>
+      </c>
+      <c r="G364" t="n">
+        <v>1262.24</v>
+      </c>
+      <c r="H364" t="n">
+        <v>1256.46</v>
+      </c>
+      <c r="I364" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J364" t="b">
+        <v>0</v>
+      </c>
+      <c r="K364" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1273.00 &lt;= Upper 1286.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO</t>
+        </is>
+      </c>
+      <c r="D365" t="n">
+        <v>11800</v>
+      </c>
+      <c r="E365" t="n">
+        <v>12216.74</v>
+      </c>
+      <c r="F365" t="n">
+        <v>12216.74</v>
+      </c>
+      <c r="G365" t="n">
+        <v>11928.25</v>
+      </c>
+      <c r="H365" t="n">
+        <v>11784.64</v>
+      </c>
+      <c r="I365" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J365" t="b">
+        <v>0</v>
+      </c>
+      <c r="K365" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 11800.00 &lt;= Upper 12216.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="D366" t="n">
+        <v>1060</v>
+      </c>
+      <c r="E366" t="n">
+        <v>1110.38</v>
+      </c>
+      <c r="F366" t="n">
+        <v>1110.38</v>
+      </c>
+      <c r="G366" t="n">
+        <v>1064.37</v>
+      </c>
+      <c r="H366" t="n">
+        <v>1072.1</v>
+      </c>
+      <c r="I366" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J366" t="b">
+        <v>0</v>
+      </c>
+      <c r="K366" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1064.37 &lt;= EMA21 1072.10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="D367" t="n">
+        <v>1938.6</v>
+      </c>
+      <c r="E367" t="n">
+        <v>2049.09</v>
+      </c>
+      <c r="F367" t="n">
+        <v>2049.09</v>
+      </c>
+      <c r="G367" t="n">
+        <v>1982.62</v>
+      </c>
+      <c r="H367" t="n">
+        <v>1989.57</v>
+      </c>
+      <c r="I367" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J367" t="b">
+        <v>0</v>
+      </c>
+      <c r="K367" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1982.62 &lt;= EMA21 1989.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>BAJAJHLDNG</t>
+        </is>
+      </c>
+      <c r="D368" t="n">
+        <v>10956</v>
+      </c>
+      <c r="E368" t="n">
+        <v>11700.43</v>
+      </c>
+      <c r="F368" t="n">
+        <v>11700.43</v>
+      </c>
+      <c r="G368" t="n">
+        <v>11210.6</v>
+      </c>
+      <c r="H368" t="n">
+        <v>11243.44</v>
+      </c>
+      <c r="I368" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J368" t="b">
+        <v>0</v>
+      </c>
+      <c r="K368" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11210.60 &lt;= EMA21 11243.44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>BANKBARODA</t>
+        </is>
+      </c>
+      <c r="D369" t="n">
+        <v>237</v>
+      </c>
+      <c r="E369" t="n">
+        <v>250.83</v>
+      </c>
+      <c r="F369" t="n">
+        <v>250.83</v>
+      </c>
+      <c r="G369" t="n">
+        <v>239.96</v>
+      </c>
+      <c r="H369" t="n">
+        <v>242.44</v>
+      </c>
+      <c r="I369" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J369" t="b">
+        <v>0</v>
+      </c>
+      <c r="K369" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 239.96 &lt;= EMA21 242.44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="D370" t="n">
+        <v>404</v>
+      </c>
+      <c r="E370" t="n">
+        <v>415.89</v>
+      </c>
+      <c r="F370" t="n">
+        <v>415.89</v>
+      </c>
+      <c r="G370" t="n">
+        <v>407.85</v>
+      </c>
+      <c r="H370" t="n">
+        <v>407.67</v>
+      </c>
+      <c r="I370" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J370" t="b">
+        <v>0</v>
+      </c>
+      <c r="K370" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 404.00 &lt;= Upper 415.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>BPCL</t>
+        </is>
+      </c>
+      <c r="D371" t="n">
+        <v>312.9</v>
+      </c>
+      <c r="E371" t="n">
+        <v>324.56</v>
+      </c>
+      <c r="F371" t="n">
+        <v>324.56</v>
+      </c>
+      <c r="G371" t="n">
+        <v>316.92</v>
+      </c>
+      <c r="H371" t="n">
+        <v>316.68</v>
+      </c>
+      <c r="I371" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="J371" t="b">
+        <v>0</v>
+      </c>
+      <c r="K371" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 312.90 &lt;= Upper 324.56)</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="D372" t="n">
+        <v>1854</v>
+      </c>
+      <c r="E372" t="n">
+        <v>2002.01</v>
+      </c>
+      <c r="F372" t="n">
+        <v>2002.01</v>
+      </c>
+      <c r="G372" t="n">
+        <v>1869.91</v>
+      </c>
+      <c r="H372" t="n">
+        <v>1894.43</v>
+      </c>
+      <c r="I372" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J372" t="b">
+        <v>0</v>
+      </c>
+      <c r="K372" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1869.91 &lt;= EMA21 1894.43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>BOSCHLTD</t>
+        </is>
+      </c>
+      <c r="D373" t="n">
+        <v>48025</v>
+      </c>
+      <c r="E373" t="n">
+        <v>50126.21</v>
+      </c>
+      <c r="F373" t="n">
+        <v>50126.21</v>
+      </c>
+      <c r="G373" t="n">
+        <v>47830.73</v>
+      </c>
+      <c r="H373" t="n">
+        <v>47030.6</v>
+      </c>
+      <c r="I373" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="J373" t="b">
+        <v>0</v>
+      </c>
+      <c r="K373" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 48025.00 &lt;= Upper 50126.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>BRITANNIA</t>
+        </is>
+      </c>
+      <c r="D374" t="n">
+        <v>5042.5</v>
+      </c>
+      <c r="E374" t="n">
+        <v>5732.79</v>
+      </c>
+      <c r="F374" t="n">
+        <v>5732.79</v>
+      </c>
+      <c r="G374" t="n">
+        <v>5187.11</v>
+      </c>
+      <c r="H374" t="n">
+        <v>5290.28</v>
+      </c>
+      <c r="I374" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J374" t="b">
+        <v>0</v>
+      </c>
+      <c r="K374" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5187.11 &lt;= EMA21 5290.28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="D375" t="n">
+        <v>895</v>
+      </c>
+      <c r="E375" t="n">
+        <v>911.33</v>
+      </c>
+      <c r="F375" t="n">
+        <v>911.33</v>
+      </c>
+      <c r="G375" t="n">
+        <v>889.72</v>
+      </c>
+      <c r="H375" t="n">
+        <v>886.63</v>
+      </c>
+      <c r="I375" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="J375" t="b">
+        <v>0</v>
+      </c>
+      <c r="K375" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 895.00 &lt;= Upper 911.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>CANBK</t>
+        </is>
+      </c>
+      <c r="D376" t="n">
+        <v>124</v>
+      </c>
+      <c r="E376" t="n">
+        <v>133.1</v>
+      </c>
+      <c r="F376" t="n">
+        <v>133.1</v>
+      </c>
+      <c r="G376" t="n">
+        <v>126.32</v>
+      </c>
+      <c r="H376" t="n">
+        <v>127.45</v>
+      </c>
+      <c r="I376" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J376" t="b">
+        <v>0</v>
+      </c>
+      <c r="K376" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 126.32 &lt;= EMA21 127.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="D377" t="n">
+        <v>1839</v>
+      </c>
+      <c r="E377" t="n">
+        <v>1935.31</v>
+      </c>
+      <c r="F377" t="n">
+        <v>1935.31</v>
+      </c>
+      <c r="G377" t="n">
+        <v>1848.54</v>
+      </c>
+      <c r="H377" t="n">
+        <v>1853.3</v>
+      </c>
+      <c r="I377" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J377" t="b">
+        <v>0</v>
+      </c>
+      <c r="K377" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1848.54 &lt;= EMA21 1853.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>CIPLA</t>
+        </is>
+      </c>
+      <c r="D378" t="n">
+        <v>1385</v>
+      </c>
+      <c r="E378" t="n">
+        <v>1475.34</v>
+      </c>
+      <c r="F378" t="n">
+        <v>1475.34</v>
+      </c>
+      <c r="G378" t="n">
+        <v>1409.71</v>
+      </c>
+      <c r="H378" t="n">
+        <v>1423.28</v>
+      </c>
+      <c r="I378" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="J378" t="b">
+        <v>0</v>
+      </c>
+      <c r="K378" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1409.71 &lt;= EMA21 1423.28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="D379" t="n">
+        <v>418.85</v>
+      </c>
+      <c r="E379" t="n">
+        <v>417.6</v>
+      </c>
+      <c r="F379" t="n">
+        <v>417.6</v>
+      </c>
+      <c r="G379" t="n">
+        <v>408.59</v>
+      </c>
+      <c r="H379" t="n">
+        <v>406.28</v>
+      </c>
+      <c r="I379" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="J379" t="b">
+        <v>1</v>
+      </c>
+      <c r="K379" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>CUMMINSIND</t>
+        </is>
+      </c>
+      <c r="D380" t="n">
+        <v>5035</v>
+      </c>
+      <c r="E380" t="n">
+        <v>5493.34</v>
+      </c>
+      <c r="F380" t="n">
+        <v>5493.34</v>
+      </c>
+      <c r="G380" t="n">
+        <v>5124.14</v>
+      </c>
+      <c r="H380" t="n">
+        <v>5222.06</v>
+      </c>
+      <c r="I380" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J380" t="b">
+        <v>0</v>
+      </c>
+      <c r="K380" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5124.14 &lt;= EMA21 5222.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>DLF</t>
+        </is>
+      </c>
+      <c r="D381" t="n">
+        <v>681.9</v>
+      </c>
+      <c r="E381" t="n">
+        <v>693.6</v>
+      </c>
+      <c r="F381" t="n">
+        <v>693.6</v>
+      </c>
+      <c r="G381" t="n">
+        <v>678.76</v>
+      </c>
+      <c r="H381" t="n">
+        <v>672.58</v>
+      </c>
+      <c r="I381" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J381" t="b">
+        <v>0</v>
+      </c>
+      <c r="K381" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 681.90 &lt;= Upper 693.60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>DIVISLAB</t>
+        </is>
+      </c>
+      <c r="D382" t="n">
+        <v>9315</v>
+      </c>
+      <c r="E382" t="n">
+        <v>9539.43</v>
+      </c>
+      <c r="F382" t="n">
+        <v>9539.43</v>
+      </c>
+      <c r="G382" t="n">
+        <v>9133.26</v>
+      </c>
+      <c r="H382" t="n">
+        <v>8822.08</v>
+      </c>
+      <c r="I382" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J382" t="b">
+        <v>0</v>
+      </c>
+      <c r="K382" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 9315.00 &lt;= Upper 9539.43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="D383" t="n">
+        <v>1144.2</v>
+      </c>
+      <c r="E383" t="n">
+        <v>1215.31</v>
+      </c>
+      <c r="F383" t="n">
+        <v>1215.31</v>
+      </c>
+      <c r="G383" t="n">
+        <v>1160.7</v>
+      </c>
+      <c r="H383" t="n">
+        <v>1172.45</v>
+      </c>
+      <c r="I383" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="J383" t="b">
+        <v>0</v>
+      </c>
+      <c r="K383" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1160.70 &lt;= EMA21 1172.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>EICHERMOT</t>
+        </is>
+      </c>
+      <c r="D384" t="n">
+        <v>7630.5</v>
+      </c>
+      <c r="E384" t="n">
+        <v>8249.530000000001</v>
+      </c>
+      <c r="F384" t="n">
+        <v>8249.530000000001</v>
+      </c>
+      <c r="G384" t="n">
+        <v>7847.75</v>
+      </c>
+      <c r="H384" t="n">
+        <v>7893.15</v>
+      </c>
+      <c r="I384" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="J384" t="b">
+        <v>0</v>
+      </c>
+      <c r="K384" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7847.75 &lt;= EMA21 7893.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>ETERNAL</t>
+        </is>
+      </c>
+      <c r="D385" t="n">
+        <v>322.75</v>
+      </c>
+      <c r="E385" t="n">
+        <v>334.92</v>
+      </c>
+      <c r="F385" t="n">
+        <v>334.92</v>
+      </c>
+      <c r="G385" t="n">
+        <v>325.57</v>
+      </c>
+      <c r="H385" t="n">
+        <v>321.06</v>
+      </c>
+      <c r="I385" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="J385" t="b">
+        <v>0</v>
+      </c>
+      <c r="K385" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 322.75 &lt;= Upper 334.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>GAIL</t>
+        </is>
+      </c>
+      <c r="D386" t="n">
+        <v>176</v>
+      </c>
+      <c r="E386" t="n">
+        <v>177.46</v>
+      </c>
+      <c r="F386" t="n">
+        <v>177.46</v>
+      </c>
+      <c r="G386" t="n">
+        <v>173.99</v>
+      </c>
+      <c r="H386" t="n">
+        <v>173.69</v>
+      </c>
+      <c r="I386" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="J386" t="b">
+        <v>0</v>
+      </c>
+      <c r="K386" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 176.00 &lt;= Upper 177.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>GODREJCP</t>
+        </is>
+      </c>
+      <c r="D387" t="n">
+        <v>861.9</v>
+      </c>
+      <c r="E387" t="n">
+        <v>984.8200000000001</v>
+      </c>
+      <c r="F387" t="n">
+        <v>984.8200000000001</v>
+      </c>
+      <c r="G387" t="n">
+        <v>895.74</v>
+      </c>
+      <c r="H387" t="n">
+        <v>929.87</v>
+      </c>
+      <c r="I387" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J387" t="b">
+        <v>0</v>
+      </c>
+      <c r="K387" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 895.74 &lt;= EMA21 929.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>GRASIM</t>
+        </is>
+      </c>
+      <c r="D388" t="n">
+        <v>3322</v>
+      </c>
+      <c r="E388" t="n">
+        <v>3367.26</v>
+      </c>
+      <c r="F388" t="n">
+        <v>3367.26</v>
+      </c>
+      <c r="G388" t="n">
+        <v>3305.75</v>
+      </c>
+      <c r="H388" t="n">
+        <v>3279.8</v>
+      </c>
+      <c r="I388" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J388" t="b">
+        <v>0</v>
+      </c>
+      <c r="K388" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3322.00 &lt;= Upper 3367.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="D389" t="n">
+        <v>1282.8</v>
+      </c>
+      <c r="E389" t="n">
+        <v>1377.25</v>
+      </c>
+      <c r="F389" t="n">
+        <v>1377.25</v>
+      </c>
+      <c r="G389" t="n">
+        <v>1309.38</v>
+      </c>
+      <c r="H389" t="n">
+        <v>1311.49</v>
+      </c>
+      <c r="I389" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="J389" t="b">
+        <v>0</v>
+      </c>
+      <c r="K389" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1309.38 &lt;= EMA21 1311.49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>HDFCAMC</t>
+        </is>
+      </c>
+      <c r="D390" t="n">
+        <v>2458.3</v>
+      </c>
+      <c r="E390" t="n">
+        <v>2686.64</v>
+      </c>
+      <c r="F390" t="n">
+        <v>2686.64</v>
+      </c>
+      <c r="G390" t="n">
+        <v>2543.04</v>
+      </c>
+      <c r="H390" t="n">
+        <v>2562.35</v>
+      </c>
+      <c r="I390" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J390" t="b">
+        <v>0</v>
+      </c>
+      <c r="K390" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2543.04 &lt;= EMA21 2562.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="D391" t="n">
+        <v>710.5</v>
+      </c>
+      <c r="E391" t="n">
+        <v>738.1</v>
+      </c>
+      <c r="F391" t="n">
+        <v>738.1</v>
+      </c>
+      <c r="G391" t="n">
+        <v>712.6900000000001</v>
+      </c>
+      <c r="H391" t="n">
+        <v>721.96</v>
+      </c>
+      <c r="I391" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="J391" t="b">
+        <v>0</v>
+      </c>
+      <c r="K391" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 712.69 &lt;= EMA21 721.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="D392" t="n">
+        <v>533.2</v>
+      </c>
+      <c r="E392" t="n">
+        <v>555.87</v>
+      </c>
+      <c r="F392" t="n">
+        <v>555.87</v>
+      </c>
+      <c r="G392" t="n">
+        <v>540.26</v>
+      </c>
+      <c r="H392" t="n">
+        <v>543.27</v>
+      </c>
+      <c r="I392" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="J392" t="b">
+        <v>0</v>
+      </c>
+      <c r="K392" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 540.26 &lt;= EMA21 543.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="D393" t="n">
+        <v>1011</v>
+      </c>
+      <c r="E393" t="n">
+        <v>1074.54</v>
+      </c>
+      <c r="F393" t="n">
+        <v>1074.54</v>
+      </c>
+      <c r="G393" t="n">
+        <v>1020.94</v>
+      </c>
+      <c r="H393" t="n">
+        <v>1023.12</v>
+      </c>
+      <c r="I393" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J393" t="b">
+        <v>0</v>
+      </c>
+      <c r="K393" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1020.94 &lt;= EMA21 1023.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="D394" t="n">
+        <v>4856</v>
+      </c>
+      <c r="E394" t="n">
+        <v>5109.33</v>
+      </c>
+      <c r="F394" t="n">
+        <v>5109.33</v>
+      </c>
+      <c r="G394" t="n">
+        <v>4841.36</v>
+      </c>
+      <c r="H394" t="n">
+        <v>4841.16</v>
+      </c>
+      <c r="I394" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="J394" t="b">
+        <v>0</v>
+      </c>
+      <c r="K394" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 4856.00 &lt;= Upper 5109.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="D395" t="n">
+        <v>1973.4</v>
+      </c>
+      <c r="E395" t="n">
+        <v>2103.52</v>
+      </c>
+      <c r="F395" t="n">
+        <v>2103.52</v>
+      </c>
+      <c r="G395" t="n">
+        <v>1990.81</v>
+      </c>
+      <c r="H395" t="n">
+        <v>2023.26</v>
+      </c>
+      <c r="I395" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="J395" t="b">
+        <v>0</v>
+      </c>
+      <c r="K395" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1990.81 &lt;= EMA21 2023.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+      <c r="D396" t="n">
+        <v>589.15</v>
+      </c>
+      <c r="E396" t="n">
+        <v>627.27</v>
+      </c>
+      <c r="F396" t="n">
+        <v>627.27</v>
+      </c>
+      <c r="G396" t="n">
+        <v>594.85</v>
+      </c>
+      <c r="H396" t="n">
+        <v>587.75</v>
+      </c>
+      <c r="I396" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="J396" t="b">
+        <v>0</v>
+      </c>
+      <c r="K396" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 589.15 &lt;= Upper 627.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>HYUNDAI</t>
+        </is>
+      </c>
+      <c r="D397" t="n">
+        <v>2205</v>
+      </c>
+      <c r="E397" t="n">
+        <v>2273.73</v>
+      </c>
+      <c r="F397" t="n">
+        <v>2273.73</v>
+      </c>
+      <c r="G397" t="n">
+        <v>2196.4</v>
+      </c>
+      <c r="H397" t="n">
+        <v>2183.83</v>
+      </c>
+      <c r="I397" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J397" t="b">
+        <v>0</v>
+      </c>
+      <c r="K397" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 2205.00 &lt;= Upper 2273.73)</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="D398" t="n">
+        <v>1427.5</v>
+      </c>
+      <c r="E398" t="n">
+        <v>1448.8</v>
+      </c>
+      <c r="F398" t="n">
+        <v>1448.8</v>
+      </c>
+      <c r="G398" t="n">
+        <v>1428.85</v>
+      </c>
+      <c r="H398" t="n">
+        <v>1426.34</v>
+      </c>
+      <c r="I398" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J398" t="b">
+        <v>0</v>
+      </c>
+      <c r="K398" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1427.50 &lt;= Upper 1448.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="D399" t="n">
+        <v>263.5</v>
+      </c>
+      <c r="E399" t="n">
+        <v>281.14</v>
+      </c>
+      <c r="F399" t="n">
+        <v>281.14</v>
+      </c>
+      <c r="G399" t="n">
+        <v>265.35</v>
+      </c>
+      <c r="H399" t="n">
+        <v>269.66</v>
+      </c>
+      <c r="I399" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="J399" t="b">
+        <v>0</v>
+      </c>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 265.35 &lt;= EMA21 269.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>INDHOTEL</t>
+        </is>
+      </c>
+      <c r="D400" t="n">
+        <v>716.2</v>
+      </c>
+      <c r="E400" t="n">
+        <v>738.45</v>
+      </c>
+      <c r="F400" t="n">
+        <v>738.45</v>
+      </c>
+      <c r="G400" t="n">
+        <v>722.9299999999999</v>
+      </c>
+      <c r="H400" t="n">
+        <v>724.97</v>
+      </c>
+      <c r="I400" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="J400" t="b">
+        <v>0</v>
+      </c>
+      <c r="K400" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 722.93 &lt;= EMA21 724.97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>IOC</t>
+        </is>
+      </c>
+      <c r="D401" t="n">
+        <v>135.15</v>
+      </c>
+      <c r="E401" t="n">
+        <v>140.7</v>
+      </c>
+      <c r="F401" t="n">
+        <v>140.7</v>
+      </c>
+      <c r="G401" t="n">
+        <v>137.19</v>
+      </c>
+      <c r="H401" t="n">
+        <v>137.94</v>
+      </c>
+      <c r="I401" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J401" t="b">
+        <v>0</v>
+      </c>
+      <c r="K401" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 137.19 &lt;= EMA21 137.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>IRFC</t>
+        </is>
+      </c>
+      <c r="D402" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="E402" t="n">
+        <v>89.65000000000001</v>
+      </c>
+      <c r="F402" t="n">
+        <v>89.65000000000001</v>
+      </c>
+      <c r="G402" t="n">
+        <v>83.78</v>
+      </c>
+      <c r="H402" t="n">
+        <v>85.31</v>
+      </c>
+      <c r="I402" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="J402" t="b">
+        <v>0</v>
+      </c>
+      <c r="K402" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 83.78 &lt;= EMA21 85.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="D403" t="n">
+        <v>1087.5</v>
+      </c>
+      <c r="E403" t="n">
+        <v>1188.43</v>
+      </c>
+      <c r="F403" t="n">
+        <v>1188.43</v>
+      </c>
+      <c r="G403" t="n">
+        <v>1125.66</v>
+      </c>
+      <c r="H403" t="n">
+        <v>1130.82</v>
+      </c>
+      <c r="I403" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J403" t="b">
+        <v>0</v>
+      </c>
+      <c r="K403" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1125.66 &lt;= EMA21 1130.82)</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>INDIGO</t>
+        </is>
+      </c>
+      <c r="D404" t="n">
+        <v>4977</v>
+      </c>
+      <c r="E404" t="n">
+        <v>5424.59</v>
+      </c>
+      <c r="F404" t="n">
+        <v>5424.59</v>
+      </c>
+      <c r="G404" t="n">
+        <v>5084.89</v>
+      </c>
+      <c r="H404" t="n">
+        <v>5154.14</v>
+      </c>
+      <c r="I404" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J404" t="b">
+        <v>0</v>
+      </c>
+      <c r="K404" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5084.89 &lt;= EMA21 5154.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>JSWSTEEL</t>
+        </is>
+      </c>
+      <c r="D405" t="n">
+        <v>1302</v>
+      </c>
+      <c r="E405" t="n">
+        <v>1350.05</v>
+      </c>
+      <c r="F405" t="n">
+        <v>1350.05</v>
+      </c>
+      <c r="G405" t="n">
+        <v>1312.32</v>
+      </c>
+      <c r="H405" t="n">
+        <v>1304.19</v>
+      </c>
+      <c r="I405" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J405" t="b">
+        <v>0</v>
+      </c>
+      <c r="K405" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1302.00 &lt;= Upper 1350.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>JINDALSTEL</t>
+        </is>
+      </c>
+      <c r="D406" t="n">
+        <v>1165</v>
+      </c>
+      <c r="E406" t="n">
+        <v>1200.67</v>
+      </c>
+      <c r="F406" t="n">
+        <v>1200.67</v>
+      </c>
+      <c r="G406" t="n">
+        <v>1157.83</v>
+      </c>
+      <c r="H406" t="n">
+        <v>1139.01</v>
+      </c>
+      <c r="I406" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="J406" t="b">
+        <v>0</v>
+      </c>
+      <c r="K406" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1165.00 &lt;= Upper 1200.67)</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>JIOFIN</t>
+        </is>
+      </c>
+      <c r="D407" t="n">
+        <v>239.5</v>
+      </c>
+      <c r="E407" t="n">
+        <v>257.26</v>
+      </c>
+      <c r="F407" t="n">
+        <v>257.26</v>
+      </c>
+      <c r="G407" t="n">
+        <v>239.62</v>
+      </c>
+      <c r="H407" t="n">
+        <v>242.57</v>
+      </c>
+      <c r="I407" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J407" t="b">
+        <v>0</v>
+      </c>
+      <c r="K407" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 239.62 &lt;= EMA21 242.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="D408" t="n">
+        <v>422.1</v>
+      </c>
+      <c r="E408" t="n">
+        <v>436.5</v>
+      </c>
+      <c r="F408" t="n">
+        <v>436.5</v>
+      </c>
+      <c r="G408" t="n">
+        <v>419.19</v>
+      </c>
+      <c r="H408" t="n">
+        <v>410.31</v>
+      </c>
+      <c r="I408" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J408" t="b">
+        <v>0</v>
+      </c>
+      <c r="K408" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 422.10 &lt;= Upper 436.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>LTM</t>
+        </is>
+      </c>
+      <c r="D409" t="n">
+        <v>4448</v>
+      </c>
+      <c r="E409" t="n">
+        <v>4822.11</v>
+      </c>
+      <c r="F409" t="n">
+        <v>4822.11</v>
+      </c>
+      <c r="G409" t="n">
+        <v>4543.42</v>
+      </c>
+      <c r="H409" t="n">
+        <v>4531.01</v>
+      </c>
+      <c r="I409" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J409" t="b">
+        <v>0</v>
+      </c>
+      <c r="K409" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 4448.00 &lt;= Upper 4822.11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="D410" t="n">
+        <v>3999</v>
+      </c>
+      <c r="E410" t="n">
+        <v>4128.55</v>
+      </c>
+      <c r="F410" t="n">
+        <v>4128.55</v>
+      </c>
+      <c r="G410" t="n">
+        <v>4005.42</v>
+      </c>
+      <c r="H410" t="n">
+        <v>4015.96</v>
+      </c>
+      <c r="I410" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J410" t="b">
+        <v>0</v>
+      </c>
+      <c r="K410" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4005.42 &lt;= EMA21 4015.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>LODHA</t>
+        </is>
+      </c>
+      <c r="D411" t="n">
+        <v>1222</v>
+      </c>
+      <c r="E411" t="n">
+        <v>1283.53</v>
+      </c>
+      <c r="F411" t="n">
+        <v>1283.53</v>
+      </c>
+      <c r="G411" t="n">
+        <v>1227.7</v>
+      </c>
+      <c r="H411" t="n">
+        <v>1225.54</v>
+      </c>
+      <c r="I411" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J411" t="b">
+        <v>0</v>
+      </c>
+      <c r="K411" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1222.00 &lt;= Upper 1283.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>M&amp;M</t>
+        </is>
+      </c>
+      <c r="D412" t="n">
+        <v>3160</v>
+      </c>
+      <c r="E412" t="n">
+        <v>3556.01</v>
+      </c>
+      <c r="F412" t="n">
+        <v>3556.01</v>
+      </c>
+      <c r="G412" t="n">
+        <v>3238.87</v>
+      </c>
+      <c r="H412" t="n">
+        <v>3296.77</v>
+      </c>
+      <c r="I412" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J412" t="b">
+        <v>0</v>
+      </c>
+      <c r="K412" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3238.87 &lt;= EMA21 3296.77)</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="D413" t="n">
+        <v>12760</v>
+      </c>
+      <c r="E413" t="n">
+        <v>14301.92</v>
+      </c>
+      <c r="F413" t="n">
+        <v>14301.92</v>
+      </c>
+      <c r="G413" t="n">
+        <v>13053.85</v>
+      </c>
+      <c r="H413" t="n">
+        <v>13345.82</v>
+      </c>
+      <c r="I413" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="J413" t="b">
+        <v>0</v>
+      </c>
+      <c r="K413" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 13053.85 &lt;= EMA21 13345.82)</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>MAXHEALTH</t>
+        </is>
+      </c>
+      <c r="D414" t="n">
+        <v>984.8</v>
+      </c>
+      <c r="E414" t="n">
+        <v>1050.06</v>
+      </c>
+      <c r="F414" t="n">
+        <v>1050.06</v>
+      </c>
+      <c r="G414" t="n">
+        <v>1002.64</v>
+      </c>
+      <c r="H414" t="n">
+        <v>1018.54</v>
+      </c>
+      <c r="I414" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="J414" t="b">
+        <v>0</v>
+      </c>
+      <c r="K414" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1002.64 &lt;= EMA21 1018.54)</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>MAZDOCK</t>
+        </is>
+      </c>
+      <c r="D415" t="n">
+        <v>2475</v>
+      </c>
+      <c r="E415" t="n">
+        <v>2640.95</v>
+      </c>
+      <c r="F415" t="n">
+        <v>2640.95</v>
+      </c>
+      <c r="G415" t="n">
+        <v>2505.76</v>
+      </c>
+      <c r="H415" t="n">
+        <v>2509.31</v>
+      </c>
+      <c r="I415" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J415" t="b">
+        <v>0</v>
+      </c>
+      <c r="K415" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2505.76 &lt;= EMA21 2509.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>MUTHOOTFIN</t>
+        </is>
+      </c>
+      <c r="D416" t="n">
+        <v>2880</v>
+      </c>
+      <c r="E416" t="n">
+        <v>3215.39</v>
+      </c>
+      <c r="F416" t="n">
+        <v>3215.39</v>
+      </c>
+      <c r="G416" t="n">
+        <v>2956.13</v>
+      </c>
+      <c r="H416" t="n">
+        <v>2976.69</v>
+      </c>
+      <c r="I416" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="J416" t="b">
+        <v>0</v>
+      </c>
+      <c r="K416" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2956.13 &lt;= EMA21 2976.69)</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="D417" t="n">
+        <v>332</v>
+      </c>
+      <c r="E417" t="n">
+        <v>341.11</v>
+      </c>
+      <c r="F417" t="n">
+        <v>341.11</v>
+      </c>
+      <c r="G417" t="n">
+        <v>330.56</v>
+      </c>
+      <c r="H417" t="n">
+        <v>332.96</v>
+      </c>
+      <c r="I417" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J417" t="b">
+        <v>0</v>
+      </c>
+      <c r="K417" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 330.56 &lt;= EMA21 332.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="D418" t="n">
+        <v>1398</v>
+      </c>
+      <c r="E418" t="n">
+        <v>1525.34</v>
+      </c>
+      <c r="F418" t="n">
+        <v>1525.34</v>
+      </c>
+      <c r="G418" t="n">
+        <v>1432.61</v>
+      </c>
+      <c r="H418" t="n">
+        <v>1453.59</v>
+      </c>
+      <c r="I418" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="J418" t="b">
+        <v>0</v>
+      </c>
+      <c r="K418" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1432.61 &lt;= EMA21 1453.59)</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="D419" t="n">
+        <v>233.7</v>
+      </c>
+      <c r="E419" t="n">
+        <v>240.55</v>
+      </c>
+      <c r="F419" t="n">
+        <v>240.55</v>
+      </c>
+      <c r="G419" t="n">
+        <v>234.27</v>
+      </c>
+      <c r="H419" t="n">
+        <v>235.61</v>
+      </c>
+      <c r="I419" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="J419" t="b">
+        <v>0</v>
+      </c>
+      <c r="K419" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 234.27 &lt;= EMA21 235.61)</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>PIDILITIND</t>
+        </is>
+      </c>
+      <c r="D420" t="n">
+        <v>1575</v>
+      </c>
+      <c r="E420" t="n">
+        <v>1715.55</v>
+      </c>
+      <c r="F420" t="n">
+        <v>1715.55</v>
+      </c>
+      <c r="G420" t="n">
+        <v>1631.45</v>
+      </c>
+      <c r="H420" t="n">
+        <v>1640.83</v>
+      </c>
+      <c r="I420" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J420" t="b">
+        <v>0</v>
+      </c>
+      <c r="K420" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1631.45 &lt;= EMA21 1640.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>PFC</t>
+        </is>
+      </c>
+      <c r="D421" t="n">
+        <v>353.1</v>
+      </c>
+      <c r="E421" t="n">
+        <v>382.72</v>
+      </c>
+      <c r="F421" t="n">
+        <v>382.72</v>
+      </c>
+      <c r="G421" t="n">
+        <v>352.5</v>
+      </c>
+      <c r="H421" t="n">
+        <v>363.28</v>
+      </c>
+      <c r="I421" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J421" t="b">
+        <v>0</v>
+      </c>
+      <c r="K421" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 352.50 &lt;= EMA21 363.28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="D422" t="n">
+        <v>266</v>
+      </c>
+      <c r="E422" t="n">
+        <v>272.24</v>
+      </c>
+      <c r="F422" t="n">
+        <v>272.24</v>
+      </c>
+      <c r="G422" t="n">
+        <v>266.22</v>
+      </c>
+      <c r="H422" t="n">
+        <v>268.97</v>
+      </c>
+      <c r="I422" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J422" t="b">
+        <v>0</v>
+      </c>
+      <c r="K422" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 266.22 &lt;= EMA21 268.97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="D423" t="n">
+        <v>115.6</v>
+      </c>
+      <c r="E423" t="n">
+        <v>119</v>
+      </c>
+      <c r="F423" t="n">
+        <v>119</v>
+      </c>
+      <c r="G423" t="n">
+        <v>116.06</v>
+      </c>
+      <c r="H423" t="n">
+        <v>115.49</v>
+      </c>
+      <c r="I423" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J423" t="b">
+        <v>0</v>
+      </c>
+      <c r="K423" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 115.60 &lt;= Upper 119.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="D424" t="n">
+        <v>316.4</v>
+      </c>
+      <c r="E424" t="n">
+        <v>349.05</v>
+      </c>
+      <c r="F424" t="n">
+        <v>349.05</v>
+      </c>
+      <c r="G424" t="n">
+        <v>319.41</v>
+      </c>
+      <c r="H424" t="n">
+        <v>328.13</v>
+      </c>
+      <c r="I424" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J424" t="b">
+        <v>0</v>
+      </c>
+      <c r="K424" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 319.41 &lt;= EMA21 328.13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="D425" t="n">
+        <v>1309.5</v>
+      </c>
+      <c r="E425" t="n">
+        <v>1336.85</v>
+      </c>
+      <c r="F425" t="n">
+        <v>1336.85</v>
+      </c>
+      <c r="G425" t="n">
+        <v>1306.79</v>
+      </c>
+      <c r="H425" t="n">
+        <v>1306.32</v>
+      </c>
+      <c r="I425" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J425" t="b">
+        <v>0</v>
+      </c>
+      <c r="K425" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1309.50 &lt;= Upper 1336.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="D426" t="n">
+        <v>1732</v>
+      </c>
+      <c r="E426" t="n">
+        <v>1838.36</v>
+      </c>
+      <c r="F426" t="n">
+        <v>1838.36</v>
+      </c>
+      <c r="G426" t="n">
+        <v>1748.38</v>
+      </c>
+      <c r="H426" t="n">
+        <v>1772.84</v>
+      </c>
+      <c r="I426" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="J426" t="b">
+        <v>0</v>
+      </c>
+      <c r="K426" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1748.38 &lt;= EMA21 1772.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>MOTHERSON</t>
+        </is>
+      </c>
+      <c r="D427" t="n">
+        <v>162</v>
+      </c>
+      <c r="E427" t="n">
+        <v>173.06</v>
+      </c>
+      <c r="F427" t="n">
+        <v>173.06</v>
+      </c>
+      <c r="G427" t="n">
+        <v>164.01</v>
+      </c>
+      <c r="H427" t="n">
+        <v>163.54</v>
+      </c>
+      <c r="I427" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="J427" t="b">
+        <v>0</v>
+      </c>
+      <c r="K427" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 162.00 &lt;= Upper 173.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="D428" t="n">
+        <v>23365</v>
+      </c>
+      <c r="E428" t="n">
+        <v>25663.95</v>
+      </c>
+      <c r="F428" t="n">
+        <v>25663.95</v>
+      </c>
+      <c r="G428" t="n">
+        <v>23843.71</v>
+      </c>
+      <c r="H428" t="n">
+        <v>24407.21</v>
+      </c>
+      <c r="I428" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J428" t="b">
+        <v>0</v>
+      </c>
+      <c r="K428" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 23843.71 &lt;= EMA21 24407.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>SHRIRAMFIN</t>
+        </is>
+      </c>
+      <c r="D429" t="n">
+        <v>1037</v>
+      </c>
+      <c r="E429" t="n">
+        <v>1168.63</v>
+      </c>
+      <c r="F429" t="n">
+        <v>1168.63</v>
+      </c>
+      <c r="G429" t="n">
+        <v>1065.68</v>
+      </c>
+      <c r="H429" t="n">
+        <v>1081.7</v>
+      </c>
+      <c r="I429" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J429" t="b">
+        <v>0</v>
+      </c>
+      <c r="K429" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1065.68 &lt;= EMA21 1081.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>ENRIN</t>
+        </is>
+      </c>
+      <c r="D430" t="n">
+        <v>3115.7</v>
+      </c>
+      <c r="E430" t="n">
+        <v>3738.83</v>
+      </c>
+      <c r="F430" t="n">
+        <v>3738.83</v>
+      </c>
+      <c r="G430" t="n">
+        <v>3221.22</v>
+      </c>
+      <c r="H430" t="n">
+        <v>3311.5</v>
+      </c>
+      <c r="I430" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J430" t="b">
+        <v>0</v>
+      </c>
+      <c r="K430" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3221.22 &lt;= EMA21 3311.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+      <c r="D431" t="n">
+        <v>3927</v>
+      </c>
+      <c r="E431" t="n">
+        <v>4137.1</v>
+      </c>
+      <c r="F431" t="n">
+        <v>4137.1</v>
+      </c>
+      <c r="G431" t="n">
+        <v>4000.21</v>
+      </c>
+      <c r="H431" t="n">
+        <v>3970.7</v>
+      </c>
+      <c r="I431" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="J431" t="b">
+        <v>0</v>
+      </c>
+      <c r="K431" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3927.00 &lt;= Upper 4137.10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>SOLARINDS</t>
+        </is>
+      </c>
+      <c r="D432" t="n">
+        <v>21950</v>
+      </c>
+      <c r="E432" t="n">
+        <v>21769.07</v>
+      </c>
+      <c r="F432" t="n">
+        <v>21769.07</v>
+      </c>
+      <c r="G432" t="n">
+        <v>20899.24</v>
+      </c>
+      <c r="H432" t="n">
+        <v>20228.05</v>
+      </c>
+      <c r="I432" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J432" t="b">
+        <v>0</v>
+      </c>
+      <c r="K432" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 1.20x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="D433" t="n">
+        <v>1005.9</v>
+      </c>
+      <c r="E433" t="n">
+        <v>1088.12</v>
+      </c>
+      <c r="F433" t="n">
+        <v>1088.12</v>
+      </c>
+      <c r="G433" t="n">
+        <v>1028.67</v>
+      </c>
+      <c r="H433" t="n">
+        <v>1039.04</v>
+      </c>
+      <c r="I433" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="J433" t="b">
+        <v>0</v>
+      </c>
+      <c r="K433" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1028.67 &lt;= EMA21 1039.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="D434" t="n">
+        <v>1895</v>
+      </c>
+      <c r="E434" t="n">
+        <v>1965.93</v>
+      </c>
+      <c r="F434" t="n">
+        <v>1965.93</v>
+      </c>
+      <c r="G434" t="n">
+        <v>1915.44</v>
+      </c>
+      <c r="H434" t="n">
+        <v>1920.91</v>
+      </c>
+      <c r="I434" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="J434" t="b">
+        <v>0</v>
+      </c>
+      <c r="K434" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1915.44 &lt;= EMA21 1920.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>TVSMOTOR</t>
+        </is>
+      </c>
+      <c r="D435" t="n">
+        <v>4132</v>
+      </c>
+      <c r="E435" t="n">
+        <v>4519.22</v>
+      </c>
+      <c r="F435" t="n">
+        <v>4519.22</v>
+      </c>
+      <c r="G435" t="n">
+        <v>4231.89</v>
+      </c>
+      <c r="H435" t="n">
+        <v>4254.91</v>
+      </c>
+      <c r="I435" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J435" t="b">
+        <v>0</v>
+      </c>
+      <c r="K435" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4231.89 &lt;= EMA21 4254.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>TATACAP</t>
+        </is>
+      </c>
+      <c r="D436" t="n">
+        <v>375.05</v>
+      </c>
+      <c r="E436" t="n">
+        <v>376.3</v>
+      </c>
+      <c r="F436" t="n">
+        <v>376.3</v>
+      </c>
+      <c r="G436" t="n">
+        <v>370.05</v>
+      </c>
+      <c r="H436" t="n">
+        <v>367.34</v>
+      </c>
+      <c r="I436" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="J436" t="b">
+        <v>0</v>
+      </c>
+      <c r="K436" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 375.05 &lt;= Upper 376.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="D437" t="n">
+        <v>2270</v>
+      </c>
+      <c r="E437" t="n">
+        <v>2422.48</v>
+      </c>
+      <c r="F437" t="n">
+        <v>2422.48</v>
+      </c>
+      <c r="G437" t="n">
+        <v>2315.16</v>
+      </c>
+      <c r="H437" t="n">
+        <v>2319.91</v>
+      </c>
+      <c r="I437" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J437" t="b">
+        <v>0</v>
+      </c>
+      <c r="K437" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2315.16 &lt;= EMA21 2319.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>TATACONSUM</t>
+        </is>
+      </c>
+      <c r="D438" t="n">
+        <v>1015</v>
+      </c>
+      <c r="E438" t="n">
+        <v>1097.01</v>
+      </c>
+      <c r="F438" t="n">
+        <v>1097.01</v>
+      </c>
+      <c r="G438" t="n">
+        <v>1027.5</v>
+      </c>
+      <c r="H438" t="n">
+        <v>1046.86</v>
+      </c>
+      <c r="I438" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="J438" t="b">
+        <v>0</v>
+      </c>
+      <c r="K438" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1027.50 &lt;= EMA21 1046.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>TMCV</t>
+        </is>
+      </c>
+      <c r="D439" t="n">
+        <v>458.2</v>
+      </c>
+      <c r="E439" t="n">
+        <v>488.36</v>
+      </c>
+      <c r="F439" t="n">
+        <v>488.36</v>
+      </c>
+      <c r="G439" t="n">
+        <v>463.38</v>
+      </c>
+      <c r="H439" t="n">
+        <v>461.05</v>
+      </c>
+      <c r="I439" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J439" t="b">
+        <v>0</v>
+      </c>
+      <c r="K439" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 458.20 &lt;= Upper 488.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>TMPV</t>
+        </is>
+      </c>
+      <c r="D440" t="n">
+        <v>307</v>
+      </c>
+      <c r="E440" t="n">
+        <v>347.16</v>
+      </c>
+      <c r="F440" t="n">
+        <v>347.16</v>
+      </c>
+      <c r="G440" t="n">
+        <v>312.74</v>
+      </c>
+      <c r="H440" t="n">
+        <v>319.86</v>
+      </c>
+      <c r="I440" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J440" t="b">
+        <v>0</v>
+      </c>
+      <c r="K440" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 312.74 &lt;= EMA21 319.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>TATAPOWER</t>
+        </is>
+      </c>
+      <c r="D441" t="n">
+        <v>365.7</v>
+      </c>
+      <c r="E441" t="n">
+        <v>392.61</v>
+      </c>
+      <c r="F441" t="n">
+        <v>392.61</v>
+      </c>
+      <c r="G441" t="n">
+        <v>363.46</v>
+      </c>
+      <c r="H441" t="n">
+        <v>367.66</v>
+      </c>
+      <c r="I441" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J441" t="b">
+        <v>0</v>
+      </c>
+      <c r="K441" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 363.46 &lt;= EMA21 367.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="D442" t="n">
+        <v>185.61</v>
+      </c>
+      <c r="E442" t="n">
+        <v>188.93</v>
+      </c>
+      <c r="F442" t="n">
+        <v>188.93</v>
+      </c>
+      <c r="G442" t="n">
+        <v>185.72</v>
+      </c>
+      <c r="H442" t="n">
+        <v>186.03</v>
+      </c>
+      <c r="I442" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J442" t="b">
+        <v>0</v>
+      </c>
+      <c r="K442" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 185.72 &lt;= EMA21 186.03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>TECHM</t>
+        </is>
+      </c>
+      <c r="D443" t="n">
+        <v>1564</v>
+      </c>
+      <c r="E443" t="n">
+        <v>1656.64</v>
+      </c>
+      <c r="F443" t="n">
+        <v>1656.64</v>
+      </c>
+      <c r="G443" t="n">
+        <v>1600</v>
+      </c>
+      <c r="H443" t="n">
+        <v>1601.3</v>
+      </c>
+      <c r="I443" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J443" t="b">
+        <v>0</v>
+      </c>
+      <c r="K443" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1600.00 &lt;= EMA21 1601.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>TITAN</t>
+        </is>
+      </c>
+      <c r="D444" t="n">
+        <v>4995</v>
+      </c>
+      <c r="E444" t="n">
+        <v>5162.74</v>
+      </c>
+      <c r="F444" t="n">
+        <v>5162.74</v>
+      </c>
+      <c r="G444" t="n">
+        <v>5051.82</v>
+      </c>
+      <c r="H444" t="n">
+        <v>5029.84</v>
+      </c>
+      <c r="I444" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J444" t="b">
+        <v>0</v>
+      </c>
+      <c r="K444" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 4995.00 &lt;= Upper 5162.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>TORNTPHARM</t>
+        </is>
+      </c>
+      <c r="D445" t="n">
+        <v>4914</v>
+      </c>
+      <c r="E445" t="n">
+        <v>5071.42</v>
+      </c>
+      <c r="F445" t="n">
+        <v>5071.42</v>
+      </c>
+      <c r="G445" t="n">
+        <v>4940.21</v>
+      </c>
+      <c r="H445" t="n">
+        <v>4942.9</v>
+      </c>
+      <c r="I445" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J445" t="b">
+        <v>0</v>
+      </c>
+      <c r="K445" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4940.21 &lt;= EMA21 4942.90)</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="D446" t="n">
+        <v>2814.5</v>
+      </c>
+      <c r="E446" t="n">
+        <v>3029</v>
+      </c>
+      <c r="F446" t="n">
+        <v>3029</v>
+      </c>
+      <c r="G446" t="n">
+        <v>2860.49</v>
+      </c>
+      <c r="H446" t="n">
+        <v>2903.68</v>
+      </c>
+      <c r="I446" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="J446" t="b">
+        <v>0</v>
+      </c>
+      <c r="K446" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2860.49 &lt;= EMA21 2903.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="D447" t="n">
+        <v>11175</v>
+      </c>
+      <c r="E447" t="n">
+        <v>11896.97</v>
+      </c>
+      <c r="F447" t="n">
+        <v>11896.97</v>
+      </c>
+      <c r="G447" t="n">
+        <v>11403.69</v>
+      </c>
+      <c r="H447" t="n">
+        <v>11523.53</v>
+      </c>
+      <c r="I447" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J447" t="b">
+        <v>0</v>
+      </c>
+      <c r="K447" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11403.69 &lt;= EMA21 11523.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="D448" t="n">
+        <v>186.04</v>
+      </c>
+      <c r="E448" t="n">
+        <v>189.84</v>
+      </c>
+      <c r="F448" t="n">
+        <v>189.84</v>
+      </c>
+      <c r="G448" t="n">
+        <v>186.59</v>
+      </c>
+      <c r="H448" t="n">
+        <v>184.51</v>
+      </c>
+      <c r="I448" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J448" t="b">
+        <v>0</v>
+      </c>
+      <c r="K448" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 186.04 &lt;= Upper 189.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>UNITDSPR</t>
+        </is>
+      </c>
+      <c r="D449" t="n">
+        <v>1440</v>
+      </c>
+      <c r="E449" t="n">
+        <v>1584.29</v>
+      </c>
+      <c r="F449" t="n">
+        <v>1584.29</v>
+      </c>
+      <c r="G449" t="n">
+        <v>1484.06</v>
+      </c>
+      <c r="H449" t="n">
+        <v>1497.04</v>
+      </c>
+      <c r="I449" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="J449" t="b">
+        <v>0</v>
+      </c>
+      <c r="K449" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1484.06 &lt;= EMA21 1497.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="D450" t="n">
+        <v>405.95</v>
+      </c>
+      <c r="E450" t="n">
+        <v>452.16</v>
+      </c>
+      <c r="F450" t="n">
+        <v>452.16</v>
+      </c>
+      <c r="G450" t="n">
+        <v>412.35</v>
+      </c>
+      <c r="H450" t="n">
+        <v>423.55</v>
+      </c>
+      <c r="I450" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J450" t="b">
+        <v>0</v>
+      </c>
+      <c r="K450" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 412.35 &lt;= EMA21 423.55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>VEDL</t>
+        </is>
+      </c>
+      <c r="D451" t="n">
+        <v>268</v>
+      </c>
+      <c r="E451" t="n">
+        <v>287.08</v>
+      </c>
+      <c r="F451" t="n">
+        <v>287.08</v>
+      </c>
+      <c r="G451" t="n">
+        <v>273.24</v>
+      </c>
+      <c r="H451" t="n">
+        <v>273.73</v>
+      </c>
+      <c r="I451" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="J451" t="b">
+        <v>0</v>
+      </c>
+      <c r="K451" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 273.24 &lt;= EMA21 273.73)</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="D452" t="n">
+        <v>172.8</v>
+      </c>
+      <c r="E452" t="n">
+        <v>186.69</v>
+      </c>
+      <c r="F452" t="n">
+        <v>186.69</v>
+      </c>
+      <c r="G452" t="n">
+        <v>177.55</v>
+      </c>
+      <c r="H452" t="n">
+        <v>179.26</v>
+      </c>
+      <c r="I452" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="J452" t="b">
+        <v>0</v>
+      </c>
+      <c r="K452" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 177.55 &lt;= EMA21 179.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>ZYDUSLIFE</t>
+        </is>
+      </c>
+      <c r="D453" t="n">
+        <v>1156.9</v>
+      </c>
+      <c r="E453" t="n">
+        <v>1209.87</v>
+      </c>
+      <c r="F453" t="n">
+        <v>1209.87</v>
+      </c>
+      <c r="G453" t="n">
+        <v>1148.35</v>
+      </c>
+      <c r="H453" t="n">
+        <v>1143.49</v>
+      </c>
+      <c r="I453" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J453" t="b">
+        <v>0</v>
+      </c>
+      <c r="K453" t="inlineStr">
         <is>
           <t>BELOW_BAND (Close 1156.90 &lt;= Upper 1209.87)</t>
         </is>
@@ -15620,41 +19920,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Signal_Price</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Initial_SL</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Vol_Ratio</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -15748,6 +20048,37 @@
         <v>1.32</v>
       </c>
       <c r="G4" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>418.85</v>
+      </c>
+      <c r="E5" t="n">
+        <v>400</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>QUEUED</t>
         </is>
@@ -15768,57 +20099,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Entry_Date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Entry_Price</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Invested</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Current_Price</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Unrealized_PnL_Pct</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Hard_SL</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Highest_High</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Days_Held</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -15880,67 +20211,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Entry_Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Exit_Date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Entry_Price</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Exit_Price</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Invested</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Gross_PnL_Pct</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Net_PnL_Pct</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>PnL_Amount</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Exit_Reason</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Days_Held</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -16777,57 +21108,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Order_ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Side</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Expected_Price</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Fill_Price</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Slippage</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -21881,27 +26212,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
@@ -21945,51 +26276,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cash_Available</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Invested_Capital</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Total_Equity</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Realized_PnL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Win_Rate_Pct</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Total_Trades</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Open_Positions</t>
         </is>
@@ -22223,6 +26554,39 @@
         <v>17</v>
       </c>
       <c r="I8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:03:20</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>179135.98</v>
+      </c>
+      <c r="D9" t="n">
+        <v>19685.95</v>
+      </c>
+      <c r="E9" t="n">
+        <v>198821.93</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-1092.43</v>
+      </c>
+      <c r="G9" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>17</v>
+      </c>
+      <c r="I9" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
state: bot run 2026-09-08T20:03 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_india.xlsx
+++ b/data/trade_log_india.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K453"/>
+  <dimension ref="A1:K553"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19906,6 +19906,4306 @@
       <c r="K453" t="inlineStr">
         <is>
           <t>BELOW_BAND (Close 1156.90 &lt;= Upper 1209.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+      <c r="D454" t="n">
+        <v>7387</v>
+      </c>
+      <c r="E454" t="n">
+        <v>7751.46</v>
+      </c>
+      <c r="F454" t="n">
+        <v>7751.46</v>
+      </c>
+      <c r="G454" t="n">
+        <v>7458.88</v>
+      </c>
+      <c r="H454" t="n">
+        <v>7475.24</v>
+      </c>
+      <c r="I454" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="J454" t="b">
+        <v>0</v>
+      </c>
+      <c r="K454" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7458.88 &lt;= EMA21 7475.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="D455" t="n">
+        <v>1407.7</v>
+      </c>
+      <c r="E455" t="n">
+        <v>1699.7</v>
+      </c>
+      <c r="F455" t="n">
+        <v>1699.7</v>
+      </c>
+      <c r="G455" t="n">
+        <v>1437.81</v>
+      </c>
+      <c r="H455" t="n">
+        <v>1500.87</v>
+      </c>
+      <c r="I455" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="J455" t="b">
+        <v>0</v>
+      </c>
+      <c r="K455" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1437.81 &lt;= EMA21 1500.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>ADANIENT</t>
+        </is>
+      </c>
+      <c r="D456" t="n">
+        <v>2953.1</v>
+      </c>
+      <c r="E456" t="n">
+        <v>3173.7</v>
+      </c>
+      <c r="F456" t="n">
+        <v>3173.7</v>
+      </c>
+      <c r="G456" t="n">
+        <v>2957.64</v>
+      </c>
+      <c r="H456" t="n">
+        <v>2988.57</v>
+      </c>
+      <c r="I456" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J456" t="b">
+        <v>0</v>
+      </c>
+      <c r="K456" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2957.64 &lt;= EMA21 2988.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>ADANIGREEN</t>
+        </is>
+      </c>
+      <c r="D457" t="n">
+        <v>1292</v>
+      </c>
+      <c r="E457" t="n">
+        <v>1360.88</v>
+      </c>
+      <c r="F457" t="n">
+        <v>1360.88</v>
+      </c>
+      <c r="G457" t="n">
+        <v>1291.9</v>
+      </c>
+      <c r="H457" t="n">
+        <v>1313.7</v>
+      </c>
+      <c r="I457" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J457" t="b">
+        <v>0</v>
+      </c>
+      <c r="K457" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1291.90 &lt;= EMA21 1313.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="D458" t="n">
+        <v>1710</v>
+      </c>
+      <c r="E458" t="n">
+        <v>1740.38</v>
+      </c>
+      <c r="F458" t="n">
+        <v>1740.38</v>
+      </c>
+      <c r="G458" t="n">
+        <v>1689.27</v>
+      </c>
+      <c r="H458" t="n">
+        <v>1694</v>
+      </c>
+      <c r="I458" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="J458" t="b">
+        <v>0</v>
+      </c>
+      <c r="K458" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1689.27 &lt;= EMA21 1694.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="D459" t="n">
+        <v>208.4</v>
+      </c>
+      <c r="E459" t="n">
+        <v>213.19</v>
+      </c>
+      <c r="F459" t="n">
+        <v>213.19</v>
+      </c>
+      <c r="G459" t="n">
+        <v>206.8</v>
+      </c>
+      <c r="H459" t="n">
+        <v>207.48</v>
+      </c>
+      <c r="I459" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J459" t="b">
+        <v>0</v>
+      </c>
+      <c r="K459" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 206.80 &lt;= EMA21 207.48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>AMBUJACEM</t>
+        </is>
+      </c>
+      <c r="D460" t="n">
+        <v>398.3</v>
+      </c>
+      <c r="E460" t="n">
+        <v>423.82</v>
+      </c>
+      <c r="F460" t="n">
+        <v>423.82</v>
+      </c>
+      <c r="G460" t="n">
+        <v>403.98</v>
+      </c>
+      <c r="H460" t="n">
+        <v>410.6</v>
+      </c>
+      <c r="I460" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="J460" t="b">
+        <v>0</v>
+      </c>
+      <c r="K460" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 403.98 &lt;= EMA21 410.60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="D461" t="n">
+        <v>8837.5</v>
+      </c>
+      <c r="E461" t="n">
+        <v>8949.030000000001</v>
+      </c>
+      <c r="F461" t="n">
+        <v>8949.030000000001</v>
+      </c>
+      <c r="G461" t="n">
+        <v>8762.559999999999</v>
+      </c>
+      <c r="H461" t="n">
+        <v>8780.059999999999</v>
+      </c>
+      <c r="I461" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J461" t="b">
+        <v>0</v>
+      </c>
+      <c r="K461" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 8762.56 &lt;= EMA21 8780.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="D462" t="n">
+        <v>2481.6</v>
+      </c>
+      <c r="E462" t="n">
+        <v>2766.27</v>
+      </c>
+      <c r="F462" t="n">
+        <v>2766.27</v>
+      </c>
+      <c r="G462" t="n">
+        <v>2548.98</v>
+      </c>
+      <c r="H462" t="n">
+        <v>2604.16</v>
+      </c>
+      <c r="I462" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J462" t="b">
+        <v>0</v>
+      </c>
+      <c r="K462" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2548.98 &lt;= EMA21 2604.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="D463" t="n">
+        <v>3720.2</v>
+      </c>
+      <c r="E463" t="n">
+        <v>4110.76</v>
+      </c>
+      <c r="F463" t="n">
+        <v>4110.76</v>
+      </c>
+      <c r="G463" t="n">
+        <v>3790.27</v>
+      </c>
+      <c r="H463" t="n">
+        <v>3861.14</v>
+      </c>
+      <c r="I463" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J463" t="b">
+        <v>0</v>
+      </c>
+      <c r="K463" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3790.27 &lt;= EMA21 3861.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="D464" t="n">
+        <v>1244.9</v>
+      </c>
+      <c r="E464" t="n">
+        <v>1286.85</v>
+      </c>
+      <c r="F464" t="n">
+        <v>1286.85</v>
+      </c>
+      <c r="G464" t="n">
+        <v>1258.77</v>
+      </c>
+      <c r="H464" t="n">
+        <v>1255.41</v>
+      </c>
+      <c r="I464" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J464" t="b">
+        <v>0</v>
+      </c>
+      <c r="K464" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1244.90 &lt;= Upper 1286.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO</t>
+        </is>
+      </c>
+      <c r="D465" t="n">
+        <v>11880</v>
+      </c>
+      <c r="E465" t="n">
+        <v>12222.07</v>
+      </c>
+      <c r="F465" t="n">
+        <v>12222.07</v>
+      </c>
+      <c r="G465" t="n">
+        <v>11918.6</v>
+      </c>
+      <c r="H465" t="n">
+        <v>11793.31</v>
+      </c>
+      <c r="I465" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J465" t="b">
+        <v>0</v>
+      </c>
+      <c r="K465" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 11880.00 &lt;= Upper 12222.07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="D466" t="n">
+        <v>1054.1</v>
+      </c>
+      <c r="E466" t="n">
+        <v>1109.36</v>
+      </c>
+      <c r="F466" t="n">
+        <v>1109.36</v>
+      </c>
+      <c r="G466" t="n">
+        <v>1062.31</v>
+      </c>
+      <c r="H466" t="n">
+        <v>1070.47</v>
+      </c>
+      <c r="I466" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J466" t="b">
+        <v>0</v>
+      </c>
+      <c r="K466" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1062.31 &lt;= EMA21 1070.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="D467" t="n">
+        <v>1938.1</v>
+      </c>
+      <c r="E467" t="n">
+        <v>2051.03</v>
+      </c>
+      <c r="F467" t="n">
+        <v>2051.03</v>
+      </c>
+      <c r="G467" t="n">
+        <v>1973.72</v>
+      </c>
+      <c r="H467" t="n">
+        <v>1984.89</v>
+      </c>
+      <c r="I467" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="J467" t="b">
+        <v>0</v>
+      </c>
+      <c r="K467" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1973.72 &lt;= EMA21 1984.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>BAJAJHLDNG</t>
+        </is>
+      </c>
+      <c r="D468" t="n">
+        <v>11046</v>
+      </c>
+      <c r="E468" t="n">
+        <v>11684.26</v>
+      </c>
+      <c r="F468" t="n">
+        <v>11684.26</v>
+      </c>
+      <c r="G468" t="n">
+        <v>11177.68</v>
+      </c>
+      <c r="H468" t="n">
+        <v>11225.49</v>
+      </c>
+      <c r="I468" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J468" t="b">
+        <v>0</v>
+      </c>
+      <c r="K468" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11177.68 &lt;= EMA21 11225.49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>BANKBARODA</t>
+        </is>
+      </c>
+      <c r="D469" t="n">
+        <v>236.6</v>
+      </c>
+      <c r="E469" t="n">
+        <v>250.73</v>
+      </c>
+      <c r="F469" t="n">
+        <v>250.73</v>
+      </c>
+      <c r="G469" t="n">
+        <v>239.29</v>
+      </c>
+      <c r="H469" t="n">
+        <v>241.91</v>
+      </c>
+      <c r="I469" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J469" t="b">
+        <v>0</v>
+      </c>
+      <c r="K469" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 239.29 &lt;= EMA21 241.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="D470" t="n">
+        <v>410.55</v>
+      </c>
+      <c r="E470" t="n">
+        <v>415.85</v>
+      </c>
+      <c r="F470" t="n">
+        <v>415.85</v>
+      </c>
+      <c r="G470" t="n">
+        <v>408.39</v>
+      </c>
+      <c r="H470" t="n">
+        <v>407.93</v>
+      </c>
+      <c r="I470" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="J470" t="b">
+        <v>0</v>
+      </c>
+      <c r="K470" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 410.55 &lt;= Upper 415.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>BPCL</t>
+        </is>
+      </c>
+      <c r="D471" t="n">
+        <v>303.85</v>
+      </c>
+      <c r="E471" t="n">
+        <v>325.34</v>
+      </c>
+      <c r="F471" t="n">
+        <v>325.34</v>
+      </c>
+      <c r="G471" t="n">
+        <v>314.31</v>
+      </c>
+      <c r="H471" t="n">
+        <v>315.51</v>
+      </c>
+      <c r="I471" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J471" t="b">
+        <v>0</v>
+      </c>
+      <c r="K471" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 314.31 &lt;= EMA21 315.51)</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="D472" t="n">
+        <v>1844</v>
+      </c>
+      <c r="E472" t="n">
+        <v>2002.65</v>
+      </c>
+      <c r="F472" t="n">
+        <v>2002.65</v>
+      </c>
+      <c r="G472" t="n">
+        <v>1864.73</v>
+      </c>
+      <c r="H472" t="n">
+        <v>1889.85</v>
+      </c>
+      <c r="I472" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J472" t="b">
+        <v>0</v>
+      </c>
+      <c r="K472" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1864.73 &lt;= EMA21 1889.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>BOSCHLTD</t>
+        </is>
+      </c>
+      <c r="D473" t="n">
+        <v>48785</v>
+      </c>
+      <c r="E473" t="n">
+        <v>49951.7</v>
+      </c>
+      <c r="F473" t="n">
+        <v>49951.7</v>
+      </c>
+      <c r="G473" t="n">
+        <v>48021.58</v>
+      </c>
+      <c r="H473" t="n">
+        <v>47190.09</v>
+      </c>
+      <c r="I473" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J473" t="b">
+        <v>0</v>
+      </c>
+      <c r="K473" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 48785.00 &lt;= Upper 49951.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>BRITANNIA</t>
+        </is>
+      </c>
+      <c r="D474" t="n">
+        <v>5064</v>
+      </c>
+      <c r="E474" t="n">
+        <v>5711.93</v>
+      </c>
+      <c r="F474" t="n">
+        <v>5711.93</v>
+      </c>
+      <c r="G474" t="n">
+        <v>5162.49</v>
+      </c>
+      <c r="H474" t="n">
+        <v>5269.71</v>
+      </c>
+      <c r="I474" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J474" t="b">
+        <v>0</v>
+      </c>
+      <c r="K474" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5162.49 &lt;= EMA21 5269.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="D475" t="n">
+        <v>910.7</v>
+      </c>
+      <c r="E475" t="n">
+        <v>915.02</v>
+      </c>
+      <c r="F475" t="n">
+        <v>915.02</v>
+      </c>
+      <c r="G475" t="n">
+        <v>893.91</v>
+      </c>
+      <c r="H475" t="n">
+        <v>888.8200000000001</v>
+      </c>
+      <c r="I475" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="J475" t="b">
+        <v>0</v>
+      </c>
+      <c r="K475" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 910.70 &lt;= Upper 915.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>CANBK</t>
+        </is>
+      </c>
+      <c r="D476" t="n">
+        <v>124.68</v>
+      </c>
+      <c r="E476" t="n">
+        <v>133.04</v>
+      </c>
+      <c r="F476" t="n">
+        <v>133.04</v>
+      </c>
+      <c r="G476" t="n">
+        <v>125.99</v>
+      </c>
+      <c r="H476" t="n">
+        <v>127.19</v>
+      </c>
+      <c r="I476" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J476" t="b">
+        <v>0</v>
+      </c>
+      <c r="K476" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 125.99 &lt;= EMA21 127.19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="D477" t="n">
+        <v>1823.4</v>
+      </c>
+      <c r="E477" t="n">
+        <v>1930.19</v>
+      </c>
+      <c r="F477" t="n">
+        <v>1930.19</v>
+      </c>
+      <c r="G477" t="n">
+        <v>1843.52</v>
+      </c>
+      <c r="H477" t="n">
+        <v>1850.58</v>
+      </c>
+      <c r="I477" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="J477" t="b">
+        <v>0</v>
+      </c>
+      <c r="K477" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1843.52 &lt;= EMA21 1850.58)</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>CIPLA</t>
+        </is>
+      </c>
+      <c r="D478" t="n">
+        <v>1384</v>
+      </c>
+      <c r="E478" t="n">
+        <v>1471.71</v>
+      </c>
+      <c r="F478" t="n">
+        <v>1471.71</v>
+      </c>
+      <c r="G478" t="n">
+        <v>1404.56</v>
+      </c>
+      <c r="H478" t="n">
+        <v>1419.71</v>
+      </c>
+      <c r="I478" t="n">
+        <v>1</v>
+      </c>
+      <c r="J478" t="b">
+        <v>0</v>
+      </c>
+      <c r="K478" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1404.56 &lt;= EMA21 1419.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="D479" t="n">
+        <v>420.25</v>
+      </c>
+      <c r="E479" t="n">
+        <v>420.07</v>
+      </c>
+      <c r="F479" t="n">
+        <v>420.07</v>
+      </c>
+      <c r="G479" t="n">
+        <v>410.92</v>
+      </c>
+      <c r="H479" t="n">
+        <v>407.55</v>
+      </c>
+      <c r="I479" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="J479" t="b">
+        <v>0</v>
+      </c>
+      <c r="K479" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 0.53x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>CUMMINSIND</t>
+        </is>
+      </c>
+      <c r="D480" t="n">
+        <v>5040</v>
+      </c>
+      <c r="E480" t="n">
+        <v>5465.79</v>
+      </c>
+      <c r="F480" t="n">
+        <v>5465.79</v>
+      </c>
+      <c r="G480" t="n">
+        <v>5107.31</v>
+      </c>
+      <c r="H480" t="n">
+        <v>5205.51</v>
+      </c>
+      <c r="I480" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J480" t="b">
+        <v>0</v>
+      </c>
+      <c r="K480" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5107.31 &lt;= EMA21 5205.51)</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>DLF</t>
+        </is>
+      </c>
+      <c r="D481" t="n">
+        <v>675.1</v>
+      </c>
+      <c r="E481" t="n">
+        <v>693.37</v>
+      </c>
+      <c r="F481" t="n">
+        <v>693.37</v>
+      </c>
+      <c r="G481" t="n">
+        <v>678.03</v>
+      </c>
+      <c r="H481" t="n">
+        <v>672.8099999999999</v>
+      </c>
+      <c r="I481" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J481" t="b">
+        <v>0</v>
+      </c>
+      <c r="K481" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 675.10 &lt;= Upper 693.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>DIVISLAB</t>
+        </is>
+      </c>
+      <c r="D482" t="n">
+        <v>9575</v>
+      </c>
+      <c r="E482" t="n">
+        <v>9647.82</v>
+      </c>
+      <c r="F482" t="n">
+        <v>9647.82</v>
+      </c>
+      <c r="G482" t="n">
+        <v>9221.610000000001</v>
+      </c>
+      <c r="H482" t="n">
+        <v>8890.52</v>
+      </c>
+      <c r="I482" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="J482" t="b">
+        <v>0</v>
+      </c>
+      <c r="K482" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 9575.00 &lt;= Upper 9647.82)</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="D483" t="n">
+        <v>1151</v>
+      </c>
+      <c r="E483" t="n">
+        <v>1212.18</v>
+      </c>
+      <c r="F483" t="n">
+        <v>1212.18</v>
+      </c>
+      <c r="G483" t="n">
+        <v>1158.76</v>
+      </c>
+      <c r="H483" t="n">
+        <v>1170.5</v>
+      </c>
+      <c r="I483" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="J483" t="b">
+        <v>0</v>
+      </c>
+      <c r="K483" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1158.76 &lt;= EMA21 1170.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>EICHERMOT</t>
+        </is>
+      </c>
+      <c r="D484" t="n">
+        <v>7747.5</v>
+      </c>
+      <c r="E484" t="n">
+        <v>8257.01</v>
+      </c>
+      <c r="F484" t="n">
+        <v>8257.01</v>
+      </c>
+      <c r="G484" t="n">
+        <v>7827.7</v>
+      </c>
+      <c r="H484" t="n">
+        <v>7879.91</v>
+      </c>
+      <c r="I484" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J484" t="b">
+        <v>0</v>
+      </c>
+      <c r="K484" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7827.70 &lt;= EMA21 7879.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>ETERNAL</t>
+        </is>
+      </c>
+      <c r="D485" t="n">
+        <v>321.6</v>
+      </c>
+      <c r="E485" t="n">
+        <v>333.89</v>
+      </c>
+      <c r="F485" t="n">
+        <v>333.89</v>
+      </c>
+      <c r="G485" t="n">
+        <v>324.77</v>
+      </c>
+      <c r="H485" t="n">
+        <v>321.11</v>
+      </c>
+      <c r="I485" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="J485" t="b">
+        <v>0</v>
+      </c>
+      <c r="K485" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 321.60 &lt;= Upper 333.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>GAIL</t>
+        </is>
+      </c>
+      <c r="D486" t="n">
+        <v>175.09</v>
+      </c>
+      <c r="E486" t="n">
+        <v>177.49</v>
+      </c>
+      <c r="F486" t="n">
+        <v>177.49</v>
+      </c>
+      <c r="G486" t="n">
+        <v>174.21</v>
+      </c>
+      <c r="H486" t="n">
+        <v>173.82</v>
+      </c>
+      <c r="I486" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J486" t="b">
+        <v>0</v>
+      </c>
+      <c r="K486" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 175.09 &lt;= Upper 177.49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>GODREJCP</t>
+        </is>
+      </c>
+      <c r="D487" t="n">
+        <v>865</v>
+      </c>
+      <c r="E487" t="n">
+        <v>962.63</v>
+      </c>
+      <c r="F487" t="n">
+        <v>962.63</v>
+      </c>
+      <c r="G487" t="n">
+        <v>889.59</v>
+      </c>
+      <c r="H487" t="n">
+        <v>923.97</v>
+      </c>
+      <c r="I487" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="J487" t="b">
+        <v>0</v>
+      </c>
+      <c r="K487" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 889.59 &lt;= EMA21 923.97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>GRASIM</t>
+        </is>
+      </c>
+      <c r="D488" t="n">
+        <v>3306.8</v>
+      </c>
+      <c r="E488" t="n">
+        <v>3351.94</v>
+      </c>
+      <c r="F488" t="n">
+        <v>3351.94</v>
+      </c>
+      <c r="G488" t="n">
+        <v>3305.96</v>
+      </c>
+      <c r="H488" t="n">
+        <v>3282.26</v>
+      </c>
+      <c r="I488" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J488" t="b">
+        <v>0</v>
+      </c>
+      <c r="K488" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3306.80 &lt;= Upper 3351.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="D489" t="n">
+        <v>1277</v>
+      </c>
+      <c r="E489" t="n">
+        <v>1372.59</v>
+      </c>
+      <c r="F489" t="n">
+        <v>1372.59</v>
+      </c>
+      <c r="G489" t="n">
+        <v>1302.9</v>
+      </c>
+      <c r="H489" t="n">
+        <v>1308.36</v>
+      </c>
+      <c r="I489" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="J489" t="b">
+        <v>0</v>
+      </c>
+      <c r="K489" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1302.90 &lt;= EMA21 1308.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>HDFCAMC</t>
+        </is>
+      </c>
+      <c r="D490" t="n">
+        <v>2447.3</v>
+      </c>
+      <c r="E490" t="n">
+        <v>2690.33</v>
+      </c>
+      <c r="F490" t="n">
+        <v>2690.33</v>
+      </c>
+      <c r="G490" t="n">
+        <v>2523.89</v>
+      </c>
+      <c r="H490" t="n">
+        <v>2551.89</v>
+      </c>
+      <c r="I490" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J490" t="b">
+        <v>0</v>
+      </c>
+      <c r="K490" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2523.89 &lt;= EMA21 2551.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="D491" t="n">
+        <v>703</v>
+      </c>
+      <c r="E491" t="n">
+        <v>737.78</v>
+      </c>
+      <c r="F491" t="n">
+        <v>737.78</v>
+      </c>
+      <c r="G491" t="n">
+        <v>710.75</v>
+      </c>
+      <c r="H491" t="n">
+        <v>720.24</v>
+      </c>
+      <c r="I491" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J491" t="b">
+        <v>0</v>
+      </c>
+      <c r="K491" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 710.75 &lt;= EMA21 720.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="D492" t="n">
+        <v>533.8</v>
+      </c>
+      <c r="E492" t="n">
+        <v>555.99</v>
+      </c>
+      <c r="F492" t="n">
+        <v>555.99</v>
+      </c>
+      <c r="G492" t="n">
+        <v>538.97</v>
+      </c>
+      <c r="H492" t="n">
+        <v>542.41</v>
+      </c>
+      <c r="I492" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="J492" t="b">
+        <v>0</v>
+      </c>
+      <c r="K492" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 538.97 &lt;= EMA21 542.41)</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="D493" t="n">
+        <v>1009</v>
+      </c>
+      <c r="E493" t="n">
+        <v>1073.32</v>
+      </c>
+      <c r="F493" t="n">
+        <v>1073.32</v>
+      </c>
+      <c r="G493" t="n">
+        <v>1018.55</v>
+      </c>
+      <c r="H493" t="n">
+        <v>1021.83</v>
+      </c>
+      <c r="I493" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J493" t="b">
+        <v>0</v>
+      </c>
+      <c r="K493" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1018.55 &lt;= EMA21 1021.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="D494" t="n">
+        <v>5031.1</v>
+      </c>
+      <c r="E494" t="n">
+        <v>5121.46</v>
+      </c>
+      <c r="F494" t="n">
+        <v>5121.46</v>
+      </c>
+      <c r="G494" t="n">
+        <v>4879.31</v>
+      </c>
+      <c r="H494" t="n">
+        <v>4858.42</v>
+      </c>
+      <c r="I494" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="J494" t="b">
+        <v>0</v>
+      </c>
+      <c r="K494" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 5031.10 &lt;= Upper 5121.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="D495" t="n">
+        <v>1980</v>
+      </c>
+      <c r="E495" t="n">
+        <v>2094.91</v>
+      </c>
+      <c r="F495" t="n">
+        <v>2094.91</v>
+      </c>
+      <c r="G495" t="n">
+        <v>1988.65</v>
+      </c>
+      <c r="H495" t="n">
+        <v>2019.32</v>
+      </c>
+      <c r="I495" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="J495" t="b">
+        <v>0</v>
+      </c>
+      <c r="K495" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1988.65 &lt;= EMA21 2019.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+      <c r="D496" t="n">
+        <v>595.5</v>
+      </c>
+      <c r="E496" t="n">
+        <v>627.8099999999999</v>
+      </c>
+      <c r="F496" t="n">
+        <v>627.8099999999999</v>
+      </c>
+      <c r="G496" t="n">
+        <v>594.98</v>
+      </c>
+      <c r="H496" t="n">
+        <v>588.46</v>
+      </c>
+      <c r="I496" t="n">
+        <v>1</v>
+      </c>
+      <c r="J496" t="b">
+        <v>0</v>
+      </c>
+      <c r="K496" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 595.50 &lt;= Upper 627.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>HYUNDAI</t>
+        </is>
+      </c>
+      <c r="D497" t="n">
+        <v>2220</v>
+      </c>
+      <c r="E497" t="n">
+        <v>2273.79</v>
+      </c>
+      <c r="F497" t="n">
+        <v>2273.79</v>
+      </c>
+      <c r="G497" t="n">
+        <v>2203.29</v>
+      </c>
+      <c r="H497" t="n">
+        <v>2189.28</v>
+      </c>
+      <c r="I497" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J497" t="b">
+        <v>0</v>
+      </c>
+      <c r="K497" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 2220.00 &lt;= Upper 2273.79)</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="D498" t="n">
+        <v>1399.4</v>
+      </c>
+      <c r="E498" t="n">
+        <v>1449.43</v>
+      </c>
+      <c r="F498" t="n">
+        <v>1449.43</v>
+      </c>
+      <c r="G498" t="n">
+        <v>1422.96</v>
+      </c>
+      <c r="H498" t="n">
+        <v>1423.89</v>
+      </c>
+      <c r="I498" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="J498" t="b">
+        <v>0</v>
+      </c>
+      <c r="K498" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1422.96 &lt;= EMA21 1423.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="D499" t="n">
+        <v>263.5</v>
+      </c>
+      <c r="E499" t="n">
+        <v>279.74</v>
+      </c>
+      <c r="F499" t="n">
+        <v>279.74</v>
+      </c>
+      <c r="G499" t="n">
+        <v>264.98</v>
+      </c>
+      <c r="H499" t="n">
+        <v>269.1</v>
+      </c>
+      <c r="I499" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J499" t="b">
+        <v>0</v>
+      </c>
+      <c r="K499" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 264.98 &lt;= EMA21 269.10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>INDHOTEL</t>
+        </is>
+      </c>
+      <c r="D500" t="n">
+        <v>720</v>
+      </c>
+      <c r="E500" t="n">
+        <v>738.35</v>
+      </c>
+      <c r="F500" t="n">
+        <v>738.35</v>
+      </c>
+      <c r="G500" t="n">
+        <v>722.35</v>
+      </c>
+      <c r="H500" t="n">
+        <v>724.52</v>
+      </c>
+      <c r="I500" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J500" t="b">
+        <v>0</v>
+      </c>
+      <c r="K500" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 722.35 &lt;= EMA21 724.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>IOC</t>
+        </is>
+      </c>
+      <c r="D501" t="n">
+        <v>134.35</v>
+      </c>
+      <c r="E501" t="n">
+        <v>140.84</v>
+      </c>
+      <c r="F501" t="n">
+        <v>140.84</v>
+      </c>
+      <c r="G501" t="n">
+        <v>136.62</v>
+      </c>
+      <c r="H501" t="n">
+        <v>137.62</v>
+      </c>
+      <c r="I501" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="J501" t="b">
+        <v>0</v>
+      </c>
+      <c r="K501" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 136.62 &lt;= EMA21 137.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>IRFC</t>
+        </is>
+      </c>
+      <c r="D502" t="n">
+        <v>82</v>
+      </c>
+      <c r="E502" t="n">
+        <v>89.39</v>
+      </c>
+      <c r="F502" t="n">
+        <v>89.39</v>
+      </c>
+      <c r="G502" t="n">
+        <v>83.42</v>
+      </c>
+      <c r="H502" t="n">
+        <v>85.01000000000001</v>
+      </c>
+      <c r="I502" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J502" t="b">
+        <v>0</v>
+      </c>
+      <c r="K502" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 83.42 &lt;= EMA21 85.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="D503" t="n">
+        <v>1082</v>
+      </c>
+      <c r="E503" t="n">
+        <v>1182.58</v>
+      </c>
+      <c r="F503" t="n">
+        <v>1182.58</v>
+      </c>
+      <c r="G503" t="n">
+        <v>1116.93</v>
+      </c>
+      <c r="H503" t="n">
+        <v>1126.38</v>
+      </c>
+      <c r="I503" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J503" t="b">
+        <v>0</v>
+      </c>
+      <c r="K503" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1116.93 &lt;= EMA21 1126.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>INDIGO</t>
+        </is>
+      </c>
+      <c r="D504" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E504" t="n">
+        <v>5412.27</v>
+      </c>
+      <c r="F504" t="n">
+        <v>5412.27</v>
+      </c>
+      <c r="G504" t="n">
+        <v>5067.91</v>
+      </c>
+      <c r="H504" t="n">
+        <v>5140.12</v>
+      </c>
+      <c r="I504" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J504" t="b">
+        <v>0</v>
+      </c>
+      <c r="K504" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5067.91 &lt;= EMA21 5140.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>JSWSTEEL</t>
+        </is>
+      </c>
+      <c r="D505" t="n">
+        <v>1297.3</v>
+      </c>
+      <c r="E505" t="n">
+        <v>1349.99</v>
+      </c>
+      <c r="F505" t="n">
+        <v>1349.99</v>
+      </c>
+      <c r="G505" t="n">
+        <v>1309.32</v>
+      </c>
+      <c r="H505" t="n">
+        <v>1303.56</v>
+      </c>
+      <c r="I505" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J505" t="b">
+        <v>0</v>
+      </c>
+      <c r="K505" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1297.30 &lt;= Upper 1349.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>JINDALSTEL</t>
+        </is>
+      </c>
+      <c r="D506" t="n">
+        <v>1136.3</v>
+      </c>
+      <c r="E506" t="n">
+        <v>1201.01</v>
+      </c>
+      <c r="F506" t="n">
+        <v>1201.01</v>
+      </c>
+      <c r="G506" t="n">
+        <v>1153.52</v>
+      </c>
+      <c r="H506" t="n">
+        <v>1138.76</v>
+      </c>
+      <c r="I506" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="J506" t="b">
+        <v>0</v>
+      </c>
+      <c r="K506" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1136.30 &lt;= Upper 1201.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>JIOFIN</t>
+        </is>
+      </c>
+      <c r="D507" t="n">
+        <v>233.15</v>
+      </c>
+      <c r="E507" t="n">
+        <v>256.33</v>
+      </c>
+      <c r="F507" t="n">
+        <v>256.33</v>
+      </c>
+      <c r="G507" t="n">
+        <v>238.32</v>
+      </c>
+      <c r="H507" t="n">
+        <v>241.71</v>
+      </c>
+      <c r="I507" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J507" t="b">
+        <v>0</v>
+      </c>
+      <c r="K507" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 238.32 &lt;= EMA21 241.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="D508" t="n">
+        <v>419.25</v>
+      </c>
+      <c r="E508" t="n">
+        <v>437.51</v>
+      </c>
+      <c r="F508" t="n">
+        <v>437.51</v>
+      </c>
+      <c r="G508" t="n">
+        <v>419.2</v>
+      </c>
+      <c r="H508" t="n">
+        <v>411.13</v>
+      </c>
+      <c r="I508" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J508" t="b">
+        <v>0</v>
+      </c>
+      <c r="K508" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 419.25 &lt;= Upper 437.51)</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>LTM</t>
+        </is>
+      </c>
+      <c r="D509" t="n">
+        <v>4430</v>
+      </c>
+      <c r="E509" t="n">
+        <v>4778.8</v>
+      </c>
+      <c r="F509" t="n">
+        <v>4778.8</v>
+      </c>
+      <c r="G509" t="n">
+        <v>4520.74</v>
+      </c>
+      <c r="H509" t="n">
+        <v>4521.83</v>
+      </c>
+      <c r="I509" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="J509" t="b">
+        <v>0</v>
+      </c>
+      <c r="K509" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4520.74 &lt;= EMA21 4521.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="D510" t="n">
+        <v>3946.1</v>
+      </c>
+      <c r="E510" t="n">
+        <v>4133.68</v>
+      </c>
+      <c r="F510" t="n">
+        <v>4133.68</v>
+      </c>
+      <c r="G510" t="n">
+        <v>3993.55</v>
+      </c>
+      <c r="H510" t="n">
+        <v>4009.61</v>
+      </c>
+      <c r="I510" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J510" t="b">
+        <v>0</v>
+      </c>
+      <c r="K510" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3993.55 &lt;= EMA21 4009.61)</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>LODHA</t>
+        </is>
+      </c>
+      <c r="D511" t="n">
+        <v>1212</v>
+      </c>
+      <c r="E511" t="n">
+        <v>1283.56</v>
+      </c>
+      <c r="F511" t="n">
+        <v>1283.56</v>
+      </c>
+      <c r="G511" t="n">
+        <v>1224.56</v>
+      </c>
+      <c r="H511" t="n">
+        <v>1224.31</v>
+      </c>
+      <c r="I511" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J511" t="b">
+        <v>0</v>
+      </c>
+      <c r="K511" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1212.00 &lt;= Upper 1283.56)</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>M&amp;M</t>
+        </is>
+      </c>
+      <c r="D512" t="n">
+        <v>3160</v>
+      </c>
+      <c r="E512" t="n">
+        <v>3549.3</v>
+      </c>
+      <c r="F512" t="n">
+        <v>3549.3</v>
+      </c>
+      <c r="G512" t="n">
+        <v>3223.1</v>
+      </c>
+      <c r="H512" t="n">
+        <v>3284.34</v>
+      </c>
+      <c r="I512" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="J512" t="b">
+        <v>0</v>
+      </c>
+      <c r="K512" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3223.10 &lt;= EMA21 3284.34)</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="D513" t="n">
+        <v>12641</v>
+      </c>
+      <c r="E513" t="n">
+        <v>14274.91</v>
+      </c>
+      <c r="F513" t="n">
+        <v>14274.91</v>
+      </c>
+      <c r="G513" t="n">
+        <v>12971.28</v>
+      </c>
+      <c r="H513" t="n">
+        <v>13281.74</v>
+      </c>
+      <c r="I513" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J513" t="b">
+        <v>0</v>
+      </c>
+      <c r="K513" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 12971.28 &lt;= EMA21 13281.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>MAXHEALTH</t>
+        </is>
+      </c>
+      <c r="D514" t="n">
+        <v>993</v>
+      </c>
+      <c r="E514" t="n">
+        <v>1035.77</v>
+      </c>
+      <c r="F514" t="n">
+        <v>1035.77</v>
+      </c>
+      <c r="G514" t="n">
+        <v>1000.71</v>
+      </c>
+      <c r="H514" t="n">
+        <v>1016.22</v>
+      </c>
+      <c r="I514" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J514" t="b">
+        <v>0</v>
+      </c>
+      <c r="K514" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1000.71 &lt;= EMA21 1016.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>MAZDOCK</t>
+        </is>
+      </c>
+      <c r="D515" t="n">
+        <v>2466.4</v>
+      </c>
+      <c r="E515" t="n">
+        <v>2641.47</v>
+      </c>
+      <c r="F515" t="n">
+        <v>2641.47</v>
+      </c>
+      <c r="G515" t="n">
+        <v>2497.89</v>
+      </c>
+      <c r="H515" t="n">
+        <v>2505.41</v>
+      </c>
+      <c r="I515" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J515" t="b">
+        <v>0</v>
+      </c>
+      <c r="K515" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2497.89 &lt;= EMA21 2505.41)</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>MUTHOOTFIN</t>
+        </is>
+      </c>
+      <c r="D516" t="n">
+        <v>2899.7</v>
+      </c>
+      <c r="E516" t="n">
+        <v>3215.51</v>
+      </c>
+      <c r="F516" t="n">
+        <v>3215.51</v>
+      </c>
+      <c r="G516" t="n">
+        <v>2944.85</v>
+      </c>
+      <c r="H516" t="n">
+        <v>2969.69</v>
+      </c>
+      <c r="I516" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J516" t="b">
+        <v>0</v>
+      </c>
+      <c r="K516" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2944.85 &lt;= EMA21 2969.69)</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="D517" t="n">
+        <v>330.8</v>
+      </c>
+      <c r="E517" t="n">
+        <v>340.85</v>
+      </c>
+      <c r="F517" t="n">
+        <v>340.85</v>
+      </c>
+      <c r="G517" t="n">
+        <v>330.6</v>
+      </c>
+      <c r="H517" t="n">
+        <v>332.77</v>
+      </c>
+      <c r="I517" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J517" t="b">
+        <v>0</v>
+      </c>
+      <c r="K517" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 330.60 &lt;= EMA21 332.77)</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="D518" t="n">
+        <v>1400.5</v>
+      </c>
+      <c r="E518" t="n">
+        <v>1524.36</v>
+      </c>
+      <c r="F518" t="n">
+        <v>1524.36</v>
+      </c>
+      <c r="G518" t="n">
+        <v>1426.19</v>
+      </c>
+      <c r="H518" t="n">
+        <v>1448.76</v>
+      </c>
+      <c r="I518" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J518" t="b">
+        <v>0</v>
+      </c>
+      <c r="K518" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1426.19 &lt;= EMA21 1448.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="D519" t="n">
+        <v>236</v>
+      </c>
+      <c r="E519" t="n">
+        <v>240.22</v>
+      </c>
+      <c r="F519" t="n">
+        <v>240.22</v>
+      </c>
+      <c r="G519" t="n">
+        <v>234.62</v>
+      </c>
+      <c r="H519" t="n">
+        <v>235.64</v>
+      </c>
+      <c r="I519" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J519" t="b">
+        <v>0</v>
+      </c>
+      <c r="K519" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 234.62 &lt;= EMA21 235.64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>PIDILITIND</t>
+        </is>
+      </c>
+      <c r="D520" t="n">
+        <v>1593</v>
+      </c>
+      <c r="E520" t="n">
+        <v>1715.72</v>
+      </c>
+      <c r="F520" t="n">
+        <v>1715.72</v>
+      </c>
+      <c r="G520" t="n">
+        <v>1623.76</v>
+      </c>
+      <c r="H520" t="n">
+        <v>1636.48</v>
+      </c>
+      <c r="I520" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J520" t="b">
+        <v>0</v>
+      </c>
+      <c r="K520" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1623.76 &lt;= EMA21 1636.48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>PFC</t>
+        </is>
+      </c>
+      <c r="D521" t="n">
+        <v>355.9</v>
+      </c>
+      <c r="E521" t="n">
+        <v>380.28</v>
+      </c>
+      <c r="F521" t="n">
+        <v>380.28</v>
+      </c>
+      <c r="G521" t="n">
+        <v>353.18</v>
+      </c>
+      <c r="H521" t="n">
+        <v>362.61</v>
+      </c>
+      <c r="I521" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J521" t="b">
+        <v>0</v>
+      </c>
+      <c r="K521" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 353.18 &lt;= EMA21 362.61)</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="D522" t="n">
+        <v>265.75</v>
+      </c>
+      <c r="E522" t="n">
+        <v>271.84</v>
+      </c>
+      <c r="F522" t="n">
+        <v>271.84</v>
+      </c>
+      <c r="G522" t="n">
+        <v>266.12</v>
+      </c>
+      <c r="H522" t="n">
+        <v>268.68</v>
+      </c>
+      <c r="I522" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J522" t="b">
+        <v>0</v>
+      </c>
+      <c r="K522" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 266.12 &lt;= EMA21 268.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="D523" t="n">
+        <v>116</v>
+      </c>
+      <c r="E523" t="n">
+        <v>118.85</v>
+      </c>
+      <c r="F523" t="n">
+        <v>118.85</v>
+      </c>
+      <c r="G523" t="n">
+        <v>116.05</v>
+      </c>
+      <c r="H523" t="n">
+        <v>115.53</v>
+      </c>
+      <c r="I523" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J523" t="b">
+        <v>0</v>
+      </c>
+      <c r="K523" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 116.00 &lt;= Upper 118.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="D524" t="n">
+        <v>317.85</v>
+      </c>
+      <c r="E524" t="n">
+        <v>346.91</v>
+      </c>
+      <c r="F524" t="n">
+        <v>346.91</v>
+      </c>
+      <c r="G524" t="n">
+        <v>319.1</v>
+      </c>
+      <c r="H524" t="n">
+        <v>327.19</v>
+      </c>
+      <c r="I524" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J524" t="b">
+        <v>0</v>
+      </c>
+      <c r="K524" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 319.10 &lt;= EMA21 327.19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="D525" t="n">
+        <v>1294.9</v>
+      </c>
+      <c r="E525" t="n">
+        <v>1335.2</v>
+      </c>
+      <c r="F525" t="n">
+        <v>1335.2</v>
+      </c>
+      <c r="G525" t="n">
+        <v>1304.41</v>
+      </c>
+      <c r="H525" t="n">
+        <v>1305.28</v>
+      </c>
+      <c r="I525" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J525" t="b">
+        <v>0</v>
+      </c>
+      <c r="K525" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1304.41 &lt;= EMA21 1305.28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="D526" t="n">
+        <v>1696.6</v>
+      </c>
+      <c r="E526" t="n">
+        <v>1831.91</v>
+      </c>
+      <c r="F526" t="n">
+        <v>1831.91</v>
+      </c>
+      <c r="G526" t="n">
+        <v>1738.03</v>
+      </c>
+      <c r="H526" t="n">
+        <v>1765.91</v>
+      </c>
+      <c r="I526" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="J526" t="b">
+        <v>0</v>
+      </c>
+      <c r="K526" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1738.03 &lt;= EMA21 1765.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>MOTHERSON</t>
+        </is>
+      </c>
+      <c r="D527" t="n">
+        <v>163.85</v>
+      </c>
+      <c r="E527" t="n">
+        <v>172.84</v>
+      </c>
+      <c r="F527" t="n">
+        <v>172.84</v>
+      </c>
+      <c r="G527" t="n">
+        <v>163.98</v>
+      </c>
+      <c r="H527" t="n">
+        <v>163.57</v>
+      </c>
+      <c r="I527" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J527" t="b">
+        <v>0</v>
+      </c>
+      <c r="K527" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 163.85 &lt;= Upper 172.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="D528" t="n">
+        <v>23160</v>
+      </c>
+      <c r="E528" t="n">
+        <v>25522.68</v>
+      </c>
+      <c r="F528" t="n">
+        <v>25522.68</v>
+      </c>
+      <c r="G528" t="n">
+        <v>23706.97</v>
+      </c>
+      <c r="H528" t="n">
+        <v>24293.83</v>
+      </c>
+      <c r="I528" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="J528" t="b">
+        <v>0</v>
+      </c>
+      <c r="K528" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 23706.97 &lt;= EMA21 24293.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>SHRIRAMFIN</t>
+        </is>
+      </c>
+      <c r="D529" t="n">
+        <v>1029</v>
+      </c>
+      <c r="E529" t="n">
+        <v>1168.9</v>
+      </c>
+      <c r="F529" t="n">
+        <v>1168.9</v>
+      </c>
+      <c r="G529" t="n">
+        <v>1058.34</v>
+      </c>
+      <c r="H529" t="n">
+        <v>1076.91</v>
+      </c>
+      <c r="I529" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J529" t="b">
+        <v>0</v>
+      </c>
+      <c r="K529" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1058.34 &lt;= EMA21 1076.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>ENRIN</t>
+        </is>
+      </c>
+      <c r="D530" t="n">
+        <v>3200.1</v>
+      </c>
+      <c r="E530" t="n">
+        <v>3703.34</v>
+      </c>
+      <c r="F530" t="n">
+        <v>3703.34</v>
+      </c>
+      <c r="G530" t="n">
+        <v>3201.1</v>
+      </c>
+      <c r="H530" t="n">
+        <v>3285.7</v>
+      </c>
+      <c r="I530" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="J530" t="b">
+        <v>0</v>
+      </c>
+      <c r="K530" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3201.10 &lt;= EMA21 3285.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+      <c r="D531" t="n">
+        <v>3951.3</v>
+      </c>
+      <c r="E531" t="n">
+        <v>4135.7</v>
+      </c>
+      <c r="F531" t="n">
+        <v>4135.7</v>
+      </c>
+      <c r="G531" t="n">
+        <v>3990.43</v>
+      </c>
+      <c r="H531" t="n">
+        <v>3968.94</v>
+      </c>
+      <c r="I531" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J531" t="b">
+        <v>0</v>
+      </c>
+      <c r="K531" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3951.30 &lt;= Upper 4135.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>SOLARINDS</t>
+        </is>
+      </c>
+      <c r="D532" t="n">
+        <v>22455</v>
+      </c>
+      <c r="E532" t="n">
+        <v>22105.91</v>
+      </c>
+      <c r="F532" t="n">
+        <v>22105.91</v>
+      </c>
+      <c r="G532" t="n">
+        <v>21210.39</v>
+      </c>
+      <c r="H532" t="n">
+        <v>20430.5</v>
+      </c>
+      <c r="I532" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="J532" t="b">
+        <v>0</v>
+      </c>
+      <c r="K532" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 1.11x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="D533" t="n">
+        <v>1008</v>
+      </c>
+      <c r="E533" t="n">
+        <v>1087.83</v>
+      </c>
+      <c r="F533" t="n">
+        <v>1087.83</v>
+      </c>
+      <c r="G533" t="n">
+        <v>1024.53</v>
+      </c>
+      <c r="H533" t="n">
+        <v>1036.22</v>
+      </c>
+      <c r="I533" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J533" t="b">
+        <v>0</v>
+      </c>
+      <c r="K533" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1024.53 &lt;= EMA21 1036.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="D534" t="n">
+        <v>1885.9</v>
+      </c>
+      <c r="E534" t="n">
+        <v>1963.42</v>
+      </c>
+      <c r="F534" t="n">
+        <v>1963.42</v>
+      </c>
+      <c r="G534" t="n">
+        <v>1909.54</v>
+      </c>
+      <c r="H534" t="n">
+        <v>1917.73</v>
+      </c>
+      <c r="I534" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J534" t="b">
+        <v>0</v>
+      </c>
+      <c r="K534" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1909.54 &lt;= EMA21 1917.73)</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>TVSMOTOR</t>
+        </is>
+      </c>
+      <c r="D535" t="n">
+        <v>4133.2</v>
+      </c>
+      <c r="E535" t="n">
+        <v>4519.95</v>
+      </c>
+      <c r="F535" t="n">
+        <v>4519.95</v>
+      </c>
+      <c r="G535" t="n">
+        <v>4212.15</v>
+      </c>
+      <c r="H535" t="n">
+        <v>4243.85</v>
+      </c>
+      <c r="I535" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J535" t="b">
+        <v>0</v>
+      </c>
+      <c r="K535" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4212.15 &lt;= EMA21 4243.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>TATACAP</t>
+        </is>
+      </c>
+      <c r="D536" t="n">
+        <v>368.05</v>
+      </c>
+      <c r="E536" t="n">
+        <v>376.53</v>
+      </c>
+      <c r="F536" t="n">
+        <v>376.53</v>
+      </c>
+      <c r="G536" t="n">
+        <v>369.63</v>
+      </c>
+      <c r="H536" t="n">
+        <v>367.62</v>
+      </c>
+      <c r="I536" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J536" t="b">
+        <v>0</v>
+      </c>
+      <c r="K536" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 368.05 &lt;= Upper 376.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="D537" t="n">
+        <v>2255.5</v>
+      </c>
+      <c r="E537" t="n">
+        <v>2399.04</v>
+      </c>
+      <c r="F537" t="n">
+        <v>2399.04</v>
+      </c>
+      <c r="G537" t="n">
+        <v>2303.23</v>
+      </c>
+      <c r="H537" t="n">
+        <v>2314.06</v>
+      </c>
+      <c r="I537" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J537" t="b">
+        <v>0</v>
+      </c>
+      <c r="K537" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2303.23 &lt;= EMA21 2314.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>TATACONSUM</t>
+        </is>
+      </c>
+      <c r="D538" t="n">
+        <v>1014.1</v>
+      </c>
+      <c r="E538" t="n">
+        <v>1094.4</v>
+      </c>
+      <c r="F538" t="n">
+        <v>1094.4</v>
+      </c>
+      <c r="G538" t="n">
+        <v>1024.82</v>
+      </c>
+      <c r="H538" t="n">
+        <v>1043.88</v>
+      </c>
+      <c r="I538" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J538" t="b">
+        <v>0</v>
+      </c>
+      <c r="K538" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1024.82 &lt;= EMA21 1043.88)</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>TMCV</t>
+        </is>
+      </c>
+      <c r="D539" t="n">
+        <v>456.05</v>
+      </c>
+      <c r="E539" t="n">
+        <v>486.86</v>
+      </c>
+      <c r="F539" t="n">
+        <v>486.86</v>
+      </c>
+      <c r="G539" t="n">
+        <v>461.32</v>
+      </c>
+      <c r="H539" t="n">
+        <v>460.48</v>
+      </c>
+      <c r="I539" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J539" t="b">
+        <v>0</v>
+      </c>
+      <c r="K539" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 456.05 &lt;= Upper 486.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>TMPV</t>
+        </is>
+      </c>
+      <c r="D540" t="n">
+        <v>306.45</v>
+      </c>
+      <c r="E540" t="n">
+        <v>342.73</v>
+      </c>
+      <c r="F540" t="n">
+        <v>342.73</v>
+      </c>
+      <c r="G540" t="n">
+        <v>311.49</v>
+      </c>
+      <c r="H540" t="n">
+        <v>318.64</v>
+      </c>
+      <c r="I540" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J540" t="b">
+        <v>0</v>
+      </c>
+      <c r="K540" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 311.49 &lt;= EMA21 318.64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>TATAPOWER</t>
+        </is>
+      </c>
+      <c r="D541" t="n">
+        <v>365.55</v>
+      </c>
+      <c r="E541" t="n">
+        <v>391.39</v>
+      </c>
+      <c r="F541" t="n">
+        <v>391.39</v>
+      </c>
+      <c r="G541" t="n">
+        <v>363.88</v>
+      </c>
+      <c r="H541" t="n">
+        <v>367.47</v>
+      </c>
+      <c r="I541" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J541" t="b">
+        <v>0</v>
+      </c>
+      <c r="K541" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 363.88 &lt;= EMA21 367.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="D542" t="n">
+        <v>184.15</v>
+      </c>
+      <c r="E542" t="n">
+        <v>188.52</v>
+      </c>
+      <c r="F542" t="n">
+        <v>188.52</v>
+      </c>
+      <c r="G542" t="n">
+        <v>185.41</v>
+      </c>
+      <c r="H542" t="n">
+        <v>185.86</v>
+      </c>
+      <c r="I542" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J542" t="b">
+        <v>0</v>
+      </c>
+      <c r="K542" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 185.41 &lt;= EMA21 185.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>TECHM</t>
+        </is>
+      </c>
+      <c r="D543" t="n">
+        <v>1559</v>
+      </c>
+      <c r="E543" t="n">
+        <v>1653.74</v>
+      </c>
+      <c r="F543" t="n">
+        <v>1653.74</v>
+      </c>
+      <c r="G543" t="n">
+        <v>1591.8</v>
+      </c>
+      <c r="H543" t="n">
+        <v>1597.45</v>
+      </c>
+      <c r="I543" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J543" t="b">
+        <v>0</v>
+      </c>
+      <c r="K543" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1591.80 &lt;= EMA21 1597.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>TITAN</t>
+        </is>
+      </c>
+      <c r="D544" t="n">
+        <v>4987</v>
+      </c>
+      <c r="E544" t="n">
+        <v>5161.58</v>
+      </c>
+      <c r="F544" t="n">
+        <v>5161.58</v>
+      </c>
+      <c r="G544" t="n">
+        <v>5038.86</v>
+      </c>
+      <c r="H544" t="n">
+        <v>5025.95</v>
+      </c>
+      <c r="I544" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J544" t="b">
+        <v>0</v>
+      </c>
+      <c r="K544" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 4987.00 &lt;= Upper 5161.58)</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>TORNTPHARM</t>
+        </is>
+      </c>
+      <c r="D545" t="n">
+        <v>4960</v>
+      </c>
+      <c r="E545" t="n">
+        <v>5072.94</v>
+      </c>
+      <c r="F545" t="n">
+        <v>5072.94</v>
+      </c>
+      <c r="G545" t="n">
+        <v>4944.17</v>
+      </c>
+      <c r="H545" t="n">
+        <v>4944.45</v>
+      </c>
+      <c r="I545" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J545" t="b">
+        <v>0</v>
+      </c>
+      <c r="K545" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4944.17 &lt;= EMA21 4944.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="D546" t="n">
+        <v>2793.6</v>
+      </c>
+      <c r="E546" t="n">
+        <v>3023.14</v>
+      </c>
+      <c r="F546" t="n">
+        <v>3023.14</v>
+      </c>
+      <c r="G546" t="n">
+        <v>2847.12</v>
+      </c>
+      <c r="H546" t="n">
+        <v>2893.68</v>
+      </c>
+      <c r="I546" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J546" t="b">
+        <v>0</v>
+      </c>
+      <c r="K546" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2847.12 &lt;= EMA21 2893.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="D547" t="n">
+        <v>11009</v>
+      </c>
+      <c r="E547" t="n">
+        <v>11915.52</v>
+      </c>
+      <c r="F547" t="n">
+        <v>11915.52</v>
+      </c>
+      <c r="G547" t="n">
+        <v>11324.75</v>
+      </c>
+      <c r="H547" t="n">
+        <v>11476.75</v>
+      </c>
+      <c r="I547" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="J547" t="b">
+        <v>0</v>
+      </c>
+      <c r="K547" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11324.75 &lt;= EMA21 11476.75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="D548" t="n">
+        <v>183.22</v>
+      </c>
+      <c r="E548" t="n">
+        <v>189.74</v>
+      </c>
+      <c r="F548" t="n">
+        <v>189.74</v>
+      </c>
+      <c r="G548" t="n">
+        <v>185.91</v>
+      </c>
+      <c r="H548" t="n">
+        <v>184.4</v>
+      </c>
+      <c r="I548" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="J548" t="b">
+        <v>0</v>
+      </c>
+      <c r="K548" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 183.22 &lt;= Upper 189.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>UNITDSPR</t>
+        </is>
+      </c>
+      <c r="D549" t="n">
+        <v>1440</v>
+      </c>
+      <c r="E549" t="n">
+        <v>1585.13</v>
+      </c>
+      <c r="F549" t="n">
+        <v>1585.13</v>
+      </c>
+      <c r="G549" t="n">
+        <v>1475.25</v>
+      </c>
+      <c r="H549" t="n">
+        <v>1491.85</v>
+      </c>
+      <c r="I549" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J549" t="b">
+        <v>0</v>
+      </c>
+      <c r="K549" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1475.25 &lt;= EMA21 1491.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="D550" t="n">
+        <v>405.7</v>
+      </c>
+      <c r="E550" t="n">
+        <v>451.14</v>
+      </c>
+      <c r="F550" t="n">
+        <v>451.14</v>
+      </c>
+      <c r="G550" t="n">
+        <v>411.02</v>
+      </c>
+      <c r="H550" t="n">
+        <v>421.93</v>
+      </c>
+      <c r="I550" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J550" t="b">
+        <v>0</v>
+      </c>
+      <c r="K550" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 411.02 &lt;= EMA21 421.93)</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>VEDL</t>
+        </is>
+      </c>
+      <c r="D551" t="n">
+        <v>272</v>
+      </c>
+      <c r="E551" t="n">
+        <v>286.93</v>
+      </c>
+      <c r="F551" t="n">
+        <v>286.93</v>
+      </c>
+      <c r="G551" t="n">
+        <v>272.99</v>
+      </c>
+      <c r="H551" t="n">
+        <v>273.58</v>
+      </c>
+      <c r="I551" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J551" t="b">
+        <v>0</v>
+      </c>
+      <c r="K551" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 272.99 &lt;= EMA21 273.58)</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="D552" t="n">
+        <v>171.5</v>
+      </c>
+      <c r="E552" t="n">
+        <v>186.7</v>
+      </c>
+      <c r="F552" t="n">
+        <v>186.7</v>
+      </c>
+      <c r="G552" t="n">
+        <v>176.34</v>
+      </c>
+      <c r="H552" t="n">
+        <v>178.55</v>
+      </c>
+      <c r="I552" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J552" t="b">
+        <v>0</v>
+      </c>
+      <c r="K552" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 176.34 &lt;= EMA21 178.55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>ZYDUSLIFE</t>
+        </is>
+      </c>
+      <c r="D553" t="n">
+        <v>1145.5</v>
+      </c>
+      <c r="E553" t="n">
+        <v>1204.08</v>
+      </c>
+      <c r="F553" t="n">
+        <v>1204.08</v>
+      </c>
+      <c r="G553" t="n">
+        <v>1147.78</v>
+      </c>
+      <c r="H553" t="n">
+        <v>1143.67</v>
+      </c>
+      <c r="I553" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="J553" t="b">
+        <v>0</v>
+      </c>
+      <c r="K553" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1145.50 &lt;= Upper 1204.08)</t>
         </is>
       </c>
     </row>
@@ -26276,7 +30576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26590,6 +30890,39 @@
         <v>1</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>20:03:54</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>179135.98</v>
+      </c>
+      <c r="D10" t="n">
+        <v>19685.95</v>
+      </c>
+      <c r="E10" t="n">
+        <v>198821.93</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-1092.43</v>
+      </c>
+      <c r="G10" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H10" t="n">
+        <v>17</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-09T20:07 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_india.xlsx
+++ b/data/trade_log_india.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K553"/>
+  <dimension ref="A1:K653"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24206,6 +24206,4306 @@
       <c r="K553" t="inlineStr">
         <is>
           <t>BELOW_BAND (Close 1145.50 &lt;= Upper 1204.08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+      <c r="D554" t="n">
+        <v>7401.5</v>
+      </c>
+      <c r="E554" t="n">
+        <v>7745.32</v>
+      </c>
+      <c r="F554" t="n">
+        <v>7745.32</v>
+      </c>
+      <c r="G554" t="n">
+        <v>7447.41</v>
+      </c>
+      <c r="H554" t="n">
+        <v>7468.54</v>
+      </c>
+      <c r="I554" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="J554" t="b">
+        <v>0</v>
+      </c>
+      <c r="K554" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7447.41 &lt;= EMA21 7468.54)</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="D555" t="n">
+        <v>1423.3</v>
+      </c>
+      <c r="E555" t="n">
+        <v>1691.1</v>
+      </c>
+      <c r="F555" t="n">
+        <v>1691.1</v>
+      </c>
+      <c r="G555" t="n">
+        <v>1434.91</v>
+      </c>
+      <c r="H555" t="n">
+        <v>1493.81</v>
+      </c>
+      <c r="I555" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="J555" t="b">
+        <v>0</v>
+      </c>
+      <c r="K555" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1434.91 &lt;= EMA21 1493.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>ADANIENT</t>
+        </is>
+      </c>
+      <c r="D556" t="n">
+        <v>3104.7</v>
+      </c>
+      <c r="E556" t="n">
+        <v>3186.19</v>
+      </c>
+      <c r="F556" t="n">
+        <v>3186.19</v>
+      </c>
+      <c r="G556" t="n">
+        <v>2987.05</v>
+      </c>
+      <c r="H556" t="n">
+        <v>2999.13</v>
+      </c>
+      <c r="I556" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="J556" t="b">
+        <v>0</v>
+      </c>
+      <c r="K556" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2987.05 &lt;= EMA21 2999.13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>ADANIGREEN</t>
+        </is>
+      </c>
+      <c r="D557" t="n">
+        <v>1315</v>
+      </c>
+      <c r="E557" t="n">
+        <v>1358.69</v>
+      </c>
+      <c r="F557" t="n">
+        <v>1358.69</v>
+      </c>
+      <c r="G557" t="n">
+        <v>1296.52</v>
+      </c>
+      <c r="H557" t="n">
+        <v>1313.82</v>
+      </c>
+      <c r="I557" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="J557" t="b">
+        <v>0</v>
+      </c>
+      <c r="K557" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1296.52 &lt;= EMA21 1313.82)</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="D558" t="n">
+        <v>1775</v>
+      </c>
+      <c r="E558" t="n">
+        <v>1758.35</v>
+      </c>
+      <c r="F558" t="n">
+        <v>1758.35</v>
+      </c>
+      <c r="G558" t="n">
+        <v>1706.41</v>
+      </c>
+      <c r="H558" t="n">
+        <v>1701.36</v>
+      </c>
+      <c r="I558" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="J558" t="b">
+        <v>1</v>
+      </c>
+      <c r="K558" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="D559" t="n">
+        <v>214.9</v>
+      </c>
+      <c r="E559" t="n">
+        <v>214.59</v>
+      </c>
+      <c r="F559" t="n">
+        <v>214.59</v>
+      </c>
+      <c r="G559" t="n">
+        <v>208.42</v>
+      </c>
+      <c r="H559" t="n">
+        <v>208.15</v>
+      </c>
+      <c r="I559" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="J559" t="b">
+        <v>1</v>
+      </c>
+      <c r="K559" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>AMBUJACEM</t>
+        </is>
+      </c>
+      <c r="D560" t="n">
+        <v>397</v>
+      </c>
+      <c r="E560" t="n">
+        <v>422.68</v>
+      </c>
+      <c r="F560" t="n">
+        <v>422.68</v>
+      </c>
+      <c r="G560" t="n">
+        <v>402.59</v>
+      </c>
+      <c r="H560" t="n">
+        <v>409.37</v>
+      </c>
+      <c r="I560" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="J560" t="b">
+        <v>0</v>
+      </c>
+      <c r="K560" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 402.59 &lt;= EMA21 409.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="D561" t="n">
+        <v>8967</v>
+      </c>
+      <c r="E561" t="n">
+        <v>8981.360000000001</v>
+      </c>
+      <c r="F561" t="n">
+        <v>8981.360000000001</v>
+      </c>
+      <c r="G561" t="n">
+        <v>8803.450000000001</v>
+      </c>
+      <c r="H561" t="n">
+        <v>8797.049999999999</v>
+      </c>
+      <c r="I561" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J561" t="b">
+        <v>0</v>
+      </c>
+      <c r="K561" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 8967.00 &lt;= Upper 8981.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="D562" t="n">
+        <v>2489</v>
+      </c>
+      <c r="E562" t="n">
+        <v>2752.7</v>
+      </c>
+      <c r="F562" t="n">
+        <v>2752.7</v>
+      </c>
+      <c r="G562" t="n">
+        <v>2536.98</v>
+      </c>
+      <c r="H562" t="n">
+        <v>2593.69</v>
+      </c>
+      <c r="I562" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J562" t="b">
+        <v>0</v>
+      </c>
+      <c r="K562" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2536.98 &lt;= EMA21 2593.69)</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="D563" t="n">
+        <v>3735</v>
+      </c>
+      <c r="E563" t="n">
+        <v>4094.47</v>
+      </c>
+      <c r="F563" t="n">
+        <v>4094.47</v>
+      </c>
+      <c r="G563" t="n">
+        <v>3779.22</v>
+      </c>
+      <c r="H563" t="n">
+        <v>3849.67</v>
+      </c>
+      <c r="I563" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="J563" t="b">
+        <v>0</v>
+      </c>
+      <c r="K563" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3779.22 &lt;= EMA21 3849.67)</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="D564" t="n">
+        <v>1238.5</v>
+      </c>
+      <c r="E564" t="n">
+        <v>1286.67</v>
+      </c>
+      <c r="F564" t="n">
+        <v>1286.67</v>
+      </c>
+      <c r="G564" t="n">
+        <v>1254.72</v>
+      </c>
+      <c r="H564" t="n">
+        <v>1253.87</v>
+      </c>
+      <c r="I564" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="J564" t="b">
+        <v>0</v>
+      </c>
+      <c r="K564" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1238.50 &lt;= Upper 1286.67)</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO</t>
+        </is>
+      </c>
+      <c r="D565" t="n">
+        <v>11790</v>
+      </c>
+      <c r="E565" t="n">
+        <v>12222.06</v>
+      </c>
+      <c r="F565" t="n">
+        <v>12222.06</v>
+      </c>
+      <c r="G565" t="n">
+        <v>11892.88</v>
+      </c>
+      <c r="H565" t="n">
+        <v>11793.01</v>
+      </c>
+      <c r="I565" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="J565" t="b">
+        <v>0</v>
+      </c>
+      <c r="K565" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 11790.00 &lt;= Upper 12222.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="D566" t="n">
+        <v>1039.3</v>
+      </c>
+      <c r="E566" t="n">
+        <v>1109.41</v>
+      </c>
+      <c r="F566" t="n">
+        <v>1109.41</v>
+      </c>
+      <c r="G566" t="n">
+        <v>1057.71</v>
+      </c>
+      <c r="H566" t="n">
+        <v>1067.63</v>
+      </c>
+      <c r="I566" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="J566" t="b">
+        <v>0</v>
+      </c>
+      <c r="K566" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1057.71 &lt;= EMA21 1067.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="D567" t="n">
+        <v>1927</v>
+      </c>
+      <c r="E567" t="n">
+        <v>2054.43</v>
+      </c>
+      <c r="F567" t="n">
+        <v>2054.43</v>
+      </c>
+      <c r="G567" t="n">
+        <v>1964.38</v>
+      </c>
+      <c r="H567" t="n">
+        <v>1979.63</v>
+      </c>
+      <c r="I567" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J567" t="b">
+        <v>0</v>
+      </c>
+      <c r="K567" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1964.38 &lt;= EMA21 1979.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>BAJAJHLDNG</t>
+        </is>
+      </c>
+      <c r="D568" t="n">
+        <v>11078</v>
+      </c>
+      <c r="E568" t="n">
+        <v>11652.07</v>
+      </c>
+      <c r="F568" t="n">
+        <v>11652.07</v>
+      </c>
+      <c r="G568" t="n">
+        <v>11157.74</v>
+      </c>
+      <c r="H568" t="n">
+        <v>11212.08</v>
+      </c>
+      <c r="I568" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J568" t="b">
+        <v>0</v>
+      </c>
+      <c r="K568" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11157.74 &lt;= EMA21 11212.08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>BANKBARODA</t>
+        </is>
+      </c>
+      <c r="D569" t="n">
+        <v>234.1</v>
+      </c>
+      <c r="E569" t="n">
+        <v>249.74</v>
+      </c>
+      <c r="F569" t="n">
+        <v>249.74</v>
+      </c>
+      <c r="G569" t="n">
+        <v>238.25</v>
+      </c>
+      <c r="H569" t="n">
+        <v>241.2</v>
+      </c>
+      <c r="I569" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="J569" t="b">
+        <v>0</v>
+      </c>
+      <c r="K569" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 238.25 &lt;= EMA21 241.20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="D570" t="n">
+        <v>406</v>
+      </c>
+      <c r="E570" t="n">
+        <v>415.77</v>
+      </c>
+      <c r="F570" t="n">
+        <v>415.77</v>
+      </c>
+      <c r="G570" t="n">
+        <v>407.91</v>
+      </c>
+      <c r="H570" t="n">
+        <v>407.75</v>
+      </c>
+      <c r="I570" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J570" t="b">
+        <v>0</v>
+      </c>
+      <c r="K570" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 406.00 &lt;= Upper 415.77)</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>BPCL</t>
+        </is>
+      </c>
+      <c r="D571" t="n">
+        <v>303.55</v>
+      </c>
+      <c r="E571" t="n">
+        <v>325.88</v>
+      </c>
+      <c r="F571" t="n">
+        <v>325.88</v>
+      </c>
+      <c r="G571" t="n">
+        <v>312.16</v>
+      </c>
+      <c r="H571" t="n">
+        <v>314.43</v>
+      </c>
+      <c r="I571" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J571" t="b">
+        <v>0</v>
+      </c>
+      <c r="K571" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 312.16 &lt;= EMA21 314.43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="D572" t="n">
+        <v>1814.7</v>
+      </c>
+      <c r="E572" t="n">
+        <v>2001.99</v>
+      </c>
+      <c r="F572" t="n">
+        <v>2001.99</v>
+      </c>
+      <c r="G572" t="n">
+        <v>1854.73</v>
+      </c>
+      <c r="H572" t="n">
+        <v>1883.02</v>
+      </c>
+      <c r="I572" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J572" t="b">
+        <v>0</v>
+      </c>
+      <c r="K572" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1854.73 &lt;= EMA21 1883.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>BOSCHLTD</t>
+        </is>
+      </c>
+      <c r="D573" t="n">
+        <v>49100</v>
+      </c>
+      <c r="E573" t="n">
+        <v>49986.46</v>
+      </c>
+      <c r="F573" t="n">
+        <v>49986.46</v>
+      </c>
+      <c r="G573" t="n">
+        <v>48237.27</v>
+      </c>
+      <c r="H573" t="n">
+        <v>47363.72</v>
+      </c>
+      <c r="I573" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J573" t="b">
+        <v>0</v>
+      </c>
+      <c r="K573" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 49100.00 &lt;= Upper 49986.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>BRITANNIA</t>
+        </is>
+      </c>
+      <c r="D574" t="n">
+        <v>5090</v>
+      </c>
+      <c r="E574" t="n">
+        <v>5669.96</v>
+      </c>
+      <c r="F574" t="n">
+        <v>5669.96</v>
+      </c>
+      <c r="G574" t="n">
+        <v>5147.99</v>
+      </c>
+      <c r="H574" t="n">
+        <v>5253.37</v>
+      </c>
+      <c r="I574" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J574" t="b">
+        <v>0</v>
+      </c>
+      <c r="K574" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5147.99 &lt;= EMA21 5253.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="D575" t="n">
+        <v>926.95</v>
+      </c>
+      <c r="E575" t="n">
+        <v>922.1799999999999</v>
+      </c>
+      <c r="F575" t="n">
+        <v>922.1799999999999</v>
+      </c>
+      <c r="G575" t="n">
+        <v>900.52</v>
+      </c>
+      <c r="H575" t="n">
+        <v>892.28</v>
+      </c>
+      <c r="I575" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="J575" t="b">
+        <v>1</v>
+      </c>
+      <c r="K575" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>CANBK</t>
+        </is>
+      </c>
+      <c r="D576" t="n">
+        <v>124.08</v>
+      </c>
+      <c r="E576" t="n">
+        <v>132.64</v>
+      </c>
+      <c r="F576" t="n">
+        <v>132.64</v>
+      </c>
+      <c r="G576" t="n">
+        <v>125.61</v>
+      </c>
+      <c r="H576" t="n">
+        <v>126.91</v>
+      </c>
+      <c r="I576" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J576" t="b">
+        <v>0</v>
+      </c>
+      <c r="K576" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 125.61 &lt;= EMA21 126.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="D577" t="n">
+        <v>1829</v>
+      </c>
+      <c r="E577" t="n">
+        <v>1924.32</v>
+      </c>
+      <c r="F577" t="n">
+        <v>1924.32</v>
+      </c>
+      <c r="G577" t="n">
+        <v>1840.61</v>
+      </c>
+      <c r="H577" t="n">
+        <v>1848.62</v>
+      </c>
+      <c r="I577" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J577" t="b">
+        <v>0</v>
+      </c>
+      <c r="K577" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1840.61 &lt;= EMA21 1848.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>CIPLA</t>
+        </is>
+      </c>
+      <c r="D578" t="n">
+        <v>1363.1</v>
+      </c>
+      <c r="E578" t="n">
+        <v>1470.9</v>
+      </c>
+      <c r="F578" t="n">
+        <v>1470.9</v>
+      </c>
+      <c r="G578" t="n">
+        <v>1396.27</v>
+      </c>
+      <c r="H578" t="n">
+        <v>1414.56</v>
+      </c>
+      <c r="I578" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="J578" t="b">
+        <v>0</v>
+      </c>
+      <c r="K578" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1396.27 &lt;= EMA21 1414.56)</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="D579" t="n">
+        <v>431</v>
+      </c>
+      <c r="E579" t="n">
+        <v>425.46</v>
+      </c>
+      <c r="F579" t="n">
+        <v>425.46</v>
+      </c>
+      <c r="G579" t="n">
+        <v>414.94</v>
+      </c>
+      <c r="H579" t="n">
+        <v>409.68</v>
+      </c>
+      <c r="I579" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="J579" t="b">
+        <v>1</v>
+      </c>
+      <c r="K579" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>CUMMINSIND</t>
+        </is>
+      </c>
+      <c r="D580" t="n">
+        <v>5170.5</v>
+      </c>
+      <c r="E580" t="n">
+        <v>5443.48</v>
+      </c>
+      <c r="F580" t="n">
+        <v>5443.48</v>
+      </c>
+      <c r="G580" t="n">
+        <v>5119.95</v>
+      </c>
+      <c r="H580" t="n">
+        <v>5202.33</v>
+      </c>
+      <c r="I580" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J580" t="b">
+        <v>0</v>
+      </c>
+      <c r="K580" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5119.95 &lt;= EMA21 5202.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>DLF</t>
+        </is>
+      </c>
+      <c r="D581" t="n">
+        <v>655.1</v>
+      </c>
+      <c r="E581" t="n">
+        <v>692.41</v>
+      </c>
+      <c r="F581" t="n">
+        <v>692.41</v>
+      </c>
+      <c r="G581" t="n">
+        <v>673.45</v>
+      </c>
+      <c r="H581" t="n">
+        <v>671.2</v>
+      </c>
+      <c r="I581" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="J581" t="b">
+        <v>0</v>
+      </c>
+      <c r="K581" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 655.10 &lt;= Upper 692.41)</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>DIVISLAB</t>
+        </is>
+      </c>
+      <c r="D582" t="n">
+        <v>9488</v>
+      </c>
+      <c r="E582" t="n">
+        <v>9721.76</v>
+      </c>
+      <c r="F582" t="n">
+        <v>9721.76</v>
+      </c>
+      <c r="G582" t="n">
+        <v>9274.889999999999</v>
+      </c>
+      <c r="H582" t="n">
+        <v>8944.84</v>
+      </c>
+      <c r="I582" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J582" t="b">
+        <v>0</v>
+      </c>
+      <c r="K582" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 9488.00 &lt;= Upper 9721.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="D583" t="n">
+        <v>1145</v>
+      </c>
+      <c r="E583" t="n">
+        <v>1209.86</v>
+      </c>
+      <c r="F583" t="n">
+        <v>1209.86</v>
+      </c>
+      <c r="G583" t="n">
+        <v>1156.01</v>
+      </c>
+      <c r="H583" t="n">
+        <v>1168.19</v>
+      </c>
+      <c r="I583" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J583" t="b">
+        <v>0</v>
+      </c>
+      <c r="K583" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1156.01 &lt;= EMA21 1168.19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>EICHERMOT</t>
+        </is>
+      </c>
+      <c r="D584" t="n">
+        <v>7734.5</v>
+      </c>
+      <c r="E584" t="n">
+        <v>8260.98</v>
+      </c>
+      <c r="F584" t="n">
+        <v>8260.98</v>
+      </c>
+      <c r="G584" t="n">
+        <v>7809.06</v>
+      </c>
+      <c r="H584" t="n">
+        <v>7866.69</v>
+      </c>
+      <c r="I584" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J584" t="b">
+        <v>0</v>
+      </c>
+      <c r="K584" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7809.06 &lt;= EMA21 7866.69)</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>ETERNAL</t>
+        </is>
+      </c>
+      <c r="D585" t="n">
+        <v>320.6</v>
+      </c>
+      <c r="E585" t="n">
+        <v>333.79</v>
+      </c>
+      <c r="F585" t="n">
+        <v>333.79</v>
+      </c>
+      <c r="G585" t="n">
+        <v>323.94</v>
+      </c>
+      <c r="H585" t="n">
+        <v>321.07</v>
+      </c>
+      <c r="I585" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J585" t="b">
+        <v>0</v>
+      </c>
+      <c r="K585" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 320.60 &lt;= Upper 333.79)</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>GAIL</t>
+        </is>
+      </c>
+      <c r="D586" t="n">
+        <v>174.9</v>
+      </c>
+      <c r="E586" t="n">
+        <v>176.99</v>
+      </c>
+      <c r="F586" t="n">
+        <v>176.99</v>
+      </c>
+      <c r="G586" t="n">
+        <v>174.35</v>
+      </c>
+      <c r="H586" t="n">
+        <v>173.92</v>
+      </c>
+      <c r="I586" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J586" t="b">
+        <v>0</v>
+      </c>
+      <c r="K586" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 174.90 &lt;= Upper 176.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>GODREJCP</t>
+        </is>
+      </c>
+      <c r="D587" t="n">
+        <v>863.8</v>
+      </c>
+      <c r="E587" t="n">
+        <v>965.1799999999999</v>
+      </c>
+      <c r="F587" t="n">
+        <v>965.1799999999999</v>
+      </c>
+      <c r="G587" t="n">
+        <v>884.4299999999999</v>
+      </c>
+      <c r="H587" t="n">
+        <v>918.5</v>
+      </c>
+      <c r="I587" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J587" t="b">
+        <v>0</v>
+      </c>
+      <c r="K587" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 884.43 &lt;= EMA21 918.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>GRASIM</t>
+        </is>
+      </c>
+      <c r="D588" t="n">
+        <v>3300</v>
+      </c>
+      <c r="E588" t="n">
+        <v>3349.38</v>
+      </c>
+      <c r="F588" t="n">
+        <v>3349.38</v>
+      </c>
+      <c r="G588" t="n">
+        <v>3304.77</v>
+      </c>
+      <c r="H588" t="n">
+        <v>3283.87</v>
+      </c>
+      <c r="I588" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J588" t="b">
+        <v>0</v>
+      </c>
+      <c r="K588" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3300.00 &lt;= Upper 3349.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="D589" t="n">
+        <v>1229.8</v>
+      </c>
+      <c r="E589" t="n">
+        <v>1374.25</v>
+      </c>
+      <c r="F589" t="n">
+        <v>1374.25</v>
+      </c>
+      <c r="G589" t="n">
+        <v>1288.28</v>
+      </c>
+      <c r="H589" t="n">
+        <v>1301.21</v>
+      </c>
+      <c r="I589" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J589" t="b">
+        <v>0</v>
+      </c>
+      <c r="K589" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1288.28 &lt;= EMA21 1301.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>HDFCAMC</t>
+        </is>
+      </c>
+      <c r="D590" t="n">
+        <v>2440</v>
+      </c>
+      <c r="E590" t="n">
+        <v>2694.8</v>
+      </c>
+      <c r="F590" t="n">
+        <v>2694.8</v>
+      </c>
+      <c r="G590" t="n">
+        <v>2507.11</v>
+      </c>
+      <c r="H590" t="n">
+        <v>2541.72</v>
+      </c>
+      <c r="I590" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J590" t="b">
+        <v>0</v>
+      </c>
+      <c r="K590" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2507.11 &lt;= EMA21 2541.72)</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="D591" t="n">
+        <v>687.1</v>
+      </c>
+      <c r="E591" t="n">
+        <v>739.7</v>
+      </c>
+      <c r="F591" t="n">
+        <v>739.7</v>
+      </c>
+      <c r="G591" t="n">
+        <v>706.02</v>
+      </c>
+      <c r="H591" t="n">
+        <v>717.23</v>
+      </c>
+      <c r="I591" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="J591" t="b">
+        <v>0</v>
+      </c>
+      <c r="K591" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 706.02 &lt;= EMA21 717.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="D592" t="n">
+        <v>514</v>
+      </c>
+      <c r="E592" t="n">
+        <v>559.49</v>
+      </c>
+      <c r="F592" t="n">
+        <v>559.49</v>
+      </c>
+      <c r="G592" t="n">
+        <v>533.97</v>
+      </c>
+      <c r="H592" t="n">
+        <v>539.83</v>
+      </c>
+      <c r="I592" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="J592" t="b">
+        <v>0</v>
+      </c>
+      <c r="K592" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 533.97 &lt;= EMA21 539.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="D593" t="n">
+        <v>1026.9</v>
+      </c>
+      <c r="E593" t="n">
+        <v>1071.72</v>
+      </c>
+      <c r="F593" t="n">
+        <v>1071.72</v>
+      </c>
+      <c r="G593" t="n">
+        <v>1020.22</v>
+      </c>
+      <c r="H593" t="n">
+        <v>1022.3</v>
+      </c>
+      <c r="I593" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J593" t="b">
+        <v>0</v>
+      </c>
+      <c r="K593" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1020.22 &lt;= EMA21 1022.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="D594" t="n">
+        <v>5000.5</v>
+      </c>
+      <c r="E594" t="n">
+        <v>5128.95</v>
+      </c>
+      <c r="F594" t="n">
+        <v>5128.95</v>
+      </c>
+      <c r="G594" t="n">
+        <v>4903.55</v>
+      </c>
+      <c r="H594" t="n">
+        <v>4871.34</v>
+      </c>
+      <c r="I594" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="J594" t="b">
+        <v>0</v>
+      </c>
+      <c r="K594" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 5000.50 &lt;= Upper 5128.95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="D595" t="n">
+        <v>1945</v>
+      </c>
+      <c r="E595" t="n">
+        <v>2092.83</v>
+      </c>
+      <c r="F595" t="n">
+        <v>2092.83</v>
+      </c>
+      <c r="G595" t="n">
+        <v>1979.92</v>
+      </c>
+      <c r="H595" t="n">
+        <v>2012.57</v>
+      </c>
+      <c r="I595" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="J595" t="b">
+        <v>0</v>
+      </c>
+      <c r="K595" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1979.92 &lt;= EMA21 2012.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+      <c r="D596" t="n">
+        <v>605.4</v>
+      </c>
+      <c r="E596" t="n">
+        <v>629.4299999999999</v>
+      </c>
+      <c r="F596" t="n">
+        <v>629.4299999999999</v>
+      </c>
+      <c r="G596" t="n">
+        <v>597.0599999999999</v>
+      </c>
+      <c r="H596" t="n">
+        <v>590</v>
+      </c>
+      <c r="I596" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J596" t="b">
+        <v>0</v>
+      </c>
+      <c r="K596" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 605.40 &lt;= Upper 629.43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>HYUNDAI</t>
+        </is>
+      </c>
+      <c r="D597" t="n">
+        <v>2182.4</v>
+      </c>
+      <c r="E597" t="n">
+        <v>2270.48</v>
+      </c>
+      <c r="F597" t="n">
+        <v>2270.48</v>
+      </c>
+      <c r="G597" t="n">
+        <v>2199.12</v>
+      </c>
+      <c r="H597" t="n">
+        <v>2188.65</v>
+      </c>
+      <c r="I597" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J597" t="b">
+        <v>0</v>
+      </c>
+      <c r="K597" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 2182.40 &lt;= Upper 2270.48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="D598" t="n">
+        <v>1389.1</v>
+      </c>
+      <c r="E598" t="n">
+        <v>1450.72</v>
+      </c>
+      <c r="F598" t="n">
+        <v>1450.72</v>
+      </c>
+      <c r="G598" t="n">
+        <v>1416.19</v>
+      </c>
+      <c r="H598" t="n">
+        <v>1420.73</v>
+      </c>
+      <c r="I598" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="J598" t="b">
+        <v>0</v>
+      </c>
+      <c r="K598" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1416.19 &lt;= EMA21 1420.73)</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="D599" t="n">
+        <v>260.8</v>
+      </c>
+      <c r="E599" t="n">
+        <v>278.9</v>
+      </c>
+      <c r="F599" t="n">
+        <v>278.9</v>
+      </c>
+      <c r="G599" t="n">
+        <v>264.14</v>
+      </c>
+      <c r="H599" t="n">
+        <v>268.35</v>
+      </c>
+      <c r="I599" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J599" t="b">
+        <v>0</v>
+      </c>
+      <c r="K599" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 264.14 &lt;= EMA21 268.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>INDHOTEL</t>
+        </is>
+      </c>
+      <c r="D600" t="n">
+        <v>722.75</v>
+      </c>
+      <c r="E600" t="n">
+        <v>738.29</v>
+      </c>
+      <c r="F600" t="n">
+        <v>738.29</v>
+      </c>
+      <c r="G600" t="n">
+        <v>722.4299999999999</v>
+      </c>
+      <c r="H600" t="n">
+        <v>724.36</v>
+      </c>
+      <c r="I600" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="J600" t="b">
+        <v>0</v>
+      </c>
+      <c r="K600" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 722.43 &lt;= EMA21 724.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>IOC</t>
+        </is>
+      </c>
+      <c r="D601" t="n">
+        <v>135.6</v>
+      </c>
+      <c r="E601" t="n">
+        <v>140.67</v>
+      </c>
+      <c r="F601" t="n">
+        <v>140.67</v>
+      </c>
+      <c r="G601" t="n">
+        <v>136.42</v>
+      </c>
+      <c r="H601" t="n">
+        <v>137.43</v>
+      </c>
+      <c r="I601" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J601" t="b">
+        <v>0</v>
+      </c>
+      <c r="K601" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 136.42 &lt;= EMA21 137.43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>IRFC</t>
+        </is>
+      </c>
+      <c r="D602" t="n">
+        <v>81.39</v>
+      </c>
+      <c r="E602" t="n">
+        <v>89.20999999999999</v>
+      </c>
+      <c r="F602" t="n">
+        <v>89.20999999999999</v>
+      </c>
+      <c r="G602" t="n">
+        <v>83.01000000000001</v>
+      </c>
+      <c r="H602" t="n">
+        <v>84.68000000000001</v>
+      </c>
+      <c r="I602" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J602" t="b">
+        <v>0</v>
+      </c>
+      <c r="K602" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 83.01 &lt;= EMA21 84.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="D603" t="n">
+        <v>1035</v>
+      </c>
+      <c r="E603" t="n">
+        <v>1188.04</v>
+      </c>
+      <c r="F603" t="n">
+        <v>1188.04</v>
+      </c>
+      <c r="G603" t="n">
+        <v>1100.54</v>
+      </c>
+      <c r="H603" t="n">
+        <v>1118.07</v>
+      </c>
+      <c r="I603" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J603" t="b">
+        <v>0</v>
+      </c>
+      <c r="K603" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1100.54 &lt;= EMA21 1118.07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>INDIGO</t>
+        </is>
+      </c>
+      <c r="D604" t="n">
+        <v>4975</v>
+      </c>
+      <c r="E604" t="n">
+        <v>5406.39</v>
+      </c>
+      <c r="F604" t="n">
+        <v>5406.39</v>
+      </c>
+      <c r="G604" t="n">
+        <v>5049.33</v>
+      </c>
+      <c r="H604" t="n">
+        <v>5125.11</v>
+      </c>
+      <c r="I604" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J604" t="b">
+        <v>0</v>
+      </c>
+      <c r="K604" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5049.33 &lt;= EMA21 5125.11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>JSWSTEEL</t>
+        </is>
+      </c>
+      <c r="D605" t="n">
+        <v>1310</v>
+      </c>
+      <c r="E605" t="n">
+        <v>1349.32</v>
+      </c>
+      <c r="F605" t="n">
+        <v>1349.32</v>
+      </c>
+      <c r="G605" t="n">
+        <v>1309.45</v>
+      </c>
+      <c r="H605" t="n">
+        <v>1304.15</v>
+      </c>
+      <c r="I605" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J605" t="b">
+        <v>0</v>
+      </c>
+      <c r="K605" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1310.00 &lt;= Upper 1349.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>JINDALSTEL</t>
+        </is>
+      </c>
+      <c r="D606" t="n">
+        <v>1146.5</v>
+      </c>
+      <c r="E606" t="n">
+        <v>1200.23</v>
+      </c>
+      <c r="F606" t="n">
+        <v>1200.23</v>
+      </c>
+      <c r="G606" t="n">
+        <v>1152.12</v>
+      </c>
+      <c r="H606" t="n">
+        <v>1139.47</v>
+      </c>
+      <c r="I606" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J606" t="b">
+        <v>0</v>
+      </c>
+      <c r="K606" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1146.50 &lt;= Upper 1200.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>JIOFIN</t>
+        </is>
+      </c>
+      <c r="D607" t="n">
+        <v>231</v>
+      </c>
+      <c r="E607" t="n">
+        <v>255.57</v>
+      </c>
+      <c r="F607" t="n">
+        <v>255.57</v>
+      </c>
+      <c r="G607" t="n">
+        <v>236.86</v>
+      </c>
+      <c r="H607" t="n">
+        <v>240.74</v>
+      </c>
+      <c r="I607" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J607" t="b">
+        <v>0</v>
+      </c>
+      <c r="K607" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 236.86 &lt;= EMA21 240.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="D608" t="n">
+        <v>414</v>
+      </c>
+      <c r="E608" t="n">
+        <v>437.52</v>
+      </c>
+      <c r="F608" t="n">
+        <v>437.52</v>
+      </c>
+      <c r="G608" t="n">
+        <v>418.16</v>
+      </c>
+      <c r="H608" t="n">
+        <v>411.39</v>
+      </c>
+      <c r="I608" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J608" t="b">
+        <v>0</v>
+      </c>
+      <c r="K608" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 414.00 &lt;= Upper 437.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>LTM</t>
+        </is>
+      </c>
+      <c r="D609" t="n">
+        <v>4412</v>
+      </c>
+      <c r="E609" t="n">
+        <v>4753.75</v>
+      </c>
+      <c r="F609" t="n">
+        <v>4753.75</v>
+      </c>
+      <c r="G609" t="n">
+        <v>4498.99</v>
+      </c>
+      <c r="H609" t="n">
+        <v>4511.85</v>
+      </c>
+      <c r="I609" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="J609" t="b">
+        <v>0</v>
+      </c>
+      <c r="K609" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4498.99 &lt;= EMA21 4511.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="D610" t="n">
+        <v>3922.6</v>
+      </c>
+      <c r="E610" t="n">
+        <v>4141.17</v>
+      </c>
+      <c r="F610" t="n">
+        <v>4141.17</v>
+      </c>
+      <c r="G610" t="n">
+        <v>3979.36</v>
+      </c>
+      <c r="H610" t="n">
+        <v>4001.7</v>
+      </c>
+      <c r="I610" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="J610" t="b">
+        <v>0</v>
+      </c>
+      <c r="K610" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3979.36 &lt;= EMA21 4001.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>LODHA</t>
+        </is>
+      </c>
+      <c r="D611" t="n">
+        <v>1166</v>
+      </c>
+      <c r="E611" t="n">
+        <v>1288.71</v>
+      </c>
+      <c r="F611" t="n">
+        <v>1288.71</v>
+      </c>
+      <c r="G611" t="n">
+        <v>1212.85</v>
+      </c>
+      <c r="H611" t="n">
+        <v>1219.01</v>
+      </c>
+      <c r="I611" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="J611" t="b">
+        <v>0</v>
+      </c>
+      <c r="K611" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1212.85 &lt;= EMA21 1219.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>M&amp;M</t>
+        </is>
+      </c>
+      <c r="D612" t="n">
+        <v>3150</v>
+      </c>
+      <c r="E612" t="n">
+        <v>3547.95</v>
+      </c>
+      <c r="F612" t="n">
+        <v>3547.95</v>
+      </c>
+      <c r="G612" t="n">
+        <v>3208.48</v>
+      </c>
+      <c r="H612" t="n">
+        <v>3272.13</v>
+      </c>
+      <c r="I612" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J612" t="b">
+        <v>0</v>
+      </c>
+      <c r="K612" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3208.48 &lt;= EMA21 3272.13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="D613" t="n">
+        <v>12618</v>
+      </c>
+      <c r="E613" t="n">
+        <v>14249.24</v>
+      </c>
+      <c r="F613" t="n">
+        <v>14249.24</v>
+      </c>
+      <c r="G613" t="n">
+        <v>12900.63</v>
+      </c>
+      <c r="H613" t="n">
+        <v>13221.4</v>
+      </c>
+      <c r="I613" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="J613" t="b">
+        <v>0</v>
+      </c>
+      <c r="K613" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 12900.63 &lt;= EMA21 13221.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>MAXHEALTH</t>
+        </is>
+      </c>
+      <c r="D614" t="n">
+        <v>1037.5</v>
+      </c>
+      <c r="E614" t="n">
+        <v>1035.06</v>
+      </c>
+      <c r="F614" t="n">
+        <v>1035.06</v>
+      </c>
+      <c r="G614" t="n">
+        <v>1008.07</v>
+      </c>
+      <c r="H614" t="n">
+        <v>1018.16</v>
+      </c>
+      <c r="I614" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="J614" t="b">
+        <v>0</v>
+      </c>
+      <c r="K614" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1008.07 &lt;= EMA21 1018.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>MAZDOCK</t>
+        </is>
+      </c>
+      <c r="D615" t="n">
+        <v>2408.8</v>
+      </c>
+      <c r="E615" t="n">
+        <v>2650.46</v>
+      </c>
+      <c r="F615" t="n">
+        <v>2650.46</v>
+      </c>
+      <c r="G615" t="n">
+        <v>2480.07</v>
+      </c>
+      <c r="H615" t="n">
+        <v>2496.62</v>
+      </c>
+      <c r="I615" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J615" t="b">
+        <v>0</v>
+      </c>
+      <c r="K615" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2480.07 &lt;= EMA21 2496.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>MUTHOOTFIN</t>
+        </is>
+      </c>
+      <c r="D616" t="n">
+        <v>2815</v>
+      </c>
+      <c r="E616" t="n">
+        <v>3219.05</v>
+      </c>
+      <c r="F616" t="n">
+        <v>3219.05</v>
+      </c>
+      <c r="G616" t="n">
+        <v>2918.88</v>
+      </c>
+      <c r="H616" t="n">
+        <v>2955.63</v>
+      </c>
+      <c r="I616" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="J616" t="b">
+        <v>0</v>
+      </c>
+      <c r="K616" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2918.88 &lt;= EMA21 2955.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="D617" t="n">
+        <v>334.5</v>
+      </c>
+      <c r="E617" t="n">
+        <v>340.69</v>
+      </c>
+      <c r="F617" t="n">
+        <v>340.69</v>
+      </c>
+      <c r="G617" t="n">
+        <v>331.38</v>
+      </c>
+      <c r="H617" t="n">
+        <v>332.92</v>
+      </c>
+      <c r="I617" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="J617" t="b">
+        <v>0</v>
+      </c>
+      <c r="K617" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 331.38 &lt;= EMA21 332.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="D618" t="n">
+        <v>1393</v>
+      </c>
+      <c r="E618" t="n">
+        <v>1520.06</v>
+      </c>
+      <c r="F618" t="n">
+        <v>1520.06</v>
+      </c>
+      <c r="G618" t="n">
+        <v>1419.55</v>
+      </c>
+      <c r="H618" t="n">
+        <v>1443.7</v>
+      </c>
+      <c r="I618" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J618" t="b">
+        <v>0</v>
+      </c>
+      <c r="K618" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1419.55 &lt;= EMA21 1443.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="D619" t="n">
+        <v>234.02</v>
+      </c>
+      <c r="E619" t="n">
+        <v>239.85</v>
+      </c>
+      <c r="F619" t="n">
+        <v>239.85</v>
+      </c>
+      <c r="G619" t="n">
+        <v>234.5</v>
+      </c>
+      <c r="H619" t="n">
+        <v>235.5</v>
+      </c>
+      <c r="I619" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J619" t="b">
+        <v>0</v>
+      </c>
+      <c r="K619" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 234.50 &lt;= EMA21 235.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>PIDILITIND</t>
+        </is>
+      </c>
+      <c r="D620" t="n">
+        <v>1572</v>
+      </c>
+      <c r="E620" t="n">
+        <v>1714.27</v>
+      </c>
+      <c r="F620" t="n">
+        <v>1714.27</v>
+      </c>
+      <c r="G620" t="n">
+        <v>1613.41</v>
+      </c>
+      <c r="H620" t="n">
+        <v>1630.62</v>
+      </c>
+      <c r="I620" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="J620" t="b">
+        <v>0</v>
+      </c>
+      <c r="K620" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1613.41 &lt;= EMA21 1630.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>PFC</t>
+        </is>
+      </c>
+      <c r="D621" t="n">
+        <v>351.4</v>
+      </c>
+      <c r="E621" t="n">
+        <v>378.49</v>
+      </c>
+      <c r="F621" t="n">
+        <v>378.49</v>
+      </c>
+      <c r="G621" t="n">
+        <v>352.82</v>
+      </c>
+      <c r="H621" t="n">
+        <v>361.59</v>
+      </c>
+      <c r="I621" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J621" t="b">
+        <v>0</v>
+      </c>
+      <c r="K621" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 352.82 &lt;= EMA21 361.59)</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="D622" t="n">
+        <v>265.85</v>
+      </c>
+      <c r="E622" t="n">
+        <v>271.72</v>
+      </c>
+      <c r="F622" t="n">
+        <v>271.72</v>
+      </c>
+      <c r="G622" t="n">
+        <v>266.07</v>
+      </c>
+      <c r="H622" t="n">
+        <v>268.42</v>
+      </c>
+      <c r="I622" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J622" t="b">
+        <v>0</v>
+      </c>
+      <c r="K622" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 266.07 &lt;= EMA21 268.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="D623" t="n">
+        <v>115.61</v>
+      </c>
+      <c r="E623" t="n">
+        <v>118.41</v>
+      </c>
+      <c r="F623" t="n">
+        <v>118.41</v>
+      </c>
+      <c r="G623" t="n">
+        <v>115.96</v>
+      </c>
+      <c r="H623" t="n">
+        <v>115.54</v>
+      </c>
+      <c r="I623" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J623" t="b">
+        <v>0</v>
+      </c>
+      <c r="K623" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 115.61 &lt;= Upper 118.41)</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="D624" t="n">
+        <v>314.5</v>
+      </c>
+      <c r="E624" t="n">
+        <v>344.21</v>
+      </c>
+      <c r="F624" t="n">
+        <v>344.21</v>
+      </c>
+      <c r="G624" t="n">
+        <v>318.18</v>
+      </c>
+      <c r="H624" t="n">
+        <v>326.04</v>
+      </c>
+      <c r="I624" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="J624" t="b">
+        <v>0</v>
+      </c>
+      <c r="K624" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 318.18 &lt;= EMA21 326.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="D625" t="n">
+        <v>1279</v>
+      </c>
+      <c r="E625" t="n">
+        <v>1333.67</v>
+      </c>
+      <c r="F625" t="n">
+        <v>1333.67</v>
+      </c>
+      <c r="G625" t="n">
+        <v>1299.33</v>
+      </c>
+      <c r="H625" t="n">
+        <v>1302.89</v>
+      </c>
+      <c r="I625" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="J625" t="b">
+        <v>0</v>
+      </c>
+      <c r="K625" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1299.33 &lt;= EMA21 1302.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="D626" t="n">
+        <v>1684</v>
+      </c>
+      <c r="E626" t="n">
+        <v>1826.54</v>
+      </c>
+      <c r="F626" t="n">
+        <v>1826.54</v>
+      </c>
+      <c r="G626" t="n">
+        <v>1727.22</v>
+      </c>
+      <c r="H626" t="n">
+        <v>1758.46</v>
+      </c>
+      <c r="I626" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J626" t="b">
+        <v>0</v>
+      </c>
+      <c r="K626" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1727.22 &lt;= EMA21 1758.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>MOTHERSON</t>
+        </is>
+      </c>
+      <c r="D627" t="n">
+        <v>163.7</v>
+      </c>
+      <c r="E627" t="n">
+        <v>172.53</v>
+      </c>
+      <c r="F627" t="n">
+        <v>172.53</v>
+      </c>
+      <c r="G627" t="n">
+        <v>163.92</v>
+      </c>
+      <c r="H627" t="n">
+        <v>163.58</v>
+      </c>
+      <c r="I627" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J627" t="b">
+        <v>0</v>
+      </c>
+      <c r="K627" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 163.70 &lt;= Upper 172.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="D628" t="n">
+        <v>22950</v>
+      </c>
+      <c r="E628" t="n">
+        <v>25343.31</v>
+      </c>
+      <c r="F628" t="n">
+        <v>25343.31</v>
+      </c>
+      <c r="G628" t="n">
+        <v>23555.58</v>
+      </c>
+      <c r="H628" t="n">
+        <v>24171.66</v>
+      </c>
+      <c r="I628" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J628" t="b">
+        <v>0</v>
+      </c>
+      <c r="K628" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 23555.58 &lt;= EMA21 24171.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>SHRIRAMFIN</t>
+        </is>
+      </c>
+      <c r="D629" t="n">
+        <v>1029</v>
+      </c>
+      <c r="E629" t="n">
+        <v>1169.23</v>
+      </c>
+      <c r="F629" t="n">
+        <v>1169.23</v>
+      </c>
+      <c r="G629" t="n">
+        <v>1052.48</v>
+      </c>
+      <c r="H629" t="n">
+        <v>1072.55</v>
+      </c>
+      <c r="I629" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J629" t="b">
+        <v>0</v>
+      </c>
+      <c r="K629" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1052.48 &lt;= EMA21 1072.55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>ENRIN</t>
+        </is>
+      </c>
+      <c r="D630" t="n">
+        <v>3183.7</v>
+      </c>
+      <c r="E630" t="n">
+        <v>3677.32</v>
+      </c>
+      <c r="F630" t="n">
+        <v>3677.32</v>
+      </c>
+      <c r="G630" t="n">
+        <v>3197.62</v>
+      </c>
+      <c r="H630" t="n">
+        <v>3276.43</v>
+      </c>
+      <c r="I630" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J630" t="b">
+        <v>0</v>
+      </c>
+      <c r="K630" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3197.62 &lt;= EMA21 3276.43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+      <c r="D631" t="n">
+        <v>3949.1</v>
+      </c>
+      <c r="E631" t="n">
+        <v>4133.39</v>
+      </c>
+      <c r="F631" t="n">
+        <v>4133.39</v>
+      </c>
+      <c r="G631" t="n">
+        <v>3982.16</v>
+      </c>
+      <c r="H631" t="n">
+        <v>3967.14</v>
+      </c>
+      <c r="I631" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J631" t="b">
+        <v>0</v>
+      </c>
+      <c r="K631" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3949.10 &lt;= Upper 4133.39)</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>SOLARINDS</t>
+        </is>
+      </c>
+      <c r="D632" t="n">
+        <v>22355</v>
+      </c>
+      <c r="E632" t="n">
+        <v>22318.57</v>
+      </c>
+      <c r="F632" t="n">
+        <v>22318.57</v>
+      </c>
+      <c r="G632" t="n">
+        <v>21439.31</v>
+      </c>
+      <c r="H632" t="n">
+        <v>20605.45</v>
+      </c>
+      <c r="I632" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="J632" t="b">
+        <v>0</v>
+      </c>
+      <c r="K632" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 0.48x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="D633" t="n">
+        <v>1000.5</v>
+      </c>
+      <c r="E633" t="n">
+        <v>1084.25</v>
+      </c>
+      <c r="F633" t="n">
+        <v>1084.25</v>
+      </c>
+      <c r="G633" t="n">
+        <v>1019.73</v>
+      </c>
+      <c r="H633" t="n">
+        <v>1032.97</v>
+      </c>
+      <c r="I633" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J633" t="b">
+        <v>0</v>
+      </c>
+      <c r="K633" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1019.73 &lt;= EMA21 1032.97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="D634" t="n">
+        <v>1864.9</v>
+      </c>
+      <c r="E634" t="n">
+        <v>1961.88</v>
+      </c>
+      <c r="F634" t="n">
+        <v>1961.88</v>
+      </c>
+      <c r="G634" t="n">
+        <v>1900.61</v>
+      </c>
+      <c r="H634" t="n">
+        <v>1912.93</v>
+      </c>
+      <c r="I634" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J634" t="b">
+        <v>0</v>
+      </c>
+      <c r="K634" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1900.61 &lt;= EMA21 1912.93)</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>TVSMOTOR</t>
+        </is>
+      </c>
+      <c r="D635" t="n">
+        <v>4151.1</v>
+      </c>
+      <c r="E635" t="n">
+        <v>4517.99</v>
+      </c>
+      <c r="F635" t="n">
+        <v>4517.99</v>
+      </c>
+      <c r="G635" t="n">
+        <v>4199.94</v>
+      </c>
+      <c r="H635" t="n">
+        <v>4235.42</v>
+      </c>
+      <c r="I635" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J635" t="b">
+        <v>0</v>
+      </c>
+      <c r="K635" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4199.94 &lt;= EMA21 4235.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>TATACAP</t>
+        </is>
+      </c>
+      <c r="D636" t="n">
+        <v>363</v>
+      </c>
+      <c r="E636" t="n">
+        <v>376.55</v>
+      </c>
+      <c r="F636" t="n">
+        <v>376.55</v>
+      </c>
+      <c r="G636" t="n">
+        <v>368.31</v>
+      </c>
+      <c r="H636" t="n">
+        <v>367.2</v>
+      </c>
+      <c r="I636" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="J636" t="b">
+        <v>0</v>
+      </c>
+      <c r="K636" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 363.00 &lt;= Upper 376.55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="D637" t="n">
+        <v>2208</v>
+      </c>
+      <c r="E637" t="n">
+        <v>2402.28</v>
+      </c>
+      <c r="F637" t="n">
+        <v>2402.28</v>
+      </c>
+      <c r="G637" t="n">
+        <v>2284.18</v>
+      </c>
+      <c r="H637" t="n">
+        <v>2304.42</v>
+      </c>
+      <c r="I637" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J637" t="b">
+        <v>0</v>
+      </c>
+      <c r="K637" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2284.18 &lt;= EMA21 2304.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>TATACONSUM</t>
+        </is>
+      </c>
+      <c r="D638" t="n">
+        <v>1001</v>
+      </c>
+      <c r="E638" t="n">
+        <v>1094.86</v>
+      </c>
+      <c r="F638" t="n">
+        <v>1094.86</v>
+      </c>
+      <c r="G638" t="n">
+        <v>1020.06</v>
+      </c>
+      <c r="H638" t="n">
+        <v>1039.98</v>
+      </c>
+      <c r="I638" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J638" t="b">
+        <v>0</v>
+      </c>
+      <c r="K638" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1020.06 &lt;= EMA21 1039.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>TMCV</t>
+        </is>
+      </c>
+      <c r="D639" t="n">
+        <v>444.95</v>
+      </c>
+      <c r="E639" t="n">
+        <v>488.47</v>
+      </c>
+      <c r="F639" t="n">
+        <v>488.47</v>
+      </c>
+      <c r="G639" t="n">
+        <v>458.04</v>
+      </c>
+      <c r="H639" t="n">
+        <v>459.07</v>
+      </c>
+      <c r="I639" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J639" t="b">
+        <v>0</v>
+      </c>
+      <c r="K639" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 458.04 &lt;= EMA21 459.07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>TMPV</t>
+        </is>
+      </c>
+      <c r="D640" t="n">
+        <v>303</v>
+      </c>
+      <c r="E640" t="n">
+        <v>338.97</v>
+      </c>
+      <c r="F640" t="n">
+        <v>338.97</v>
+      </c>
+      <c r="G640" t="n">
+        <v>309.79</v>
+      </c>
+      <c r="H640" t="n">
+        <v>317.22</v>
+      </c>
+      <c r="I640" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J640" t="b">
+        <v>0</v>
+      </c>
+      <c r="K640" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 309.79 &lt;= EMA21 317.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>TATAPOWER</t>
+        </is>
+      </c>
+      <c r="D641" t="n">
+        <v>370</v>
+      </c>
+      <c r="E641" t="n">
+        <v>390.36</v>
+      </c>
+      <c r="F641" t="n">
+        <v>390.36</v>
+      </c>
+      <c r="G641" t="n">
+        <v>365.1</v>
+      </c>
+      <c r="H641" t="n">
+        <v>367.7</v>
+      </c>
+      <c r="I641" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J641" t="b">
+        <v>0</v>
+      </c>
+      <c r="K641" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 365.10 &lt;= EMA21 367.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="D642" t="n">
+        <v>188.75</v>
+      </c>
+      <c r="E642" t="n">
+        <v>188.98</v>
+      </c>
+      <c r="F642" t="n">
+        <v>188.98</v>
+      </c>
+      <c r="G642" t="n">
+        <v>186.08</v>
+      </c>
+      <c r="H642" t="n">
+        <v>186.12</v>
+      </c>
+      <c r="I642" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="J642" t="b">
+        <v>0</v>
+      </c>
+      <c r="K642" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 186.08 &lt;= EMA21 186.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>TECHM</t>
+        </is>
+      </c>
+      <c r="D643" t="n">
+        <v>1508</v>
+      </c>
+      <c r="E643" t="n">
+        <v>1661.95</v>
+      </c>
+      <c r="F643" t="n">
+        <v>1661.95</v>
+      </c>
+      <c r="G643" t="n">
+        <v>1575.04</v>
+      </c>
+      <c r="H643" t="n">
+        <v>1589.32</v>
+      </c>
+      <c r="I643" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="J643" t="b">
+        <v>0</v>
+      </c>
+      <c r="K643" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1575.04 &lt;= EMA21 1589.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>TITAN</t>
+        </is>
+      </c>
+      <c r="D644" t="n">
+        <v>5005</v>
+      </c>
+      <c r="E644" t="n">
+        <v>5160.52</v>
+      </c>
+      <c r="F644" t="n">
+        <v>5160.52</v>
+      </c>
+      <c r="G644" t="n">
+        <v>5032.09</v>
+      </c>
+      <c r="H644" t="n">
+        <v>5024.04</v>
+      </c>
+      <c r="I644" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J644" t="b">
+        <v>0</v>
+      </c>
+      <c r="K644" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 5005.00 &lt;= Upper 5160.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>TORNTPHARM</t>
+        </is>
+      </c>
+      <c r="D645" t="n">
+        <v>4930</v>
+      </c>
+      <c r="E645" t="n">
+        <v>5072.82</v>
+      </c>
+      <c r="F645" t="n">
+        <v>5072.82</v>
+      </c>
+      <c r="G645" t="n">
+        <v>4941.33</v>
+      </c>
+      <c r="H645" t="n">
+        <v>4943.14</v>
+      </c>
+      <c r="I645" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="J645" t="b">
+        <v>0</v>
+      </c>
+      <c r="K645" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4941.33 &lt;= EMA21 4943.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="D646" t="n">
+        <v>2820</v>
+      </c>
+      <c r="E646" t="n">
+        <v>3013.61</v>
+      </c>
+      <c r="F646" t="n">
+        <v>3013.61</v>
+      </c>
+      <c r="G646" t="n">
+        <v>2841.69</v>
+      </c>
+      <c r="H646" t="n">
+        <v>2886.98</v>
+      </c>
+      <c r="I646" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J646" t="b">
+        <v>0</v>
+      </c>
+      <c r="K646" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2841.69 &lt;= EMA21 2886.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="D647" t="n">
+        <v>10900</v>
+      </c>
+      <c r="E647" t="n">
+        <v>11908.87</v>
+      </c>
+      <c r="F647" t="n">
+        <v>11908.87</v>
+      </c>
+      <c r="G647" t="n">
+        <v>11239.8</v>
+      </c>
+      <c r="H647" t="n">
+        <v>11424.32</v>
+      </c>
+      <c r="I647" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="J647" t="b">
+        <v>0</v>
+      </c>
+      <c r="K647" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11239.80 &lt;= EMA21 11424.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="D648" t="n">
+        <v>183.89</v>
+      </c>
+      <c r="E648" t="n">
+        <v>189.71</v>
+      </c>
+      <c r="F648" t="n">
+        <v>189.71</v>
+      </c>
+      <c r="G648" t="n">
+        <v>185.51</v>
+      </c>
+      <c r="H648" t="n">
+        <v>184.35</v>
+      </c>
+      <c r="I648" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J648" t="b">
+        <v>0</v>
+      </c>
+      <c r="K648" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 183.89 &lt;= Upper 189.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>UNITDSPR</t>
+        </is>
+      </c>
+      <c r="D649" t="n">
+        <v>1405.2</v>
+      </c>
+      <c r="E649" t="n">
+        <v>1591.45</v>
+      </c>
+      <c r="F649" t="n">
+        <v>1591.45</v>
+      </c>
+      <c r="G649" t="n">
+        <v>1461.24</v>
+      </c>
+      <c r="H649" t="n">
+        <v>1483.98</v>
+      </c>
+      <c r="I649" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J649" t="b">
+        <v>0</v>
+      </c>
+      <c r="K649" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1461.24 &lt;= EMA21 1483.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="D650" t="n">
+        <v>407</v>
+      </c>
+      <c r="E650" t="n">
+        <v>449.03</v>
+      </c>
+      <c r="F650" t="n">
+        <v>449.03</v>
+      </c>
+      <c r="G650" t="n">
+        <v>410.22</v>
+      </c>
+      <c r="H650" t="n">
+        <v>420.57</v>
+      </c>
+      <c r="I650" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="J650" t="b">
+        <v>0</v>
+      </c>
+      <c r="K650" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 410.22 &lt;= EMA21 420.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>VEDL</t>
+        </is>
+      </c>
+      <c r="D651" t="n">
+        <v>272.5</v>
+      </c>
+      <c r="E651" t="n">
+        <v>286.73</v>
+      </c>
+      <c r="F651" t="n">
+        <v>286.73</v>
+      </c>
+      <c r="G651" t="n">
+        <v>272.89</v>
+      </c>
+      <c r="H651" t="n">
+        <v>273.48</v>
+      </c>
+      <c r="I651" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J651" t="b">
+        <v>0</v>
+      </c>
+      <c r="K651" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 272.89 &lt;= EMA21 273.48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="D652" t="n">
+        <v>167</v>
+      </c>
+      <c r="E652" t="n">
+        <v>187.41</v>
+      </c>
+      <c r="F652" t="n">
+        <v>187.41</v>
+      </c>
+      <c r="G652" t="n">
+        <v>174.47</v>
+      </c>
+      <c r="H652" t="n">
+        <v>177.5</v>
+      </c>
+      <c r="I652" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="J652" t="b">
+        <v>0</v>
+      </c>
+      <c r="K652" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 174.47 &lt;= EMA21 177.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>ZYDUSLIFE</t>
+        </is>
+      </c>
+      <c r="D653" t="n">
+        <v>1127.4</v>
+      </c>
+      <c r="E653" t="n">
+        <v>1193.36</v>
+      </c>
+      <c r="F653" t="n">
+        <v>1193.36</v>
+      </c>
+      <c r="G653" t="n">
+        <v>1143.7</v>
+      </c>
+      <c r="H653" t="n">
+        <v>1142.19</v>
+      </c>
+      <c r="I653" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J653" t="b">
+        <v>0</v>
+      </c>
+      <c r="K653" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1127.40 &lt;= Upper 1193.36)</t>
         </is>
       </c>
     </row>
@@ -24220,7 +28520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24379,6 +28679,130 @@
         <v>1.32</v>
       </c>
       <c r="G5" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1775</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1695.12</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>214.9</v>
+      </c>
+      <c r="E7" t="n">
+        <v>205.23</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>926.95</v>
+      </c>
+      <c r="E8" t="n">
+        <v>885.24</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>431</v>
+      </c>
+      <c r="E9" t="n">
+        <v>411.6</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>QUEUED</t>
         </is>
@@ -24395,7 +28819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24476,21 +28900,144 @@
         <v>19685.95</v>
       </c>
       <c r="F2" t="n">
-        <v>418.85</v>
+        <v>431</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>2.9</v>
       </c>
       <c r="H2" t="n">
-        <v>400</v>
+        <v>415.76</v>
       </c>
       <c r="I2" t="n">
-        <v>418.85</v>
+        <v>435.3500061035156</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1775</v>
+      </c>
+      <c r="D3" t="n">
+        <v>11</v>
+      </c>
+      <c r="E3" t="n">
+        <v>19525</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1775</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1695.12</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1775</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>214.9</v>
+      </c>
+      <c r="D4" t="n">
+        <v>93</v>
+      </c>
+      <c r="E4" t="n">
+        <v>19985.7</v>
+      </c>
+      <c r="F4" t="n">
+        <v>214.9</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>205.23</v>
+      </c>
+      <c r="I4" t="n">
+        <v>214.9</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>926.95</v>
+      </c>
+      <c r="D5" t="n">
+        <v>21</v>
+      </c>
+      <c r="E5" t="n">
+        <v>19465.95</v>
+      </c>
+      <c r="F5" t="n">
+        <v>926.95</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>885.24</v>
+      </c>
+      <c r="I5" t="n">
+        <v>926.95</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -25404,7 +29951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K144"/>
+  <dimension ref="A1:K147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30492,6 +35039,153 @@
         </is>
       </c>
       <c r="K144" t="inlineStr">
+        <is>
+          <t>Entry Breakout</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-09-09 20:07:43</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>D21271DAB0</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F145" t="n">
+        <v>1775</v>
+      </c>
+      <c r="G145" t="n">
+        <v>1775</v>
+      </c>
+      <c r="H145" t="n">
+        <v>0</v>
+      </c>
+      <c r="I145" t="n">
+        <v>11</v>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>Entry Breakout</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-09-09 20:07:43</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>382E550052</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F146" t="n">
+        <v>214.9</v>
+      </c>
+      <c r="G146" t="n">
+        <v>214.9</v>
+      </c>
+      <c r="H146" t="n">
+        <v>0</v>
+      </c>
+      <c r="I146" t="n">
+        <v>93</v>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Entry Breakout</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-09-09 20:07:43</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>B855BA8DDE</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F147" t="n">
+        <v>926.95</v>
+      </c>
+      <c r="G147" t="n">
+        <v>926.95</v>
+      </c>
+      <c r="H147" t="n">
+        <v>0</v>
+      </c>
+      <c r="I147" t="n">
+        <v>21</v>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
         <is>
           <t>Entry Breakout</t>
         </is>
@@ -30576,7 +35270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30923,6 +35617,39 @@
         <v>1</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>20:07:45</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>120159.33</v>
+      </c>
+      <c r="D11" t="n">
+        <v>78662.60000000001</v>
+      </c>
+      <c r="E11" t="n">
+        <v>198821.93</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-1092.43</v>
+      </c>
+      <c r="G11" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H11" t="n">
+        <v>17</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-10T19:57 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_india.xlsx
+++ b/data/trade_log_india.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K653"/>
+  <dimension ref="A1:K753"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28506,6 +28506,4306 @@
       <c r="K653" t="inlineStr">
         <is>
           <t>BELOW_BAND (Close 1127.40 &lt;= Upper 1193.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+      <c r="D654" t="n">
+        <v>7329</v>
+      </c>
+      <c r="E654" t="n">
+        <v>7724.08</v>
+      </c>
+      <c r="F654" t="n">
+        <v>7724.08</v>
+      </c>
+      <c r="G654" t="n">
+        <v>7423.73</v>
+      </c>
+      <c r="H654" t="n">
+        <v>7455.85</v>
+      </c>
+      <c r="I654" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="J654" t="b">
+        <v>0</v>
+      </c>
+      <c r="K654" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7423.73 &lt;= EMA21 7455.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="D655" t="n">
+        <v>1391.9</v>
+      </c>
+      <c r="E655" t="n">
+        <v>1684.9</v>
+      </c>
+      <c r="F655" t="n">
+        <v>1684.9</v>
+      </c>
+      <c r="G655" t="n">
+        <v>1426.31</v>
+      </c>
+      <c r="H655" t="n">
+        <v>1484.55</v>
+      </c>
+      <c r="I655" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="J655" t="b">
+        <v>0</v>
+      </c>
+      <c r="K655" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1426.31 &lt;= EMA21 1484.55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>ADANIENT</t>
+        </is>
+      </c>
+      <c r="D656" t="n">
+        <v>3077.2</v>
+      </c>
+      <c r="E656" t="n">
+        <v>3194.04</v>
+      </c>
+      <c r="F656" t="n">
+        <v>3194.04</v>
+      </c>
+      <c r="G656" t="n">
+        <v>3005.08</v>
+      </c>
+      <c r="H656" t="n">
+        <v>3006.23</v>
+      </c>
+      <c r="I656" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J656" t="b">
+        <v>0</v>
+      </c>
+      <c r="K656" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3005.08 &lt;= EMA21 3006.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>ADANIGREEN</t>
+        </is>
+      </c>
+      <c r="D657" t="n">
+        <v>1299.1</v>
+      </c>
+      <c r="E657" t="n">
+        <v>1357.18</v>
+      </c>
+      <c r="F657" t="n">
+        <v>1357.18</v>
+      </c>
+      <c r="G657" t="n">
+        <v>1297.04</v>
+      </c>
+      <c r="H657" t="n">
+        <v>1312.48</v>
+      </c>
+      <c r="I657" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J657" t="b">
+        <v>0</v>
+      </c>
+      <c r="K657" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1297.04 &lt;= EMA21 1312.48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="D658" t="n">
+        <v>1768</v>
+      </c>
+      <c r="E658" t="n">
+        <v>1770.95</v>
+      </c>
+      <c r="F658" t="n">
+        <v>1770.95</v>
+      </c>
+      <c r="G658" t="n">
+        <v>1718.73</v>
+      </c>
+      <c r="H658" t="n">
+        <v>1707.42</v>
+      </c>
+      <c r="I658" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J658" t="b">
+        <v>0</v>
+      </c>
+      <c r="K658" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1768.00 &lt;= Upper 1770.95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="D659" t="n">
+        <v>213.5</v>
+      </c>
+      <c r="E659" t="n">
+        <v>215.53</v>
+      </c>
+      <c r="F659" t="n">
+        <v>215.53</v>
+      </c>
+      <c r="G659" t="n">
+        <v>209.44</v>
+      </c>
+      <c r="H659" t="n">
+        <v>208.64</v>
+      </c>
+      <c r="I659" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J659" t="b">
+        <v>0</v>
+      </c>
+      <c r="K659" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 213.50 &lt;= Upper 215.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>AMBUJACEM</t>
+        </is>
+      </c>
+      <c r="D660" t="n">
+        <v>395.6</v>
+      </c>
+      <c r="E660" t="n">
+        <v>421.67</v>
+      </c>
+      <c r="F660" t="n">
+        <v>421.67</v>
+      </c>
+      <c r="G660" t="n">
+        <v>401.19</v>
+      </c>
+      <c r="H660" t="n">
+        <v>408.11</v>
+      </c>
+      <c r="I660" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J660" t="b">
+        <v>0</v>
+      </c>
+      <c r="K660" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 401.19 &lt;= EMA21 408.11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="D661" t="n">
+        <v>8900</v>
+      </c>
+      <c r="E661" t="n">
+        <v>8985.389999999999</v>
+      </c>
+      <c r="F661" t="n">
+        <v>8985.389999999999</v>
+      </c>
+      <c r="G661" t="n">
+        <v>8822.76</v>
+      </c>
+      <c r="H661" t="n">
+        <v>8806.41</v>
+      </c>
+      <c r="I661" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="J661" t="b">
+        <v>0</v>
+      </c>
+      <c r="K661" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 8900.00 &lt;= Upper 8985.39)</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="D662" t="n">
+        <v>2498.1</v>
+      </c>
+      <c r="E662" t="n">
+        <v>2729.2</v>
+      </c>
+      <c r="F662" t="n">
+        <v>2729.2</v>
+      </c>
+      <c r="G662" t="n">
+        <v>2529.2</v>
+      </c>
+      <c r="H662" t="n">
+        <v>2585</v>
+      </c>
+      <c r="I662" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J662" t="b">
+        <v>0</v>
+      </c>
+      <c r="K662" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2529.20 &lt;= EMA21 2585.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="D663" t="n">
+        <v>3690</v>
+      </c>
+      <c r="E663" t="n">
+        <v>4070.6</v>
+      </c>
+      <c r="F663" t="n">
+        <v>4070.6</v>
+      </c>
+      <c r="G663" t="n">
+        <v>3761.37</v>
+      </c>
+      <c r="H663" t="n">
+        <v>3835.15</v>
+      </c>
+      <c r="I663" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="J663" t="b">
+        <v>0</v>
+      </c>
+      <c r="K663" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3761.37 &lt;= EMA21 3835.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="D664" t="n">
+        <v>1246</v>
+      </c>
+      <c r="E664" t="n">
+        <v>1286.59</v>
+      </c>
+      <c r="F664" t="n">
+        <v>1286.59</v>
+      </c>
+      <c r="G664" t="n">
+        <v>1252.97</v>
+      </c>
+      <c r="H664" t="n">
+        <v>1253.15</v>
+      </c>
+      <c r="I664" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J664" t="b">
+        <v>0</v>
+      </c>
+      <c r="K664" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1252.97 &lt;= EMA21 1253.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO</t>
+        </is>
+      </c>
+      <c r="D665" t="n">
+        <v>11768</v>
+      </c>
+      <c r="E665" t="n">
+        <v>12219.85</v>
+      </c>
+      <c r="F665" t="n">
+        <v>12219.85</v>
+      </c>
+      <c r="G665" t="n">
+        <v>11867.9</v>
+      </c>
+      <c r="H665" t="n">
+        <v>11790.74</v>
+      </c>
+      <c r="I665" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J665" t="b">
+        <v>0</v>
+      </c>
+      <c r="K665" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 11768.00 &lt;= Upper 12219.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="D666" t="n">
+        <v>1043.5</v>
+      </c>
+      <c r="E666" t="n">
+        <v>1108.51</v>
+      </c>
+      <c r="F666" t="n">
+        <v>1108.51</v>
+      </c>
+      <c r="G666" t="n">
+        <v>1054.87</v>
+      </c>
+      <c r="H666" t="n">
+        <v>1065.44</v>
+      </c>
+      <c r="I666" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J666" t="b">
+        <v>0</v>
+      </c>
+      <c r="K666" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1054.87 &lt;= EMA21 1065.44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="D667" t="n">
+        <v>1940.5</v>
+      </c>
+      <c r="E667" t="n">
+        <v>2052.96</v>
+      </c>
+      <c r="F667" t="n">
+        <v>2052.96</v>
+      </c>
+      <c r="G667" t="n">
+        <v>1959.6</v>
+      </c>
+      <c r="H667" t="n">
+        <v>1976.07</v>
+      </c>
+      <c r="I667" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="J667" t="b">
+        <v>0</v>
+      </c>
+      <c r="K667" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1959.60 &lt;= EMA21 1976.07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>BAJAJHLDNG</t>
+        </is>
+      </c>
+      <c r="D668" t="n">
+        <v>10992</v>
+      </c>
+      <c r="E668" t="n">
+        <v>11636.21</v>
+      </c>
+      <c r="F668" t="n">
+        <v>11636.21</v>
+      </c>
+      <c r="G668" t="n">
+        <v>11124.59</v>
+      </c>
+      <c r="H668" t="n">
+        <v>11192.08</v>
+      </c>
+      <c r="I668" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="J668" t="b">
+        <v>0</v>
+      </c>
+      <c r="K668" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11124.59 &lt;= EMA21 11192.08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>BANKBARODA</t>
+        </is>
+      </c>
+      <c r="D669" t="n">
+        <v>237.62</v>
+      </c>
+      <c r="E669" t="n">
+        <v>248.86</v>
+      </c>
+      <c r="F669" t="n">
+        <v>248.86</v>
+      </c>
+      <c r="G669" t="n">
+        <v>238.13</v>
+      </c>
+      <c r="H669" t="n">
+        <v>240.88</v>
+      </c>
+      <c r="I669" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="J669" t="b">
+        <v>0</v>
+      </c>
+      <c r="K669" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 238.13 &lt;= EMA21 240.88)</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="D670" t="n">
+        <v>405</v>
+      </c>
+      <c r="E670" t="n">
+        <v>415.85</v>
+      </c>
+      <c r="F670" t="n">
+        <v>415.85</v>
+      </c>
+      <c r="G670" t="n">
+        <v>407.33</v>
+      </c>
+      <c r="H670" t="n">
+        <v>407.5</v>
+      </c>
+      <c r="I670" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J670" t="b">
+        <v>0</v>
+      </c>
+      <c r="K670" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 407.33 &lt;= EMA21 407.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>BPCL</t>
+        </is>
+      </c>
+      <c r="D671" t="n">
+        <v>303</v>
+      </c>
+      <c r="E671" t="n">
+        <v>326.39</v>
+      </c>
+      <c r="F671" t="n">
+        <v>326.39</v>
+      </c>
+      <c r="G671" t="n">
+        <v>310.32</v>
+      </c>
+      <c r="H671" t="n">
+        <v>313.39</v>
+      </c>
+      <c r="I671" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J671" t="b">
+        <v>0</v>
+      </c>
+      <c r="K671" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 310.32 &lt;= EMA21 313.39)</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="D672" t="n">
+        <v>1839</v>
+      </c>
+      <c r="E672" t="n">
+        <v>1998.31</v>
+      </c>
+      <c r="F672" t="n">
+        <v>1998.31</v>
+      </c>
+      <c r="G672" t="n">
+        <v>1851.58</v>
+      </c>
+      <c r="H672" t="n">
+        <v>1879.02</v>
+      </c>
+      <c r="I672" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J672" t="b">
+        <v>0</v>
+      </c>
+      <c r="K672" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1851.58 &lt;= EMA21 1879.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>BOSCHLTD</t>
+        </is>
+      </c>
+      <c r="D673" t="n">
+        <v>48775</v>
+      </c>
+      <c r="E673" t="n">
+        <v>49973.87</v>
+      </c>
+      <c r="F673" t="n">
+        <v>49973.87</v>
+      </c>
+      <c r="G673" t="n">
+        <v>48344.81</v>
+      </c>
+      <c r="H673" t="n">
+        <v>47492.02</v>
+      </c>
+      <c r="I673" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J673" t="b">
+        <v>0</v>
+      </c>
+      <c r="K673" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 48775.00 &lt;= Upper 49973.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>BRITANNIA</t>
+        </is>
+      </c>
+      <c r="D674" t="n">
+        <v>5009</v>
+      </c>
+      <c r="E674" t="n">
+        <v>5633.25</v>
+      </c>
+      <c r="F674" t="n">
+        <v>5633.25</v>
+      </c>
+      <c r="G674" t="n">
+        <v>5120.19</v>
+      </c>
+      <c r="H674" t="n">
+        <v>5231.16</v>
+      </c>
+      <c r="I674" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J674" t="b">
+        <v>0</v>
+      </c>
+      <c r="K674" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5120.19 &lt;= EMA21 5231.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="D675" t="n">
+        <v>914.55</v>
+      </c>
+      <c r="E675" t="n">
+        <v>925.4400000000001</v>
+      </c>
+      <c r="F675" t="n">
+        <v>925.4400000000001</v>
+      </c>
+      <c r="G675" t="n">
+        <v>903.33</v>
+      </c>
+      <c r="H675" t="n">
+        <v>894.3099999999999</v>
+      </c>
+      <c r="I675" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J675" t="b">
+        <v>0</v>
+      </c>
+      <c r="K675" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 914.55 &lt;= Upper 925.44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>CANBK</t>
+        </is>
+      </c>
+      <c r="D676" t="n">
+        <v>124.6</v>
+      </c>
+      <c r="E676" t="n">
+        <v>132.11</v>
+      </c>
+      <c r="F676" t="n">
+        <v>132.11</v>
+      </c>
+      <c r="G676" t="n">
+        <v>125.41</v>
+      </c>
+      <c r="H676" t="n">
+        <v>126.7</v>
+      </c>
+      <c r="I676" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="J676" t="b">
+        <v>0</v>
+      </c>
+      <c r="K676" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 125.41 &lt;= EMA21 126.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="D677" t="n">
+        <v>1859</v>
+      </c>
+      <c r="E677" t="n">
+        <v>1915.88</v>
+      </c>
+      <c r="F677" t="n">
+        <v>1915.88</v>
+      </c>
+      <c r="G677" t="n">
+        <v>1844.29</v>
+      </c>
+      <c r="H677" t="n">
+        <v>1849.57</v>
+      </c>
+      <c r="I677" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="J677" t="b">
+        <v>0</v>
+      </c>
+      <c r="K677" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1844.29 &lt;= EMA21 1849.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>CIPLA</t>
+        </is>
+      </c>
+      <c r="D678" t="n">
+        <v>1373.3</v>
+      </c>
+      <c r="E678" t="n">
+        <v>1466.35</v>
+      </c>
+      <c r="F678" t="n">
+        <v>1466.35</v>
+      </c>
+      <c r="G678" t="n">
+        <v>1391.68</v>
+      </c>
+      <c r="H678" t="n">
+        <v>1410.81</v>
+      </c>
+      <c r="I678" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="J678" t="b">
+        <v>0</v>
+      </c>
+      <c r="K678" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1391.68 &lt;= EMA21 1410.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="D679" t="n">
+        <v>432</v>
+      </c>
+      <c r="E679" t="n">
+        <v>430.09</v>
+      </c>
+      <c r="F679" t="n">
+        <v>430.09</v>
+      </c>
+      <c r="G679" t="n">
+        <v>418.35</v>
+      </c>
+      <c r="H679" t="n">
+        <v>411.71</v>
+      </c>
+      <c r="I679" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J679" t="b">
+        <v>0</v>
+      </c>
+      <c r="K679" t="inlineStr">
+        <is>
+          <t>LOW_VOLUME (VolRatio 0.79x &lt; 1.3x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>CUMMINSIND</t>
+        </is>
+      </c>
+      <c r="D680" t="n">
+        <v>5155</v>
+      </c>
+      <c r="E680" t="n">
+        <v>5421.11</v>
+      </c>
+      <c r="F680" t="n">
+        <v>5421.11</v>
+      </c>
+      <c r="G680" t="n">
+        <v>5126.96</v>
+      </c>
+      <c r="H680" t="n">
+        <v>5198.03</v>
+      </c>
+      <c r="I680" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="J680" t="b">
+        <v>0</v>
+      </c>
+      <c r="K680" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5126.96 &lt;= EMA21 5198.03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>DLF</t>
+        </is>
+      </c>
+      <c r="D681" t="n">
+        <v>655.85</v>
+      </c>
+      <c r="E681" t="n">
+        <v>693.14</v>
+      </c>
+      <c r="F681" t="n">
+        <v>693.14</v>
+      </c>
+      <c r="G681" t="n">
+        <v>669.9299999999999</v>
+      </c>
+      <c r="H681" t="n">
+        <v>669.8</v>
+      </c>
+      <c r="I681" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J681" t="b">
+        <v>0</v>
+      </c>
+      <c r="K681" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 655.85 &lt;= Upper 693.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>DIVISLAB</t>
+        </is>
+      </c>
+      <c r="D682" t="n">
+        <v>9438.5</v>
+      </c>
+      <c r="E682" t="n">
+        <v>9768.66</v>
+      </c>
+      <c r="F682" t="n">
+        <v>9768.66</v>
+      </c>
+      <c r="G682" t="n">
+        <v>9307.610000000001</v>
+      </c>
+      <c r="H682" t="n">
+        <v>8989.719999999999</v>
+      </c>
+      <c r="I682" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J682" t="b">
+        <v>0</v>
+      </c>
+      <c r="K682" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 9438.50 &lt;= Upper 9768.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="D683" t="n">
+        <v>1143</v>
+      </c>
+      <c r="E683" t="n">
+        <v>1205.42</v>
+      </c>
+      <c r="F683" t="n">
+        <v>1205.42</v>
+      </c>
+      <c r="G683" t="n">
+        <v>1153.41</v>
+      </c>
+      <c r="H683" t="n">
+        <v>1165.9</v>
+      </c>
+      <c r="I683" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="J683" t="b">
+        <v>0</v>
+      </c>
+      <c r="K683" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1153.41 &lt;= EMA21 1165.90)</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>EICHERMOT</t>
+        </is>
+      </c>
+      <c r="D684" t="n">
+        <v>7697</v>
+      </c>
+      <c r="E684" t="n">
+        <v>8260.059999999999</v>
+      </c>
+      <c r="F684" t="n">
+        <v>8260.059999999999</v>
+      </c>
+      <c r="G684" t="n">
+        <v>7786.65</v>
+      </c>
+      <c r="H684" t="n">
+        <v>7851.26</v>
+      </c>
+      <c r="I684" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J684" t="b">
+        <v>0</v>
+      </c>
+      <c r="K684" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7786.65 &lt;= EMA21 7851.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>ETERNAL</t>
+        </is>
+      </c>
+      <c r="D685" t="n">
+        <v>322.1</v>
+      </c>
+      <c r="E685" t="n">
+        <v>333.14</v>
+      </c>
+      <c r="F685" t="n">
+        <v>333.14</v>
+      </c>
+      <c r="G685" t="n">
+        <v>323.57</v>
+      </c>
+      <c r="H685" t="n">
+        <v>321.16</v>
+      </c>
+      <c r="I685" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="J685" t="b">
+        <v>0</v>
+      </c>
+      <c r="K685" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 322.10 &lt;= Upper 333.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>GAIL</t>
+        </is>
+      </c>
+      <c r="D686" t="n">
+        <v>174.49</v>
+      </c>
+      <c r="E686" t="n">
+        <v>176.86</v>
+      </c>
+      <c r="F686" t="n">
+        <v>176.86</v>
+      </c>
+      <c r="G686" t="n">
+        <v>174.37</v>
+      </c>
+      <c r="H686" t="n">
+        <v>173.97</v>
+      </c>
+      <c r="I686" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J686" t="b">
+        <v>0</v>
+      </c>
+      <c r="K686" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 174.49 &lt;= Upper 176.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>GODREJCP</t>
+        </is>
+      </c>
+      <c r="D687" t="n">
+        <v>869.9</v>
+      </c>
+      <c r="E687" t="n">
+        <v>963.34</v>
+      </c>
+      <c r="F687" t="n">
+        <v>963.34</v>
+      </c>
+      <c r="G687" t="n">
+        <v>881.53</v>
+      </c>
+      <c r="H687" t="n">
+        <v>914.08</v>
+      </c>
+      <c r="I687" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="J687" t="b">
+        <v>0</v>
+      </c>
+      <c r="K687" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 881.53 &lt;= EMA21 914.08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>GRASIM</t>
+        </is>
+      </c>
+      <c r="D688" t="n">
+        <v>3319</v>
+      </c>
+      <c r="E688" t="n">
+        <v>3350.78</v>
+      </c>
+      <c r="F688" t="n">
+        <v>3350.78</v>
+      </c>
+      <c r="G688" t="n">
+        <v>3307.61</v>
+      </c>
+      <c r="H688" t="n">
+        <v>3287.06</v>
+      </c>
+      <c r="I688" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J688" t="b">
+        <v>0</v>
+      </c>
+      <c r="K688" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3319.00 &lt;= Upper 3350.78)</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="D689" t="n">
+        <v>1207</v>
+      </c>
+      <c r="E689" t="n">
+        <v>1375.72</v>
+      </c>
+      <c r="F689" t="n">
+        <v>1375.72</v>
+      </c>
+      <c r="G689" t="n">
+        <v>1272.03</v>
+      </c>
+      <c r="H689" t="n">
+        <v>1292.65</v>
+      </c>
+      <c r="I689" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="J689" t="b">
+        <v>0</v>
+      </c>
+      <c r="K689" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1272.03 &lt;= EMA21 1292.65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>HDFCAMC</t>
+        </is>
+      </c>
+      <c r="D690" t="n">
+        <v>2433.8</v>
+      </c>
+      <c r="E690" t="n">
+        <v>2698.82</v>
+      </c>
+      <c r="F690" t="n">
+        <v>2698.82</v>
+      </c>
+      <c r="G690" t="n">
+        <v>2492.45</v>
+      </c>
+      <c r="H690" t="n">
+        <v>2531.91</v>
+      </c>
+      <c r="I690" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="J690" t="b">
+        <v>0</v>
+      </c>
+      <c r="K690" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2492.45 &lt;= EMA21 2531.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="D691" t="n">
+        <v>693.8</v>
+      </c>
+      <c r="E691" t="n">
+        <v>739.9</v>
+      </c>
+      <c r="F691" t="n">
+        <v>739.9</v>
+      </c>
+      <c r="G691" t="n">
+        <v>703.58</v>
+      </c>
+      <c r="H691" t="n">
+        <v>715.1</v>
+      </c>
+      <c r="I691" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J691" t="b">
+        <v>0</v>
+      </c>
+      <c r="K691" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 703.58 &lt;= EMA21 715.10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="D692" t="n">
+        <v>526.15</v>
+      </c>
+      <c r="E692" t="n">
+        <v>559.98</v>
+      </c>
+      <c r="F692" t="n">
+        <v>559.98</v>
+      </c>
+      <c r="G692" t="n">
+        <v>532.41</v>
+      </c>
+      <c r="H692" t="n">
+        <v>538.58</v>
+      </c>
+      <c r="I692" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="J692" t="b">
+        <v>0</v>
+      </c>
+      <c r="K692" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 532.41 &lt;= EMA21 538.58)</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="D693" t="n">
+        <v>1014</v>
+      </c>
+      <c r="E693" t="n">
+        <v>1062.99</v>
+      </c>
+      <c r="F693" t="n">
+        <v>1062.99</v>
+      </c>
+      <c r="G693" t="n">
+        <v>1018.98</v>
+      </c>
+      <c r="H693" t="n">
+        <v>1021.54</v>
+      </c>
+      <c r="I693" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J693" t="b">
+        <v>0</v>
+      </c>
+      <c r="K693" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1018.98 &lt;= EMA21 1021.54)</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="D694" t="n">
+        <v>4950</v>
+      </c>
+      <c r="E694" t="n">
+        <v>5125.78</v>
+      </c>
+      <c r="F694" t="n">
+        <v>5125.78</v>
+      </c>
+      <c r="G694" t="n">
+        <v>4912.84</v>
+      </c>
+      <c r="H694" t="n">
+        <v>4878.49</v>
+      </c>
+      <c r="I694" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J694" t="b">
+        <v>0</v>
+      </c>
+      <c r="K694" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 4950.00 &lt;= Upper 5125.78)</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="D695" t="n">
+        <v>1942.3</v>
+      </c>
+      <c r="E695" t="n">
+        <v>2089.4</v>
+      </c>
+      <c r="F695" t="n">
+        <v>2089.4</v>
+      </c>
+      <c r="G695" t="n">
+        <v>1972.4</v>
+      </c>
+      <c r="H695" t="n">
+        <v>2006.18</v>
+      </c>
+      <c r="I695" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J695" t="b">
+        <v>0</v>
+      </c>
+      <c r="K695" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1972.40 &lt;= EMA21 2006.18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+      <c r="D696" t="n">
+        <v>593.6</v>
+      </c>
+      <c r="E696" t="n">
+        <v>629.8099999999999</v>
+      </c>
+      <c r="F696" t="n">
+        <v>629.8099999999999</v>
+      </c>
+      <c r="G696" t="n">
+        <v>596.37</v>
+      </c>
+      <c r="H696" t="n">
+        <v>590.33</v>
+      </c>
+      <c r="I696" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="J696" t="b">
+        <v>0</v>
+      </c>
+      <c r="K696" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 593.60 &lt;= Upper 629.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>HYUNDAI</t>
+        </is>
+      </c>
+      <c r="D697" t="n">
+        <v>2205</v>
+      </c>
+      <c r="E697" t="n">
+        <v>2267.32</v>
+      </c>
+      <c r="F697" t="n">
+        <v>2267.32</v>
+      </c>
+      <c r="G697" t="n">
+        <v>2200.29</v>
+      </c>
+      <c r="H697" t="n">
+        <v>2190.14</v>
+      </c>
+      <c r="I697" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="J697" t="b">
+        <v>0</v>
+      </c>
+      <c r="K697" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 2205.00 &lt;= Upper 2267.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="D698" t="n">
+        <v>1384.5</v>
+      </c>
+      <c r="E698" t="n">
+        <v>1453.13</v>
+      </c>
+      <c r="F698" t="n">
+        <v>1453.13</v>
+      </c>
+      <c r="G698" t="n">
+        <v>1409.85</v>
+      </c>
+      <c r="H698" t="n">
+        <v>1417.43</v>
+      </c>
+      <c r="I698" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="J698" t="b">
+        <v>0</v>
+      </c>
+      <c r="K698" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1409.85 &lt;= EMA21 1417.43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="D699" t="n">
+        <v>259.3</v>
+      </c>
+      <c r="E699" t="n">
+        <v>277.38</v>
+      </c>
+      <c r="F699" t="n">
+        <v>277.38</v>
+      </c>
+      <c r="G699" t="n">
+        <v>263.17</v>
+      </c>
+      <c r="H699" t="n">
+        <v>267.53</v>
+      </c>
+      <c r="I699" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="J699" t="b">
+        <v>0</v>
+      </c>
+      <c r="K699" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 263.17 &lt;= EMA21 267.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>INDHOTEL</t>
+        </is>
+      </c>
+      <c r="D700" t="n">
+        <v>715.75</v>
+      </c>
+      <c r="E700" t="n">
+        <v>738.37</v>
+      </c>
+      <c r="F700" t="n">
+        <v>738.37</v>
+      </c>
+      <c r="G700" t="n">
+        <v>721.09</v>
+      </c>
+      <c r="H700" t="n">
+        <v>723.58</v>
+      </c>
+      <c r="I700" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="J700" t="b">
+        <v>0</v>
+      </c>
+      <c r="K700" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 721.09 &lt;= EMA21 723.58)</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>IOC</t>
+        </is>
+      </c>
+      <c r="D701" t="n">
+        <v>134.94</v>
+      </c>
+      <c r="E701" t="n">
+        <v>140.31</v>
+      </c>
+      <c r="F701" t="n">
+        <v>140.31</v>
+      </c>
+      <c r="G701" t="n">
+        <v>136.12</v>
+      </c>
+      <c r="H701" t="n">
+        <v>137.21</v>
+      </c>
+      <c r="I701" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J701" t="b">
+        <v>0</v>
+      </c>
+      <c r="K701" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 136.12 &lt;= EMA21 137.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>IRFC</t>
+        </is>
+      </c>
+      <c r="D702" t="n">
+        <v>81.08</v>
+      </c>
+      <c r="E702" t="n">
+        <v>88.88</v>
+      </c>
+      <c r="F702" t="n">
+        <v>88.88</v>
+      </c>
+      <c r="G702" t="n">
+        <v>82.63</v>
+      </c>
+      <c r="H702" t="n">
+        <v>84.34999999999999</v>
+      </c>
+      <c r="I702" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="J702" t="b">
+        <v>0</v>
+      </c>
+      <c r="K702" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 82.63 &lt;= EMA21 84.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="D703" t="n">
+        <v>1036.5</v>
+      </c>
+      <c r="E703" t="n">
+        <v>1188.38</v>
+      </c>
+      <c r="F703" t="n">
+        <v>1188.38</v>
+      </c>
+      <c r="G703" t="n">
+        <v>1087.74</v>
+      </c>
+      <c r="H703" t="n">
+        <v>1110.66</v>
+      </c>
+      <c r="I703" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="J703" t="b">
+        <v>0</v>
+      </c>
+      <c r="K703" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1087.74 &lt;= EMA21 1110.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>INDIGO</t>
+        </is>
+      </c>
+      <c r="D704" t="n">
+        <v>4945</v>
+      </c>
+      <c r="E704" t="n">
+        <v>5389.91</v>
+      </c>
+      <c r="F704" t="n">
+        <v>5389.91</v>
+      </c>
+      <c r="G704" t="n">
+        <v>5028.47</v>
+      </c>
+      <c r="H704" t="n">
+        <v>5108.74</v>
+      </c>
+      <c r="I704" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="J704" t="b">
+        <v>0</v>
+      </c>
+      <c r="K704" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5028.47 &lt;= EMA21 5108.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>JSWSTEEL</t>
+        </is>
+      </c>
+      <c r="D705" t="n">
+        <v>1304</v>
+      </c>
+      <c r="E705" t="n">
+        <v>1348.48</v>
+      </c>
+      <c r="F705" t="n">
+        <v>1348.48</v>
+      </c>
+      <c r="G705" t="n">
+        <v>1308.36</v>
+      </c>
+      <c r="H705" t="n">
+        <v>1304.13</v>
+      </c>
+      <c r="I705" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J705" t="b">
+        <v>0</v>
+      </c>
+      <c r="K705" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1304.00 &lt;= Upper 1348.48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>JINDALSTEL</t>
+        </is>
+      </c>
+      <c r="D706" t="n">
+        <v>1137</v>
+      </c>
+      <c r="E706" t="n">
+        <v>1199.93</v>
+      </c>
+      <c r="F706" t="n">
+        <v>1199.93</v>
+      </c>
+      <c r="G706" t="n">
+        <v>1149.09</v>
+      </c>
+      <c r="H706" t="n">
+        <v>1139.24</v>
+      </c>
+      <c r="I706" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J706" t="b">
+        <v>0</v>
+      </c>
+      <c r="K706" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1137.00 &lt;= Upper 1199.93)</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>JIOFIN</t>
+        </is>
+      </c>
+      <c r="D707" t="n">
+        <v>230.25</v>
+      </c>
+      <c r="E707" t="n">
+        <v>253.66</v>
+      </c>
+      <c r="F707" t="n">
+        <v>253.66</v>
+      </c>
+      <c r="G707" t="n">
+        <v>235.54</v>
+      </c>
+      <c r="H707" t="n">
+        <v>239.78</v>
+      </c>
+      <c r="I707" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J707" t="b">
+        <v>0</v>
+      </c>
+      <c r="K707" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 235.54 &lt;= EMA21 239.78)</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="D708" t="n">
+        <v>416.55</v>
+      </c>
+      <c r="E708" t="n">
+        <v>437.68</v>
+      </c>
+      <c r="F708" t="n">
+        <v>437.68</v>
+      </c>
+      <c r="G708" t="n">
+        <v>417.84</v>
+      </c>
+      <c r="H708" t="n">
+        <v>411.86</v>
+      </c>
+      <c r="I708" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J708" t="b">
+        <v>0</v>
+      </c>
+      <c r="K708" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 416.55 &lt;= Upper 437.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>LTM</t>
+        </is>
+      </c>
+      <c r="D709" t="n">
+        <v>4374</v>
+      </c>
+      <c r="E709" t="n">
+        <v>4724.98</v>
+      </c>
+      <c r="F709" t="n">
+        <v>4724.98</v>
+      </c>
+      <c r="G709" t="n">
+        <v>4473.99</v>
+      </c>
+      <c r="H709" t="n">
+        <v>4499.31</v>
+      </c>
+      <c r="I709" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="J709" t="b">
+        <v>0</v>
+      </c>
+      <c r="K709" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4473.99 &lt;= EMA21 4499.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="D710" t="n">
+        <v>3955</v>
+      </c>
+      <c r="E710" t="n">
+        <v>4138.79</v>
+      </c>
+      <c r="F710" t="n">
+        <v>4138.79</v>
+      </c>
+      <c r="G710" t="n">
+        <v>3974.49</v>
+      </c>
+      <c r="H710" t="n">
+        <v>3997.46</v>
+      </c>
+      <c r="I710" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="J710" t="b">
+        <v>0</v>
+      </c>
+      <c r="K710" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3974.49 &lt;= EMA21 3997.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>LODHA</t>
+        </is>
+      </c>
+      <c r="D711" t="n">
+        <v>1163.4</v>
+      </c>
+      <c r="E711" t="n">
+        <v>1293.06</v>
+      </c>
+      <c r="F711" t="n">
+        <v>1293.06</v>
+      </c>
+      <c r="G711" t="n">
+        <v>1202.96</v>
+      </c>
+      <c r="H711" t="n">
+        <v>1213.96</v>
+      </c>
+      <c r="I711" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="J711" t="b">
+        <v>0</v>
+      </c>
+      <c r="K711" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1202.96 &lt;= EMA21 1213.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>M&amp;M</t>
+        </is>
+      </c>
+      <c r="D712" t="n">
+        <v>3123.8</v>
+      </c>
+      <c r="E712" t="n">
+        <v>3542.13</v>
+      </c>
+      <c r="F712" t="n">
+        <v>3542.13</v>
+      </c>
+      <c r="G712" t="n">
+        <v>3191.54</v>
+      </c>
+      <c r="H712" t="n">
+        <v>3258.64</v>
+      </c>
+      <c r="I712" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="J712" t="b">
+        <v>0</v>
+      </c>
+      <c r="K712" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3191.54 &lt;= EMA21 3258.64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="D713" t="n">
+        <v>12590</v>
+      </c>
+      <c r="E713" t="n">
+        <v>14201.53</v>
+      </c>
+      <c r="F713" t="n">
+        <v>14201.53</v>
+      </c>
+      <c r="G713" t="n">
+        <v>12838.5</v>
+      </c>
+      <c r="H713" t="n">
+        <v>13164</v>
+      </c>
+      <c r="I713" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J713" t="b">
+        <v>0</v>
+      </c>
+      <c r="K713" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 12838.50 &lt;= EMA21 13164.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>MAXHEALTH</t>
+        </is>
+      </c>
+      <c r="D714" t="n">
+        <v>1038.6</v>
+      </c>
+      <c r="E714" t="n">
+        <v>1040.04</v>
+      </c>
+      <c r="F714" t="n">
+        <v>1040.04</v>
+      </c>
+      <c r="G714" t="n">
+        <v>1014.17</v>
+      </c>
+      <c r="H714" t="n">
+        <v>1020.01</v>
+      </c>
+      <c r="I714" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="J714" t="b">
+        <v>0</v>
+      </c>
+      <c r="K714" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1014.17 &lt;= EMA21 1020.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>MAZDOCK</t>
+        </is>
+      </c>
+      <c r="D715" t="n">
+        <v>2383.2</v>
+      </c>
+      <c r="E715" t="n">
+        <v>2660.14</v>
+      </c>
+      <c r="F715" t="n">
+        <v>2660.14</v>
+      </c>
+      <c r="G715" t="n">
+        <v>2460.7</v>
+      </c>
+      <c r="H715" t="n">
+        <v>2486.31</v>
+      </c>
+      <c r="I715" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="J715" t="b">
+        <v>0</v>
+      </c>
+      <c r="K715" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2460.70 &lt;= EMA21 2486.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>MUTHOOTFIN</t>
+        </is>
+      </c>
+      <c r="D716" t="n">
+        <v>2841.5</v>
+      </c>
+      <c r="E716" t="n">
+        <v>3220.52</v>
+      </c>
+      <c r="F716" t="n">
+        <v>3220.52</v>
+      </c>
+      <c r="G716" t="n">
+        <v>2903.4</v>
+      </c>
+      <c r="H716" t="n">
+        <v>2945.26</v>
+      </c>
+      <c r="I716" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J716" t="b">
+        <v>0</v>
+      </c>
+      <c r="K716" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2903.40 &lt;= EMA21 2945.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="D717" t="n">
+        <v>335</v>
+      </c>
+      <c r="E717" t="n">
+        <v>339.58</v>
+      </c>
+      <c r="F717" t="n">
+        <v>339.58</v>
+      </c>
+      <c r="G717" t="n">
+        <v>332.11</v>
+      </c>
+      <c r="H717" t="n">
+        <v>333.11</v>
+      </c>
+      <c r="I717" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J717" t="b">
+        <v>0</v>
+      </c>
+      <c r="K717" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 332.11 &lt;= EMA21 333.11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="D718" t="n">
+        <v>1386.2</v>
+      </c>
+      <c r="E718" t="n">
+        <v>1514.6</v>
+      </c>
+      <c r="F718" t="n">
+        <v>1514.6</v>
+      </c>
+      <c r="G718" t="n">
+        <v>1412.88</v>
+      </c>
+      <c r="H718" t="n">
+        <v>1438.47</v>
+      </c>
+      <c r="I718" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="J718" t="b">
+        <v>0</v>
+      </c>
+      <c r="K718" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1412.88 &lt;= EMA21 1438.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="D719" t="n">
+        <v>237.27</v>
+      </c>
+      <c r="E719" t="n">
+        <v>239.55</v>
+      </c>
+      <c r="F719" t="n">
+        <v>239.55</v>
+      </c>
+      <c r="G719" t="n">
+        <v>235.05</v>
+      </c>
+      <c r="H719" t="n">
+        <v>235.66</v>
+      </c>
+      <c r="I719" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="J719" t="b">
+        <v>0</v>
+      </c>
+      <c r="K719" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 235.05 &lt;= EMA21 235.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>PIDILITIND</t>
+        </is>
+      </c>
+      <c r="D720" t="n">
+        <v>1569</v>
+      </c>
+      <c r="E720" t="n">
+        <v>1711.7</v>
+      </c>
+      <c r="F720" t="n">
+        <v>1711.7</v>
+      </c>
+      <c r="G720" t="n">
+        <v>1604.53</v>
+      </c>
+      <c r="H720" t="n">
+        <v>1625.02</v>
+      </c>
+      <c r="I720" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J720" t="b">
+        <v>0</v>
+      </c>
+      <c r="K720" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1604.53 &lt;= EMA21 1625.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>PFC</t>
+        </is>
+      </c>
+      <c r="D721" t="n">
+        <v>352.8</v>
+      </c>
+      <c r="E721" t="n">
+        <v>375.87</v>
+      </c>
+      <c r="F721" t="n">
+        <v>375.87</v>
+      </c>
+      <c r="G721" t="n">
+        <v>352.82</v>
+      </c>
+      <c r="H721" t="n">
+        <v>360.79</v>
+      </c>
+      <c r="I721" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J721" t="b">
+        <v>0</v>
+      </c>
+      <c r="K721" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 352.82 &lt;= EMA21 360.79)</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="D722" t="n">
+        <v>271.75</v>
+      </c>
+      <c r="E722" t="n">
+        <v>272.19</v>
+      </c>
+      <c r="F722" t="n">
+        <v>272.19</v>
+      </c>
+      <c r="G722" t="n">
+        <v>267.21</v>
+      </c>
+      <c r="H722" t="n">
+        <v>268.72</v>
+      </c>
+      <c r="I722" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J722" t="b">
+        <v>0</v>
+      </c>
+      <c r="K722" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 267.21 &lt;= EMA21 268.72)</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="D723" t="n">
+        <v>116.85</v>
+      </c>
+      <c r="E723" t="n">
+        <v>118.3</v>
+      </c>
+      <c r="F723" t="n">
+        <v>118.3</v>
+      </c>
+      <c r="G723" t="n">
+        <v>116.14</v>
+      </c>
+      <c r="H723" t="n">
+        <v>115.66</v>
+      </c>
+      <c r="I723" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="J723" t="b">
+        <v>0</v>
+      </c>
+      <c r="K723" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 116.85 &lt;= Upper 118.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="D724" t="n">
+        <v>313.8</v>
+      </c>
+      <c r="E724" t="n">
+        <v>340.79</v>
+      </c>
+      <c r="F724" t="n">
+        <v>340.79</v>
+      </c>
+      <c r="G724" t="n">
+        <v>317.31</v>
+      </c>
+      <c r="H724" t="n">
+        <v>324.93</v>
+      </c>
+      <c r="I724" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J724" t="b">
+        <v>0</v>
+      </c>
+      <c r="K724" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 317.31 &lt;= EMA21 324.93)</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="D725" t="n">
+        <v>1274</v>
+      </c>
+      <c r="E725" t="n">
+        <v>1334.18</v>
+      </c>
+      <c r="F725" t="n">
+        <v>1334.18</v>
+      </c>
+      <c r="G725" t="n">
+        <v>1294.26</v>
+      </c>
+      <c r="H725" t="n">
+        <v>1300.27</v>
+      </c>
+      <c r="I725" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J725" t="b">
+        <v>0</v>
+      </c>
+      <c r="K725" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1294.26 &lt;= EMA21 1300.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="D726" t="n">
+        <v>1700.6</v>
+      </c>
+      <c r="E726" t="n">
+        <v>1820.46</v>
+      </c>
+      <c r="F726" t="n">
+        <v>1820.46</v>
+      </c>
+      <c r="G726" t="n">
+        <v>1721.9</v>
+      </c>
+      <c r="H726" t="n">
+        <v>1753.2</v>
+      </c>
+      <c r="I726" t="n">
+        <v>1</v>
+      </c>
+      <c r="J726" t="b">
+        <v>0</v>
+      </c>
+      <c r="K726" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1721.90 &lt;= EMA21 1753.20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>MOTHERSON</t>
+        </is>
+      </c>
+      <c r="D727" t="n">
+        <v>163.2</v>
+      </c>
+      <c r="E727" t="n">
+        <v>172.46</v>
+      </c>
+      <c r="F727" t="n">
+        <v>172.46</v>
+      </c>
+      <c r="G727" t="n">
+        <v>163.78</v>
+      </c>
+      <c r="H727" t="n">
+        <v>163.55</v>
+      </c>
+      <c r="I727" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J727" t="b">
+        <v>0</v>
+      </c>
+      <c r="K727" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 163.20 &lt;= Upper 172.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="D728" t="n">
+        <v>22785</v>
+      </c>
+      <c r="E728" t="n">
+        <v>25222.47</v>
+      </c>
+      <c r="F728" t="n">
+        <v>25222.47</v>
+      </c>
+      <c r="G728" t="n">
+        <v>23401.46</v>
+      </c>
+      <c r="H728" t="n">
+        <v>24045.6</v>
+      </c>
+      <c r="I728" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="J728" t="b">
+        <v>0</v>
+      </c>
+      <c r="K728" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 23401.46 &lt;= EMA21 24045.60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>SHRIRAMFIN</t>
+        </is>
+      </c>
+      <c r="D729" t="n">
+        <v>1038</v>
+      </c>
+      <c r="E729" t="n">
+        <v>1165.24</v>
+      </c>
+      <c r="F729" t="n">
+        <v>1165.24</v>
+      </c>
+      <c r="G729" t="n">
+        <v>1049.58</v>
+      </c>
+      <c r="H729" t="n">
+        <v>1069.41</v>
+      </c>
+      <c r="I729" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J729" t="b">
+        <v>0</v>
+      </c>
+      <c r="K729" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1049.58 &lt;= EMA21 1069.41)</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>ENRIN</t>
+        </is>
+      </c>
+      <c r="D730" t="n">
+        <v>3179.1</v>
+      </c>
+      <c r="E730" t="n">
+        <v>3647.01</v>
+      </c>
+      <c r="F730" t="n">
+        <v>3647.01</v>
+      </c>
+      <c r="G730" t="n">
+        <v>3193.92</v>
+      </c>
+      <c r="H730" t="n">
+        <v>3267.58</v>
+      </c>
+      <c r="I730" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J730" t="b">
+        <v>0</v>
+      </c>
+      <c r="K730" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3193.92 &lt;= EMA21 3267.58)</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+      <c r="D731" t="n">
+        <v>3954.4</v>
+      </c>
+      <c r="E731" t="n">
+        <v>4132.84</v>
+      </c>
+      <c r="F731" t="n">
+        <v>4132.84</v>
+      </c>
+      <c r="G731" t="n">
+        <v>3976.61</v>
+      </c>
+      <c r="H731" t="n">
+        <v>3965.98</v>
+      </c>
+      <c r="I731" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="J731" t="b">
+        <v>0</v>
+      </c>
+      <c r="K731" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3954.40 &lt;= Upper 4132.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>SOLARINDS</t>
+        </is>
+      </c>
+      <c r="D732" t="n">
+        <v>22370</v>
+      </c>
+      <c r="E732" t="n">
+        <v>22592.52</v>
+      </c>
+      <c r="F732" t="n">
+        <v>22592.52</v>
+      </c>
+      <c r="G732" t="n">
+        <v>21625.45</v>
+      </c>
+      <c r="H732" t="n">
+        <v>20765.86</v>
+      </c>
+      <c r="I732" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="J732" t="b">
+        <v>0</v>
+      </c>
+      <c r="K732" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 22370.00 &lt;= Upper 22592.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="D733" t="n">
+        <v>1009.7</v>
+      </c>
+      <c r="E733" t="n">
+        <v>1077.78</v>
+      </c>
+      <c r="F733" t="n">
+        <v>1077.78</v>
+      </c>
+      <c r="G733" t="n">
+        <v>1017.72</v>
+      </c>
+      <c r="H733" t="n">
+        <v>1030.86</v>
+      </c>
+      <c r="I733" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J733" t="b">
+        <v>0</v>
+      </c>
+      <c r="K733" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1017.72 &lt;= EMA21 1030.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="D734" t="n">
+        <v>1861</v>
+      </c>
+      <c r="E734" t="n">
+        <v>1961.55</v>
+      </c>
+      <c r="F734" t="n">
+        <v>1961.55</v>
+      </c>
+      <c r="G734" t="n">
+        <v>1892.69</v>
+      </c>
+      <c r="H734" t="n">
+        <v>1908.21</v>
+      </c>
+      <c r="I734" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J734" t="b">
+        <v>0</v>
+      </c>
+      <c r="K734" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1892.69 &lt;= EMA21 1908.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>TVSMOTOR</t>
+        </is>
+      </c>
+      <c r="D735" t="n">
+        <v>4121.5</v>
+      </c>
+      <c r="E735" t="n">
+        <v>4519.77</v>
+      </c>
+      <c r="F735" t="n">
+        <v>4519.77</v>
+      </c>
+      <c r="G735" t="n">
+        <v>4184.25</v>
+      </c>
+      <c r="H735" t="n">
+        <v>4225.06</v>
+      </c>
+      <c r="I735" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="J735" t="b">
+        <v>0</v>
+      </c>
+      <c r="K735" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4184.25 &lt;= EMA21 4225.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>TATACAP</t>
+        </is>
+      </c>
+      <c r="D736" t="n">
+        <v>363.15</v>
+      </c>
+      <c r="E736" t="n">
+        <v>376.57</v>
+      </c>
+      <c r="F736" t="n">
+        <v>376.57</v>
+      </c>
+      <c r="G736" t="n">
+        <v>367.28</v>
+      </c>
+      <c r="H736" t="n">
+        <v>366.83</v>
+      </c>
+      <c r="I736" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J736" t="b">
+        <v>0</v>
+      </c>
+      <c r="K736" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 363.15 &lt;= Upper 376.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="D737" t="n">
+        <v>2204.1</v>
+      </c>
+      <c r="E737" t="n">
+        <v>2398.44</v>
+      </c>
+      <c r="F737" t="n">
+        <v>2398.44</v>
+      </c>
+      <c r="G737" t="n">
+        <v>2268.16</v>
+      </c>
+      <c r="H737" t="n">
+        <v>2295.3</v>
+      </c>
+      <c r="I737" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J737" t="b">
+        <v>0</v>
+      </c>
+      <c r="K737" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2268.16 &lt;= EMA21 2295.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>TATACONSUM</t>
+        </is>
+      </c>
+      <c r="D738" t="n">
+        <v>999.6</v>
+      </c>
+      <c r="E738" t="n">
+        <v>1088.86</v>
+      </c>
+      <c r="F738" t="n">
+        <v>1088.86</v>
+      </c>
+      <c r="G738" t="n">
+        <v>1015.97</v>
+      </c>
+      <c r="H738" t="n">
+        <v>1036.31</v>
+      </c>
+      <c r="I738" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J738" t="b">
+        <v>0</v>
+      </c>
+      <c r="K738" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1015.97 &lt;= EMA21 1036.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>TMCV</t>
+        </is>
+      </c>
+      <c r="D739" t="n">
+        <v>439.25</v>
+      </c>
+      <c r="E739" t="n">
+        <v>489.98</v>
+      </c>
+      <c r="F739" t="n">
+        <v>489.98</v>
+      </c>
+      <c r="G739" t="n">
+        <v>454.28</v>
+      </c>
+      <c r="H739" t="n">
+        <v>457.27</v>
+      </c>
+      <c r="I739" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J739" t="b">
+        <v>0</v>
+      </c>
+      <c r="K739" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 454.28 &lt;= EMA21 457.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>TMPV</t>
+        </is>
+      </c>
+      <c r="D740" t="n">
+        <v>300.5</v>
+      </c>
+      <c r="E740" t="n">
+        <v>331.68</v>
+      </c>
+      <c r="F740" t="n">
+        <v>331.68</v>
+      </c>
+      <c r="G740" t="n">
+        <v>307.93</v>
+      </c>
+      <c r="H740" t="n">
+        <v>315.7</v>
+      </c>
+      <c r="I740" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J740" t="b">
+        <v>0</v>
+      </c>
+      <c r="K740" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 307.93 &lt;= EMA21 315.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>TATAPOWER</t>
+        </is>
+      </c>
+      <c r="D741" t="n">
+        <v>367</v>
+      </c>
+      <c r="E741" t="n">
+        <v>388.48</v>
+      </c>
+      <c r="F741" t="n">
+        <v>388.48</v>
+      </c>
+      <c r="G741" t="n">
+        <v>365.48</v>
+      </c>
+      <c r="H741" t="n">
+        <v>367.63</v>
+      </c>
+      <c r="I741" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J741" t="b">
+        <v>0</v>
+      </c>
+      <c r="K741" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 365.48 &lt;= EMA21 367.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="D742" t="n">
+        <v>186.78</v>
+      </c>
+      <c r="E742" t="n">
+        <v>189.12</v>
+      </c>
+      <c r="F742" t="n">
+        <v>189.12</v>
+      </c>
+      <c r="G742" t="n">
+        <v>186.22</v>
+      </c>
+      <c r="H742" t="n">
+        <v>186.18</v>
+      </c>
+      <c r="I742" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J742" t="b">
+        <v>0</v>
+      </c>
+      <c r="K742" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 186.78 &lt;= Upper 189.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>TECHM</t>
+        </is>
+      </c>
+      <c r="D743" t="n">
+        <v>1525.8</v>
+      </c>
+      <c r="E743" t="n">
+        <v>1660.38</v>
+      </c>
+      <c r="F743" t="n">
+        <v>1660.38</v>
+      </c>
+      <c r="G743" t="n">
+        <v>1565.19</v>
+      </c>
+      <c r="H743" t="n">
+        <v>1583.55</v>
+      </c>
+      <c r="I743" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J743" t="b">
+        <v>0</v>
+      </c>
+      <c r="K743" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1565.19 &lt;= EMA21 1583.55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>TITAN</t>
+        </is>
+      </c>
+      <c r="D744" t="n">
+        <v>5021</v>
+      </c>
+      <c r="E744" t="n">
+        <v>5160.57</v>
+      </c>
+      <c r="F744" t="n">
+        <v>5160.57</v>
+      </c>
+      <c r="G744" t="n">
+        <v>5029.87</v>
+      </c>
+      <c r="H744" t="n">
+        <v>5023.77</v>
+      </c>
+      <c r="I744" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J744" t="b">
+        <v>0</v>
+      </c>
+      <c r="K744" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 5021.00 &lt;= Upper 5160.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>TORNTPHARM</t>
+        </is>
+      </c>
+      <c r="D745" t="n">
+        <v>4930</v>
+      </c>
+      <c r="E745" t="n">
+        <v>5073</v>
+      </c>
+      <c r="F745" t="n">
+        <v>5073</v>
+      </c>
+      <c r="G745" t="n">
+        <v>4939.07</v>
+      </c>
+      <c r="H745" t="n">
+        <v>4941.94</v>
+      </c>
+      <c r="I745" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J745" t="b">
+        <v>0</v>
+      </c>
+      <c r="K745" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4939.07 &lt;= EMA21 4941.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="D746" t="n">
+        <v>2818.7</v>
+      </c>
+      <c r="E746" t="n">
+        <v>3000.92</v>
+      </c>
+      <c r="F746" t="n">
+        <v>3000.92</v>
+      </c>
+      <c r="G746" t="n">
+        <v>2837.09</v>
+      </c>
+      <c r="H746" t="n">
+        <v>2880.77</v>
+      </c>
+      <c r="I746" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J746" t="b">
+        <v>0</v>
+      </c>
+      <c r="K746" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2837.09 &lt;= EMA21 2880.77)</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="D747" t="n">
+        <v>10979</v>
+      </c>
+      <c r="E747" t="n">
+        <v>11904.76</v>
+      </c>
+      <c r="F747" t="n">
+        <v>11904.76</v>
+      </c>
+      <c r="G747" t="n">
+        <v>11187.64</v>
+      </c>
+      <c r="H747" t="n">
+        <v>11383.84</v>
+      </c>
+      <c r="I747" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J747" t="b">
+        <v>0</v>
+      </c>
+      <c r="K747" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11187.64 &lt;= EMA21 11383.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="D748" t="n">
+        <v>179.2</v>
+      </c>
+      <c r="E748" t="n">
+        <v>190.47</v>
+      </c>
+      <c r="F748" t="n">
+        <v>190.47</v>
+      </c>
+      <c r="G748" t="n">
+        <v>184.25</v>
+      </c>
+      <c r="H748" t="n">
+        <v>183.88</v>
+      </c>
+      <c r="I748" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J748" t="b">
+        <v>0</v>
+      </c>
+      <c r="K748" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 179.20 &lt;= Upper 190.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>UNITDSPR</t>
+        </is>
+      </c>
+      <c r="D749" t="n">
+        <v>1400</v>
+      </c>
+      <c r="E749" t="n">
+        <v>1597.26</v>
+      </c>
+      <c r="F749" t="n">
+        <v>1597.26</v>
+      </c>
+      <c r="G749" t="n">
+        <v>1448.99</v>
+      </c>
+      <c r="H749" t="n">
+        <v>1476.34</v>
+      </c>
+      <c r="I749" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J749" t="b">
+        <v>0</v>
+      </c>
+      <c r="K749" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1448.99 &lt;= EMA21 1476.34)</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="D750" t="n">
+        <v>410.5</v>
+      </c>
+      <c r="E750" t="n">
+        <v>446.35</v>
+      </c>
+      <c r="F750" t="n">
+        <v>446.35</v>
+      </c>
+      <c r="G750" t="n">
+        <v>410.27</v>
+      </c>
+      <c r="H750" t="n">
+        <v>419.65</v>
+      </c>
+      <c r="I750" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="J750" t="b">
+        <v>0</v>
+      </c>
+      <c r="K750" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 410.27 &lt;= EMA21 419.65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>VEDL</t>
+        </is>
+      </c>
+      <c r="D751" t="n">
+        <v>269.05</v>
+      </c>
+      <c r="E751" t="n">
+        <v>286.74</v>
+      </c>
+      <c r="F751" t="n">
+        <v>286.74</v>
+      </c>
+      <c r="G751" t="n">
+        <v>272.12</v>
+      </c>
+      <c r="H751" t="n">
+        <v>273.08</v>
+      </c>
+      <c r="I751" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="J751" t="b">
+        <v>0</v>
+      </c>
+      <c r="K751" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 272.12 &lt;= EMA21 273.08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="D752" t="n">
+        <v>166.3</v>
+      </c>
+      <c r="E752" t="n">
+        <v>187.85</v>
+      </c>
+      <c r="F752" t="n">
+        <v>187.85</v>
+      </c>
+      <c r="G752" t="n">
+        <v>172.84</v>
+      </c>
+      <c r="H752" t="n">
+        <v>176.49</v>
+      </c>
+      <c r="I752" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="J752" t="b">
+        <v>0</v>
+      </c>
+      <c r="K752" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 172.84 &lt;= EMA21 176.49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>ZYDUSLIFE</t>
+        </is>
+      </c>
+      <c r="D753" t="n">
+        <v>1117.8</v>
+      </c>
+      <c r="E753" t="n">
+        <v>1190.29</v>
+      </c>
+      <c r="F753" t="n">
+        <v>1190.29</v>
+      </c>
+      <c r="G753" t="n">
+        <v>1138.52</v>
+      </c>
+      <c r="H753" t="n">
+        <v>1139.97</v>
+      </c>
+      <c r="I753" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J753" t="b">
+        <v>0</v>
+      </c>
+      <c r="K753" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1138.52 &lt;= EMA21 1139.97)</t>
         </is>
       </c>
     </row>
@@ -28900,19 +33200,19 @@
         <v>19685.95</v>
       </c>
       <c r="F2" t="n">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="G2" t="n">
-        <v>2.9</v>
+        <v>3.14</v>
       </c>
       <c r="H2" t="n">
-        <v>415.76</v>
+        <v>416.67</v>
       </c>
       <c r="I2" t="n">
-        <v>435.3500061035156</v>
+        <v>436.2999877929688</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -28941,19 +33241,19 @@
         <v>19525</v>
       </c>
       <c r="F3" t="n">
-        <v>1775</v>
+        <v>1768</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>-0.39</v>
       </c>
       <c r="H3" t="n">
-        <v>1695.12</v>
+        <v>1699.9</v>
       </c>
       <c r="I3" t="n">
-        <v>1775</v>
+        <v>1780</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -28982,19 +33282,19 @@
         <v>19985.7</v>
       </c>
       <c r="F4" t="n">
-        <v>214.9</v>
+        <v>213.5</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>-0.65</v>
       </c>
       <c r="H4" t="n">
-        <v>205.23</v>
+        <v>205.59</v>
       </c>
       <c r="I4" t="n">
-        <v>214.9</v>
+        <v>215.2799987792969</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -29023,19 +33323,19 @@
         <v>19465.95</v>
       </c>
       <c r="F5" t="n">
-        <v>926.95</v>
+        <v>914.55</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>-1.34</v>
       </c>
       <c r="H5" t="n">
-        <v>885.24</v>
+        <v>889.11</v>
       </c>
       <c r="I5" t="n">
-        <v>926.95</v>
+        <v>931</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -35270,7 +39570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35650,6 +39950,39 @@
         <v>4</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>19:57:46</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>120159.33</v>
+      </c>
+      <c r="D12" t="n">
+        <v>78662.60000000001</v>
+      </c>
+      <c r="E12" t="n">
+        <v>198821.93</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-1092.43</v>
+      </c>
+      <c r="G12" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H12" t="n">
+        <v>17</v>
+      </c>
+      <c r="I12" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-11T19:57 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_india.xlsx
+++ b/data/trade_log_india.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K753"/>
+  <dimension ref="A1:K853"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32806,6 +32806,4306 @@
       <c r="K753" t="inlineStr">
         <is>
           <t>EMA_BEARISH (EMA9 1138.52 &lt;= EMA21 1139.97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+      <c r="D754" t="n">
+        <v>7274</v>
+      </c>
+      <c r="E754" t="n">
+        <v>7702.71</v>
+      </c>
+      <c r="F754" t="n">
+        <v>7702.71</v>
+      </c>
+      <c r="G754" t="n">
+        <v>7393.78</v>
+      </c>
+      <c r="H754" t="n">
+        <v>7439.32</v>
+      </c>
+      <c r="I754" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J754" t="b">
+        <v>0</v>
+      </c>
+      <c r="K754" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7393.78 &lt;= EMA21 7439.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="D755" t="n">
+        <v>1373</v>
+      </c>
+      <c r="E755" t="n">
+        <v>1672.08</v>
+      </c>
+      <c r="F755" t="n">
+        <v>1672.08</v>
+      </c>
+      <c r="G755" t="n">
+        <v>1415.65</v>
+      </c>
+      <c r="H755" t="n">
+        <v>1474.41</v>
+      </c>
+      <c r="I755" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="J755" t="b">
+        <v>0</v>
+      </c>
+      <c r="K755" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1415.65 &lt;= EMA21 1474.41)</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>ADANIENT</t>
+        </is>
+      </c>
+      <c r="D756" t="n">
+        <v>3060</v>
+      </c>
+      <c r="E756" t="n">
+        <v>3196.42</v>
+      </c>
+      <c r="F756" t="n">
+        <v>3196.42</v>
+      </c>
+      <c r="G756" t="n">
+        <v>3016.07</v>
+      </c>
+      <c r="H756" t="n">
+        <v>3011.12</v>
+      </c>
+      <c r="I756" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J756" t="b">
+        <v>0</v>
+      </c>
+      <c r="K756" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3060.00 &lt;= Upper 3196.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>ADANIGREEN</t>
+        </is>
+      </c>
+      <c r="D757" t="n">
+        <v>1281.3</v>
+      </c>
+      <c r="E757" t="n">
+        <v>1350.01</v>
+      </c>
+      <c r="F757" t="n">
+        <v>1350.01</v>
+      </c>
+      <c r="G757" t="n">
+        <v>1293.89</v>
+      </c>
+      <c r="H757" t="n">
+        <v>1309.64</v>
+      </c>
+      <c r="I757" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J757" t="b">
+        <v>0</v>
+      </c>
+      <c r="K757" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1293.89 &lt;= EMA21 1309.64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="D758" t="n">
+        <v>1764.6</v>
+      </c>
+      <c r="E758" t="n">
+        <v>1780.47</v>
+      </c>
+      <c r="F758" t="n">
+        <v>1780.47</v>
+      </c>
+      <c r="G758" t="n">
+        <v>1727.91</v>
+      </c>
+      <c r="H758" t="n">
+        <v>1712.62</v>
+      </c>
+      <c r="I758" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J758" t="b">
+        <v>0</v>
+      </c>
+      <c r="K758" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1764.60 &lt;= Upper 1780.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="D759" t="n">
+        <v>209.97</v>
+      </c>
+      <c r="E759" t="n">
+        <v>215.83</v>
+      </c>
+      <c r="F759" t="n">
+        <v>215.83</v>
+      </c>
+      <c r="G759" t="n">
+        <v>209.54</v>
+      </c>
+      <c r="H759" t="n">
+        <v>208.76</v>
+      </c>
+      <c r="I759" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="J759" t="b">
+        <v>0</v>
+      </c>
+      <c r="K759" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 209.97 &lt;= Upper 215.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>AMBUJACEM</t>
+        </is>
+      </c>
+      <c r="D760" t="n">
+        <v>391.85</v>
+      </c>
+      <c r="E760" t="n">
+        <v>421.15</v>
+      </c>
+      <c r="F760" t="n">
+        <v>421.15</v>
+      </c>
+      <c r="G760" t="n">
+        <v>399.32</v>
+      </c>
+      <c r="H760" t="n">
+        <v>406.64</v>
+      </c>
+      <c r="I760" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J760" t="b">
+        <v>0</v>
+      </c>
+      <c r="K760" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 399.32 &lt;= EMA21 406.64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="D761" t="n">
+        <v>8836</v>
+      </c>
+      <c r="E761" t="n">
+        <v>8975.4</v>
+      </c>
+      <c r="F761" t="n">
+        <v>8975.4</v>
+      </c>
+      <c r="G761" t="n">
+        <v>8825.41</v>
+      </c>
+      <c r="H761" t="n">
+        <v>8809.1</v>
+      </c>
+      <c r="I761" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J761" t="b">
+        <v>0</v>
+      </c>
+      <c r="K761" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 8836.00 &lt;= Upper 8975.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="D762" t="n">
+        <v>2472.5</v>
+      </c>
+      <c r="E762" t="n">
+        <v>2718.87</v>
+      </c>
+      <c r="F762" t="n">
+        <v>2718.87</v>
+      </c>
+      <c r="G762" t="n">
+        <v>2517.86</v>
+      </c>
+      <c r="H762" t="n">
+        <v>2574.77</v>
+      </c>
+      <c r="I762" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J762" t="b">
+        <v>0</v>
+      </c>
+      <c r="K762" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2517.86 &lt;= EMA21 2574.77)</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="D763" t="n">
+        <v>3688</v>
+      </c>
+      <c r="E763" t="n">
+        <v>4042.24</v>
+      </c>
+      <c r="F763" t="n">
+        <v>4042.24</v>
+      </c>
+      <c r="G763" t="n">
+        <v>3746.7</v>
+      </c>
+      <c r="H763" t="n">
+        <v>3821.78</v>
+      </c>
+      <c r="I763" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="J763" t="b">
+        <v>0</v>
+      </c>
+      <c r="K763" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3746.70 &lt;= EMA21 3821.78)</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="D764" t="n">
+        <v>1246</v>
+      </c>
+      <c r="E764" t="n">
+        <v>1285.71</v>
+      </c>
+      <c r="F764" t="n">
+        <v>1285.71</v>
+      </c>
+      <c r="G764" t="n">
+        <v>1251.58</v>
+      </c>
+      <c r="H764" t="n">
+        <v>1252.5</v>
+      </c>
+      <c r="I764" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J764" t="b">
+        <v>0</v>
+      </c>
+      <c r="K764" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1251.58 &lt;= EMA21 1252.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO</t>
+        </is>
+      </c>
+      <c r="D765" t="n">
+        <v>11678</v>
+      </c>
+      <c r="E765" t="n">
+        <v>12220.66</v>
+      </c>
+      <c r="F765" t="n">
+        <v>12220.66</v>
+      </c>
+      <c r="G765" t="n">
+        <v>11829.92</v>
+      </c>
+      <c r="H765" t="n">
+        <v>11780.49</v>
+      </c>
+      <c r="I765" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J765" t="b">
+        <v>0</v>
+      </c>
+      <c r="K765" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 11678.00 &lt;= Upper 12220.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="D766" t="n">
+        <v>1034.5</v>
+      </c>
+      <c r="E766" t="n">
+        <v>1108.54</v>
+      </c>
+      <c r="F766" t="n">
+        <v>1108.54</v>
+      </c>
+      <c r="G766" t="n">
+        <v>1050.8</v>
+      </c>
+      <c r="H766" t="n">
+        <v>1062.63</v>
+      </c>
+      <c r="I766" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="J766" t="b">
+        <v>0</v>
+      </c>
+      <c r="K766" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1050.80 &lt;= EMA21 1062.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="D767" t="n">
+        <v>1913.5</v>
+      </c>
+      <c r="E767" t="n">
+        <v>2056.25</v>
+      </c>
+      <c r="F767" t="n">
+        <v>2056.25</v>
+      </c>
+      <c r="G767" t="n">
+        <v>1950.38</v>
+      </c>
+      <c r="H767" t="n">
+        <v>1970.38</v>
+      </c>
+      <c r="I767" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="J767" t="b">
+        <v>0</v>
+      </c>
+      <c r="K767" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1950.38 &lt;= EMA21 1970.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>BAJAJHLDNG</t>
+        </is>
+      </c>
+      <c r="D768" t="n">
+        <v>11134</v>
+      </c>
+      <c r="E768" t="n">
+        <v>11609.91</v>
+      </c>
+      <c r="F768" t="n">
+        <v>11609.91</v>
+      </c>
+      <c r="G768" t="n">
+        <v>11126.48</v>
+      </c>
+      <c r="H768" t="n">
+        <v>11186.8</v>
+      </c>
+      <c r="I768" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J768" t="b">
+        <v>0</v>
+      </c>
+      <c r="K768" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11126.48 &lt;= EMA21 11186.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>BANKBARODA</t>
+        </is>
+      </c>
+      <c r="D769" t="n">
+        <v>238.13</v>
+      </c>
+      <c r="E769" t="n">
+        <v>247.72</v>
+      </c>
+      <c r="F769" t="n">
+        <v>247.72</v>
+      </c>
+      <c r="G769" t="n">
+        <v>238.13</v>
+      </c>
+      <c r="H769" t="n">
+        <v>240.63</v>
+      </c>
+      <c r="I769" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J769" t="b">
+        <v>0</v>
+      </c>
+      <c r="K769" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 238.13 &lt;= EMA21 240.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="D770" t="n">
+        <v>404.35</v>
+      </c>
+      <c r="E770" t="n">
+        <v>415.91</v>
+      </c>
+      <c r="F770" t="n">
+        <v>415.91</v>
+      </c>
+      <c r="G770" t="n">
+        <v>406.73</v>
+      </c>
+      <c r="H770" t="n">
+        <v>407.22</v>
+      </c>
+      <c r="I770" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J770" t="b">
+        <v>0</v>
+      </c>
+      <c r="K770" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 406.73 &lt;= EMA21 407.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>BPCL</t>
+        </is>
+      </c>
+      <c r="D771" t="n">
+        <v>304.5</v>
+      </c>
+      <c r="E771" t="n">
+        <v>326.04</v>
+      </c>
+      <c r="F771" t="n">
+        <v>326.04</v>
+      </c>
+      <c r="G771" t="n">
+        <v>309.16</v>
+      </c>
+      <c r="H771" t="n">
+        <v>312.58</v>
+      </c>
+      <c r="I771" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J771" t="b">
+        <v>0</v>
+      </c>
+      <c r="K771" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 309.16 &lt;= EMA21 312.58)</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="D772" t="n">
+        <v>1831.1</v>
+      </c>
+      <c r="E772" t="n">
+        <v>1982.75</v>
+      </c>
+      <c r="F772" t="n">
+        <v>1982.75</v>
+      </c>
+      <c r="G772" t="n">
+        <v>1847.48</v>
+      </c>
+      <c r="H772" t="n">
+        <v>1874.66</v>
+      </c>
+      <c r="I772" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J772" t="b">
+        <v>0</v>
+      </c>
+      <c r="K772" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1847.48 &lt;= EMA21 1874.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>BOSCHLTD</t>
+        </is>
+      </c>
+      <c r="D773" t="n">
+        <v>48385</v>
+      </c>
+      <c r="E773" t="n">
+        <v>49944.45</v>
+      </c>
+      <c r="F773" t="n">
+        <v>49944.45</v>
+      </c>
+      <c r="G773" t="n">
+        <v>48352.85</v>
+      </c>
+      <c r="H773" t="n">
+        <v>47573.2</v>
+      </c>
+      <c r="I773" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J773" t="b">
+        <v>0</v>
+      </c>
+      <c r="K773" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 48385.00 &lt;= Upper 49944.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>BRITANNIA</t>
+        </is>
+      </c>
+      <c r="D774" t="n">
+        <v>4962</v>
+      </c>
+      <c r="E774" t="n">
+        <v>5604.87</v>
+      </c>
+      <c r="F774" t="n">
+        <v>5604.87</v>
+      </c>
+      <c r="G774" t="n">
+        <v>5088.56</v>
+      </c>
+      <c r="H774" t="n">
+        <v>5206.69</v>
+      </c>
+      <c r="I774" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J774" t="b">
+        <v>0</v>
+      </c>
+      <c r="K774" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5088.56 &lt;= EMA21 5206.69)</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="D775" t="n">
+        <v>909</v>
+      </c>
+      <c r="E775" t="n">
+        <v>927.35</v>
+      </c>
+      <c r="F775" t="n">
+        <v>927.35</v>
+      </c>
+      <c r="G775" t="n">
+        <v>904.46</v>
+      </c>
+      <c r="H775" t="n">
+        <v>895.64</v>
+      </c>
+      <c r="I775" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J775" t="b">
+        <v>0</v>
+      </c>
+      <c r="K775" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 909.00 &lt;= Upper 927.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>CANBK</t>
+        </is>
+      </c>
+      <c r="D776" t="n">
+        <v>124</v>
+      </c>
+      <c r="E776" t="n">
+        <v>131.64</v>
+      </c>
+      <c r="F776" t="n">
+        <v>131.64</v>
+      </c>
+      <c r="G776" t="n">
+        <v>125.13</v>
+      </c>
+      <c r="H776" t="n">
+        <v>126.46</v>
+      </c>
+      <c r="I776" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J776" t="b">
+        <v>0</v>
+      </c>
+      <c r="K776" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 125.13 &lt;= EMA21 126.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="D777" t="n">
+        <v>1845.9</v>
+      </c>
+      <c r="E777" t="n">
+        <v>1902.18</v>
+      </c>
+      <c r="F777" t="n">
+        <v>1902.18</v>
+      </c>
+      <c r="G777" t="n">
+        <v>1844.61</v>
+      </c>
+      <c r="H777" t="n">
+        <v>1849.23</v>
+      </c>
+      <c r="I777" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="J777" t="b">
+        <v>0</v>
+      </c>
+      <c r="K777" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1844.61 &lt;= EMA21 1849.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>CIPLA</t>
+        </is>
+      </c>
+      <c r="D778" t="n">
+        <v>1366</v>
+      </c>
+      <c r="E778" t="n">
+        <v>1462.1</v>
+      </c>
+      <c r="F778" t="n">
+        <v>1462.1</v>
+      </c>
+      <c r="G778" t="n">
+        <v>1386.54</v>
+      </c>
+      <c r="H778" t="n">
+        <v>1406.74</v>
+      </c>
+      <c r="I778" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="J778" t="b">
+        <v>0</v>
+      </c>
+      <c r="K778" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1386.54 &lt;= EMA21 1406.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="D779" t="n">
+        <v>426.4</v>
+      </c>
+      <c r="E779" t="n">
+        <v>432.82</v>
+      </c>
+      <c r="F779" t="n">
+        <v>432.82</v>
+      </c>
+      <c r="G779" t="n">
+        <v>419.96</v>
+      </c>
+      <c r="H779" t="n">
+        <v>413.04</v>
+      </c>
+      <c r="I779" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J779" t="b">
+        <v>0</v>
+      </c>
+      <c r="K779" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 426.40 &lt;= Upper 432.82)</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>CUMMINSIND</t>
+        </is>
+      </c>
+      <c r="D780" t="n">
+        <v>5070</v>
+      </c>
+      <c r="E780" t="n">
+        <v>5407.25</v>
+      </c>
+      <c r="F780" t="n">
+        <v>5407.25</v>
+      </c>
+      <c r="G780" t="n">
+        <v>5115.57</v>
+      </c>
+      <c r="H780" t="n">
+        <v>5186.39</v>
+      </c>
+      <c r="I780" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J780" t="b">
+        <v>0</v>
+      </c>
+      <c r="K780" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5115.57 &lt;= EMA21 5186.39)</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>DLF</t>
+        </is>
+      </c>
+      <c r="D781" t="n">
+        <v>644.5</v>
+      </c>
+      <c r="E781" t="n">
+        <v>695.92</v>
+      </c>
+      <c r="F781" t="n">
+        <v>695.92</v>
+      </c>
+      <c r="G781" t="n">
+        <v>664.84</v>
+      </c>
+      <c r="H781" t="n">
+        <v>667.5</v>
+      </c>
+      <c r="I781" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J781" t="b">
+        <v>0</v>
+      </c>
+      <c r="K781" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 664.84 &lt;= EMA21 667.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>DIVISLAB</t>
+        </is>
+      </c>
+      <c r="D782" t="n">
+        <v>9322</v>
+      </c>
+      <c r="E782" t="n">
+        <v>9784.209999999999</v>
+      </c>
+      <c r="F782" t="n">
+        <v>9784.209999999999</v>
+      </c>
+      <c r="G782" t="n">
+        <v>9310.49</v>
+      </c>
+      <c r="H782" t="n">
+        <v>9019.92</v>
+      </c>
+      <c r="I782" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J782" t="b">
+        <v>0</v>
+      </c>
+      <c r="K782" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 9322.00 &lt;= Upper 9784.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="D783" t="n">
+        <v>1165.5</v>
+      </c>
+      <c r="E783" t="n">
+        <v>1200.7</v>
+      </c>
+      <c r="F783" t="n">
+        <v>1200.7</v>
+      </c>
+      <c r="G783" t="n">
+        <v>1155.83</v>
+      </c>
+      <c r="H783" t="n">
+        <v>1165.86</v>
+      </c>
+      <c r="I783" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="J783" t="b">
+        <v>0</v>
+      </c>
+      <c r="K783" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1155.83 &lt;= EMA21 1165.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>EICHERMOT</t>
+        </is>
+      </c>
+      <c r="D784" t="n">
+        <v>7530</v>
+      </c>
+      <c r="E784" t="n">
+        <v>8268.68</v>
+      </c>
+      <c r="F784" t="n">
+        <v>8268.68</v>
+      </c>
+      <c r="G784" t="n">
+        <v>7735.32</v>
+      </c>
+      <c r="H784" t="n">
+        <v>7822.06</v>
+      </c>
+      <c r="I784" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="J784" t="b">
+        <v>0</v>
+      </c>
+      <c r="K784" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7735.32 &lt;= EMA21 7822.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>ETERNAL</t>
+        </is>
+      </c>
+      <c r="D785" t="n">
+        <v>323.5</v>
+      </c>
+      <c r="E785" t="n">
+        <v>332.95</v>
+      </c>
+      <c r="F785" t="n">
+        <v>332.95</v>
+      </c>
+      <c r="G785" t="n">
+        <v>323.56</v>
+      </c>
+      <c r="H785" t="n">
+        <v>321.37</v>
+      </c>
+      <c r="I785" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J785" t="b">
+        <v>0</v>
+      </c>
+      <c r="K785" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 323.50 &lt;= Upper 332.95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>GAIL</t>
+        </is>
+      </c>
+      <c r="D786" t="n">
+        <v>173.62</v>
+      </c>
+      <c r="E786" t="n">
+        <v>176.8</v>
+      </c>
+      <c r="F786" t="n">
+        <v>176.8</v>
+      </c>
+      <c r="G786" t="n">
+        <v>174.22</v>
+      </c>
+      <c r="H786" t="n">
+        <v>173.94</v>
+      </c>
+      <c r="I786" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="J786" t="b">
+        <v>0</v>
+      </c>
+      <c r="K786" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 173.62 &lt;= Upper 176.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>GODREJCP</t>
+        </is>
+      </c>
+      <c r="D787" t="n">
+        <v>865</v>
+      </c>
+      <c r="E787" t="n">
+        <v>961.48</v>
+      </c>
+      <c r="F787" t="n">
+        <v>961.48</v>
+      </c>
+      <c r="G787" t="n">
+        <v>878.22</v>
+      </c>
+      <c r="H787" t="n">
+        <v>909.62</v>
+      </c>
+      <c r="I787" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="J787" t="b">
+        <v>0</v>
+      </c>
+      <c r="K787" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 878.22 &lt;= EMA21 909.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>GRASIM</t>
+        </is>
+      </c>
+      <c r="D788" t="n">
+        <v>3281.9</v>
+      </c>
+      <c r="E788" t="n">
+        <v>3349.74</v>
+      </c>
+      <c r="F788" t="n">
+        <v>3349.74</v>
+      </c>
+      <c r="G788" t="n">
+        <v>3302.47</v>
+      </c>
+      <c r="H788" t="n">
+        <v>3286.59</v>
+      </c>
+      <c r="I788" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="J788" t="b">
+        <v>0</v>
+      </c>
+      <c r="K788" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3281.90 &lt;= Upper 3349.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="D789" t="n">
+        <v>1206.1</v>
+      </c>
+      <c r="E789" t="n">
+        <v>1375.06</v>
+      </c>
+      <c r="F789" t="n">
+        <v>1375.06</v>
+      </c>
+      <c r="G789" t="n">
+        <v>1258.84</v>
+      </c>
+      <c r="H789" t="n">
+        <v>1284.78</v>
+      </c>
+      <c r="I789" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J789" t="b">
+        <v>0</v>
+      </c>
+      <c r="K789" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1258.84 &lt;= EMA21 1284.78)</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>HDFCAMC</t>
+        </is>
+      </c>
+      <c r="D790" t="n">
+        <v>2403.9</v>
+      </c>
+      <c r="E790" t="n">
+        <v>2705.79</v>
+      </c>
+      <c r="F790" t="n">
+        <v>2705.79</v>
+      </c>
+      <c r="G790" t="n">
+        <v>2474.74</v>
+      </c>
+      <c r="H790" t="n">
+        <v>2520.27</v>
+      </c>
+      <c r="I790" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J790" t="b">
+        <v>0</v>
+      </c>
+      <c r="K790" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2474.74 &lt;= EMA21 2520.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="D791" t="n">
+        <v>708.25</v>
+      </c>
+      <c r="E791" t="n">
+        <v>738.48</v>
+      </c>
+      <c r="F791" t="n">
+        <v>738.48</v>
+      </c>
+      <c r="G791" t="n">
+        <v>704.51</v>
+      </c>
+      <c r="H791" t="n">
+        <v>714.47</v>
+      </c>
+      <c r="I791" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J791" t="b">
+        <v>0</v>
+      </c>
+      <c r="K791" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 704.51 &lt;= EMA21 714.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="D792" t="n">
+        <v>530</v>
+      </c>
+      <c r="E792" t="n">
+        <v>560.12</v>
+      </c>
+      <c r="F792" t="n">
+        <v>560.12</v>
+      </c>
+      <c r="G792" t="n">
+        <v>531.9299999999999</v>
+      </c>
+      <c r="H792" t="n">
+        <v>537.8</v>
+      </c>
+      <c r="I792" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="J792" t="b">
+        <v>0</v>
+      </c>
+      <c r="K792" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 531.93 &lt;= EMA21 537.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="D793" t="n">
+        <v>981.5</v>
+      </c>
+      <c r="E793" t="n">
+        <v>1065.39</v>
+      </c>
+      <c r="F793" t="n">
+        <v>1065.39</v>
+      </c>
+      <c r="G793" t="n">
+        <v>1011.48</v>
+      </c>
+      <c r="H793" t="n">
+        <v>1017.9</v>
+      </c>
+      <c r="I793" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="J793" t="b">
+        <v>0</v>
+      </c>
+      <c r="K793" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1011.48 &lt;= EMA21 1017.90)</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="D794" t="n">
+        <v>4905</v>
+      </c>
+      <c r="E794" t="n">
+        <v>5124.52</v>
+      </c>
+      <c r="F794" t="n">
+        <v>5124.52</v>
+      </c>
+      <c r="G794" t="n">
+        <v>4911.27</v>
+      </c>
+      <c r="H794" t="n">
+        <v>4880.9</v>
+      </c>
+      <c r="I794" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J794" t="b">
+        <v>0</v>
+      </c>
+      <c r="K794" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 4905.00 &lt;= Upper 5124.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="D795" t="n">
+        <v>1927</v>
+      </c>
+      <c r="E795" t="n">
+        <v>2078.66</v>
+      </c>
+      <c r="F795" t="n">
+        <v>2078.66</v>
+      </c>
+      <c r="G795" t="n">
+        <v>1963.32</v>
+      </c>
+      <c r="H795" t="n">
+        <v>1998.98</v>
+      </c>
+      <c r="I795" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J795" t="b">
+        <v>0</v>
+      </c>
+      <c r="K795" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1963.32 &lt;= EMA21 1998.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+      <c r="D796" t="n">
+        <v>576.45</v>
+      </c>
+      <c r="E796" t="n">
+        <v>628.73</v>
+      </c>
+      <c r="F796" t="n">
+        <v>628.73</v>
+      </c>
+      <c r="G796" t="n">
+        <v>592.39</v>
+      </c>
+      <c r="H796" t="n">
+        <v>589.0599999999999</v>
+      </c>
+      <c r="I796" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J796" t="b">
+        <v>0</v>
+      </c>
+      <c r="K796" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 576.45 &lt;= Upper 628.73)</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>HYUNDAI</t>
+        </is>
+      </c>
+      <c r="D797" t="n">
+        <v>2174</v>
+      </c>
+      <c r="E797" t="n">
+        <v>2267.66</v>
+      </c>
+      <c r="F797" t="n">
+        <v>2267.66</v>
+      </c>
+      <c r="G797" t="n">
+        <v>2195.03</v>
+      </c>
+      <c r="H797" t="n">
+        <v>2188.67</v>
+      </c>
+      <c r="I797" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J797" t="b">
+        <v>0</v>
+      </c>
+      <c r="K797" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 2174.00 &lt;= Upper 2267.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="D798" t="n">
+        <v>1379.3</v>
+      </c>
+      <c r="E798" t="n">
+        <v>1455.66</v>
+      </c>
+      <c r="F798" t="n">
+        <v>1455.66</v>
+      </c>
+      <c r="G798" t="n">
+        <v>1403.74</v>
+      </c>
+      <c r="H798" t="n">
+        <v>1413.97</v>
+      </c>
+      <c r="I798" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J798" t="b">
+        <v>0</v>
+      </c>
+      <c r="K798" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1403.74 &lt;= EMA21 1413.97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="D799" t="n">
+        <v>259.85</v>
+      </c>
+      <c r="E799" t="n">
+        <v>275.47</v>
+      </c>
+      <c r="F799" t="n">
+        <v>275.47</v>
+      </c>
+      <c r="G799" t="n">
+        <v>262.51</v>
+      </c>
+      <c r="H799" t="n">
+        <v>266.83</v>
+      </c>
+      <c r="I799" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J799" t="b">
+        <v>0</v>
+      </c>
+      <c r="K799" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 262.51 &lt;= EMA21 266.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>INDHOTEL</t>
+        </is>
+      </c>
+      <c r="D800" t="n">
+        <v>718.5</v>
+      </c>
+      <c r="E800" t="n">
+        <v>738.38</v>
+      </c>
+      <c r="F800" t="n">
+        <v>738.38</v>
+      </c>
+      <c r="G800" t="n">
+        <v>720.5700000000001</v>
+      </c>
+      <c r="H800" t="n">
+        <v>723.12</v>
+      </c>
+      <c r="I800" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J800" t="b">
+        <v>0</v>
+      </c>
+      <c r="K800" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 720.57 &lt;= EMA21 723.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>IOC</t>
+        </is>
+      </c>
+      <c r="D801" t="n">
+        <v>135.11</v>
+      </c>
+      <c r="E801" t="n">
+        <v>140.04</v>
+      </c>
+      <c r="F801" t="n">
+        <v>140.04</v>
+      </c>
+      <c r="G801" t="n">
+        <v>135.92</v>
+      </c>
+      <c r="H801" t="n">
+        <v>137.01</v>
+      </c>
+      <c r="I801" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J801" t="b">
+        <v>0</v>
+      </c>
+      <c r="K801" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 135.92 &lt;= EMA21 137.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>IRFC</t>
+        </is>
+      </c>
+      <c r="D802" t="n">
+        <v>81.09</v>
+      </c>
+      <c r="E802" t="n">
+        <v>88.40000000000001</v>
+      </c>
+      <c r="F802" t="n">
+        <v>88.40000000000001</v>
+      </c>
+      <c r="G802" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="H802" t="n">
+        <v>84.05</v>
+      </c>
+      <c r="I802" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J802" t="b">
+        <v>0</v>
+      </c>
+      <c r="K802" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 82.32 &lt;= EMA21 84.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="D803" t="n">
+        <v>1037.7</v>
+      </c>
+      <c r="E803" t="n">
+        <v>1186.43</v>
+      </c>
+      <c r="F803" t="n">
+        <v>1186.43</v>
+      </c>
+      <c r="G803" t="n">
+        <v>1077.73</v>
+      </c>
+      <c r="H803" t="n">
+        <v>1104.02</v>
+      </c>
+      <c r="I803" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J803" t="b">
+        <v>0</v>
+      </c>
+      <c r="K803" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1077.73 &lt;= EMA21 1104.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>INDIGO</t>
+        </is>
+      </c>
+      <c r="D804" t="n">
+        <v>4973</v>
+      </c>
+      <c r="E804" t="n">
+        <v>5355.29</v>
+      </c>
+      <c r="F804" t="n">
+        <v>5355.29</v>
+      </c>
+      <c r="G804" t="n">
+        <v>5017.37</v>
+      </c>
+      <c r="H804" t="n">
+        <v>5096.4</v>
+      </c>
+      <c r="I804" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="J804" t="b">
+        <v>0</v>
+      </c>
+      <c r="K804" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5017.37 &lt;= EMA21 5096.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>JSWSTEEL</t>
+        </is>
+      </c>
+      <c r="D805" t="n">
+        <v>1265</v>
+      </c>
+      <c r="E805" t="n">
+        <v>1349.19</v>
+      </c>
+      <c r="F805" t="n">
+        <v>1349.19</v>
+      </c>
+      <c r="G805" t="n">
+        <v>1299.69</v>
+      </c>
+      <c r="H805" t="n">
+        <v>1300.58</v>
+      </c>
+      <c r="I805" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J805" t="b">
+        <v>0</v>
+      </c>
+      <c r="K805" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1299.69 &lt;= EMA21 1300.58)</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>JINDALSTEL</t>
+        </is>
+      </c>
+      <c r="D806" t="n">
+        <v>1120.5</v>
+      </c>
+      <c r="E806" t="n">
+        <v>1198.33</v>
+      </c>
+      <c r="F806" t="n">
+        <v>1198.33</v>
+      </c>
+      <c r="G806" t="n">
+        <v>1143.37</v>
+      </c>
+      <c r="H806" t="n">
+        <v>1137.54</v>
+      </c>
+      <c r="I806" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J806" t="b">
+        <v>0</v>
+      </c>
+      <c r="K806" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1120.50 &lt;= Upper 1198.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>JIOFIN</t>
+        </is>
+      </c>
+      <c r="D807" t="n">
+        <v>229.9</v>
+      </c>
+      <c r="E807" t="n">
+        <v>251.3</v>
+      </c>
+      <c r="F807" t="n">
+        <v>251.3</v>
+      </c>
+      <c r="G807" t="n">
+        <v>234.41</v>
+      </c>
+      <c r="H807" t="n">
+        <v>238.89</v>
+      </c>
+      <c r="I807" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="J807" t="b">
+        <v>0</v>
+      </c>
+      <c r="K807" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 234.41 &lt;= EMA21 238.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="D808" t="n">
+        <v>419</v>
+      </c>
+      <c r="E808" t="n">
+        <v>437.64</v>
+      </c>
+      <c r="F808" t="n">
+        <v>437.64</v>
+      </c>
+      <c r="G808" t="n">
+        <v>418.07</v>
+      </c>
+      <c r="H808" t="n">
+        <v>412.51</v>
+      </c>
+      <c r="I808" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J808" t="b">
+        <v>0</v>
+      </c>
+      <c r="K808" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 419.00 &lt;= Upper 437.64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>LTM</t>
+        </is>
+      </c>
+      <c r="D809" t="n">
+        <v>4275</v>
+      </c>
+      <c r="E809" t="n">
+        <v>4718.38</v>
+      </c>
+      <c r="F809" t="n">
+        <v>4718.38</v>
+      </c>
+      <c r="G809" t="n">
+        <v>4434.19</v>
+      </c>
+      <c r="H809" t="n">
+        <v>4478.92</v>
+      </c>
+      <c r="I809" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J809" t="b">
+        <v>0</v>
+      </c>
+      <c r="K809" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4434.19 &lt;= EMA21 4478.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="D810" t="n">
+        <v>3930.7</v>
+      </c>
+      <c r="E810" t="n">
+        <v>4138.99</v>
+      </c>
+      <c r="F810" t="n">
+        <v>4138.99</v>
+      </c>
+      <c r="G810" t="n">
+        <v>3965.73</v>
+      </c>
+      <c r="H810" t="n">
+        <v>3991.39</v>
+      </c>
+      <c r="I810" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J810" t="b">
+        <v>0</v>
+      </c>
+      <c r="K810" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3965.73 &lt;= EMA21 3991.39)</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>LODHA</t>
+        </is>
+      </c>
+      <c r="D811" t="n">
+        <v>1116.9</v>
+      </c>
+      <c r="E811" t="n">
+        <v>1303.91</v>
+      </c>
+      <c r="F811" t="n">
+        <v>1303.91</v>
+      </c>
+      <c r="G811" t="n">
+        <v>1185.75</v>
+      </c>
+      <c r="H811" t="n">
+        <v>1205.13</v>
+      </c>
+      <c r="I811" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="J811" t="b">
+        <v>0</v>
+      </c>
+      <c r="K811" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1185.75 &lt;= EMA21 1205.13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>M&amp;M</t>
+        </is>
+      </c>
+      <c r="D812" t="n">
+        <v>3107</v>
+      </c>
+      <c r="E812" t="n">
+        <v>3533.62</v>
+      </c>
+      <c r="F812" t="n">
+        <v>3533.62</v>
+      </c>
+      <c r="G812" t="n">
+        <v>3174.63</v>
+      </c>
+      <c r="H812" t="n">
+        <v>3244.86</v>
+      </c>
+      <c r="I812" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J812" t="b">
+        <v>0</v>
+      </c>
+      <c r="K812" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3174.63 &lt;= EMA21 3244.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="D813" t="n">
+        <v>12400</v>
+      </c>
+      <c r="E813" t="n">
+        <v>14168.62</v>
+      </c>
+      <c r="F813" t="n">
+        <v>14168.62</v>
+      </c>
+      <c r="G813" t="n">
+        <v>12750.8</v>
+      </c>
+      <c r="H813" t="n">
+        <v>13094.55</v>
+      </c>
+      <c r="I813" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="J813" t="b">
+        <v>0</v>
+      </c>
+      <c r="K813" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 12750.80 &lt;= EMA21 13094.55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>MAXHEALTH</t>
+        </is>
+      </c>
+      <c r="D814" t="n">
+        <v>1037.7</v>
+      </c>
+      <c r="E814" t="n">
+        <v>1043.88</v>
+      </c>
+      <c r="F814" t="n">
+        <v>1043.88</v>
+      </c>
+      <c r="G814" t="n">
+        <v>1018.88</v>
+      </c>
+      <c r="H814" t="n">
+        <v>1021.62</v>
+      </c>
+      <c r="I814" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J814" t="b">
+        <v>0</v>
+      </c>
+      <c r="K814" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1018.88 &lt;= EMA21 1021.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>MAZDOCK</t>
+        </is>
+      </c>
+      <c r="D815" t="n">
+        <v>2339</v>
+      </c>
+      <c r="E815" t="n">
+        <v>2671.05</v>
+      </c>
+      <c r="F815" t="n">
+        <v>2671.05</v>
+      </c>
+      <c r="G815" t="n">
+        <v>2436.36</v>
+      </c>
+      <c r="H815" t="n">
+        <v>2472.92</v>
+      </c>
+      <c r="I815" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J815" t="b">
+        <v>0</v>
+      </c>
+      <c r="K815" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2436.36 &lt;= EMA21 2472.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>MUTHOOTFIN</t>
+        </is>
+      </c>
+      <c r="D816" t="n">
+        <v>2792.1</v>
+      </c>
+      <c r="E816" t="n">
+        <v>3224.19</v>
+      </c>
+      <c r="F816" t="n">
+        <v>3224.19</v>
+      </c>
+      <c r="G816" t="n">
+        <v>2881.14</v>
+      </c>
+      <c r="H816" t="n">
+        <v>2931.33</v>
+      </c>
+      <c r="I816" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="J816" t="b">
+        <v>0</v>
+      </c>
+      <c r="K816" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2881.14 &lt;= EMA21 2931.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="D817" t="n">
+        <v>333.4</v>
+      </c>
+      <c r="E817" t="n">
+        <v>339.17</v>
+      </c>
+      <c r="F817" t="n">
+        <v>339.17</v>
+      </c>
+      <c r="G817" t="n">
+        <v>332.37</v>
+      </c>
+      <c r="H817" t="n">
+        <v>333.14</v>
+      </c>
+      <c r="I817" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J817" t="b">
+        <v>0</v>
+      </c>
+      <c r="K817" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 332.37 &lt;= EMA21 333.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="D818" t="n">
+        <v>1383.3</v>
+      </c>
+      <c r="E818" t="n">
+        <v>1509.16</v>
+      </c>
+      <c r="F818" t="n">
+        <v>1509.16</v>
+      </c>
+      <c r="G818" t="n">
+        <v>1406.97</v>
+      </c>
+      <c r="H818" t="n">
+        <v>1433.45</v>
+      </c>
+      <c r="I818" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="J818" t="b">
+        <v>0</v>
+      </c>
+      <c r="K818" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1406.97 &lt;= EMA21 1433.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="D819" t="n">
+        <v>232.5</v>
+      </c>
+      <c r="E819" t="n">
+        <v>239.51</v>
+      </c>
+      <c r="F819" t="n">
+        <v>239.51</v>
+      </c>
+      <c r="G819" t="n">
+        <v>234.54</v>
+      </c>
+      <c r="H819" t="n">
+        <v>235.37</v>
+      </c>
+      <c r="I819" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="J819" t="b">
+        <v>0</v>
+      </c>
+      <c r="K819" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 234.54 &lt;= EMA21 235.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>PIDILITIND</t>
+        </is>
+      </c>
+      <c r="D820" t="n">
+        <v>1566.9</v>
+      </c>
+      <c r="E820" t="n">
+        <v>1707.64</v>
+      </c>
+      <c r="F820" t="n">
+        <v>1707.64</v>
+      </c>
+      <c r="G820" t="n">
+        <v>1597</v>
+      </c>
+      <c r="H820" t="n">
+        <v>1619.73</v>
+      </c>
+      <c r="I820" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="J820" t="b">
+        <v>0</v>
+      </c>
+      <c r="K820" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1597.00 &lt;= EMA21 1619.73)</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>PFC</t>
+        </is>
+      </c>
+      <c r="D821" t="n">
+        <v>353.45</v>
+      </c>
+      <c r="E821" t="n">
+        <v>373.59</v>
+      </c>
+      <c r="F821" t="n">
+        <v>373.59</v>
+      </c>
+      <c r="G821" t="n">
+        <v>352.94</v>
+      </c>
+      <c r="H821" t="n">
+        <v>360.12</v>
+      </c>
+      <c r="I821" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J821" t="b">
+        <v>0</v>
+      </c>
+      <c r="K821" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 352.94 &lt;= EMA21 360.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="D822" t="n">
+        <v>269.1</v>
+      </c>
+      <c r="E822" t="n">
+        <v>272.41</v>
+      </c>
+      <c r="F822" t="n">
+        <v>272.41</v>
+      </c>
+      <c r="G822" t="n">
+        <v>267.58</v>
+      </c>
+      <c r="H822" t="n">
+        <v>268.76</v>
+      </c>
+      <c r="I822" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="J822" t="b">
+        <v>0</v>
+      </c>
+      <c r="K822" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 267.58 &lt;= EMA21 268.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="D823" t="n">
+        <v>116.75</v>
+      </c>
+      <c r="E823" t="n">
+        <v>118.09</v>
+      </c>
+      <c r="F823" t="n">
+        <v>118.09</v>
+      </c>
+      <c r="G823" t="n">
+        <v>116.26</v>
+      </c>
+      <c r="H823" t="n">
+        <v>115.76</v>
+      </c>
+      <c r="I823" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J823" t="b">
+        <v>0</v>
+      </c>
+      <c r="K823" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 116.75 &lt;= Upper 118.09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="D824" t="n">
+        <v>312.7</v>
+      </c>
+      <c r="E824" t="n">
+        <v>339.4</v>
+      </c>
+      <c r="F824" t="n">
+        <v>339.4</v>
+      </c>
+      <c r="G824" t="n">
+        <v>316.38</v>
+      </c>
+      <c r="H824" t="n">
+        <v>323.82</v>
+      </c>
+      <c r="I824" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J824" t="b">
+        <v>0</v>
+      </c>
+      <c r="K824" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 316.38 &lt;= EMA21 323.82)</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="D825" t="n">
+        <v>1257.5</v>
+      </c>
+      <c r="E825" t="n">
+        <v>1337.45</v>
+      </c>
+      <c r="F825" t="n">
+        <v>1337.45</v>
+      </c>
+      <c r="G825" t="n">
+        <v>1286.91</v>
+      </c>
+      <c r="H825" t="n">
+        <v>1296.38</v>
+      </c>
+      <c r="I825" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J825" t="b">
+        <v>0</v>
+      </c>
+      <c r="K825" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1286.91 &lt;= EMA21 1296.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="D826" t="n">
+        <v>1684.7</v>
+      </c>
+      <c r="E826" t="n">
+        <v>1818.08</v>
+      </c>
+      <c r="F826" t="n">
+        <v>1818.08</v>
+      </c>
+      <c r="G826" t="n">
+        <v>1714.46</v>
+      </c>
+      <c r="H826" t="n">
+        <v>1746.98</v>
+      </c>
+      <c r="I826" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="J826" t="b">
+        <v>0</v>
+      </c>
+      <c r="K826" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1714.46 &lt;= EMA21 1746.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>MOTHERSON</t>
+        </is>
+      </c>
+      <c r="D827" t="n">
+        <v>164.45</v>
+      </c>
+      <c r="E827" t="n">
+        <v>172.22</v>
+      </c>
+      <c r="F827" t="n">
+        <v>172.22</v>
+      </c>
+      <c r="G827" t="n">
+        <v>163.91</v>
+      </c>
+      <c r="H827" t="n">
+        <v>163.63</v>
+      </c>
+      <c r="I827" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J827" t="b">
+        <v>0</v>
+      </c>
+      <c r="K827" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 164.45 &lt;= Upper 172.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="D828" t="n">
+        <v>22570</v>
+      </c>
+      <c r="E828" t="n">
+        <v>25190.51</v>
+      </c>
+      <c r="F828" t="n">
+        <v>25190.51</v>
+      </c>
+      <c r="G828" t="n">
+        <v>23235.17</v>
+      </c>
+      <c r="H828" t="n">
+        <v>23911.45</v>
+      </c>
+      <c r="I828" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J828" t="b">
+        <v>0</v>
+      </c>
+      <c r="K828" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 23235.17 &lt;= EMA21 23911.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>SHRIRAMFIN</t>
+        </is>
+      </c>
+      <c r="D829" t="n">
+        <v>1028.6</v>
+      </c>
+      <c r="E829" t="n">
+        <v>1162.54</v>
+      </c>
+      <c r="F829" t="n">
+        <v>1162.54</v>
+      </c>
+      <c r="G829" t="n">
+        <v>1045.38</v>
+      </c>
+      <c r="H829" t="n">
+        <v>1065.7</v>
+      </c>
+      <c r="I829" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J829" t="b">
+        <v>0</v>
+      </c>
+      <c r="K829" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1045.38 &lt;= EMA21 1065.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>ENRIN</t>
+        </is>
+      </c>
+      <c r="D830" t="n">
+        <v>3181.3</v>
+      </c>
+      <c r="E830" t="n">
+        <v>3616.86</v>
+      </c>
+      <c r="F830" t="n">
+        <v>3616.86</v>
+      </c>
+      <c r="G830" t="n">
+        <v>3191.39</v>
+      </c>
+      <c r="H830" t="n">
+        <v>3259.74</v>
+      </c>
+      <c r="I830" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J830" t="b">
+        <v>0</v>
+      </c>
+      <c r="K830" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3191.39 &lt;= EMA21 3259.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+      <c r="D831" t="n">
+        <v>3957</v>
+      </c>
+      <c r="E831" t="n">
+        <v>4132.57</v>
+      </c>
+      <c r="F831" t="n">
+        <v>4132.57</v>
+      </c>
+      <c r="G831" t="n">
+        <v>3972.69</v>
+      </c>
+      <c r="H831" t="n">
+        <v>3965.16</v>
+      </c>
+      <c r="I831" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J831" t="b">
+        <v>0</v>
+      </c>
+      <c r="K831" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3957.00 &lt;= Upper 4132.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>SOLARINDS</t>
+        </is>
+      </c>
+      <c r="D832" t="n">
+        <v>22290</v>
+      </c>
+      <c r="E832" t="n">
+        <v>22809.23</v>
+      </c>
+      <c r="F832" t="n">
+        <v>22809.23</v>
+      </c>
+      <c r="G832" t="n">
+        <v>21758.36</v>
+      </c>
+      <c r="H832" t="n">
+        <v>20904.42</v>
+      </c>
+      <c r="I832" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J832" t="b">
+        <v>0</v>
+      </c>
+      <c r="K832" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 22290.00 &lt;= Upper 22809.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="D833" t="n">
+        <v>995.7</v>
+      </c>
+      <c r="E833" t="n">
+        <v>1075.39</v>
+      </c>
+      <c r="F833" t="n">
+        <v>1075.39</v>
+      </c>
+      <c r="G833" t="n">
+        <v>1013.32</v>
+      </c>
+      <c r="H833" t="n">
+        <v>1027.66</v>
+      </c>
+      <c r="I833" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J833" t="b">
+        <v>0</v>
+      </c>
+      <c r="K833" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1013.32 &lt;= EMA21 1027.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="D834" t="n">
+        <v>1840</v>
+      </c>
+      <c r="E834" t="n">
+        <v>1963.23</v>
+      </c>
+      <c r="F834" t="n">
+        <v>1963.23</v>
+      </c>
+      <c r="G834" t="n">
+        <v>1882.15</v>
+      </c>
+      <c r="H834" t="n">
+        <v>1902.01</v>
+      </c>
+      <c r="I834" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J834" t="b">
+        <v>0</v>
+      </c>
+      <c r="K834" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1882.15 &lt;= EMA21 1902.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>TVSMOTOR</t>
+        </is>
+      </c>
+      <c r="D835" t="n">
+        <v>4125</v>
+      </c>
+      <c r="E835" t="n">
+        <v>4521.64</v>
+      </c>
+      <c r="F835" t="n">
+        <v>4521.64</v>
+      </c>
+      <c r="G835" t="n">
+        <v>4172.4</v>
+      </c>
+      <c r="H835" t="n">
+        <v>4215.96</v>
+      </c>
+      <c r="I835" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="J835" t="b">
+        <v>0</v>
+      </c>
+      <c r="K835" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4172.40 &lt;= EMA21 4215.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>TATACAP</t>
+        </is>
+      </c>
+      <c r="D836" t="n">
+        <v>362.9</v>
+      </c>
+      <c r="E836" t="n">
+        <v>376.61</v>
+      </c>
+      <c r="F836" t="n">
+        <v>376.61</v>
+      </c>
+      <c r="G836" t="n">
+        <v>366.4</v>
+      </c>
+      <c r="H836" t="n">
+        <v>366.47</v>
+      </c>
+      <c r="I836" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J836" t="b">
+        <v>0</v>
+      </c>
+      <c r="K836" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 366.40 &lt;= EMA21 366.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="D837" t="n">
+        <v>2200.8</v>
+      </c>
+      <c r="E837" t="n">
+        <v>2394.77</v>
+      </c>
+      <c r="F837" t="n">
+        <v>2394.77</v>
+      </c>
+      <c r="G837" t="n">
+        <v>2254.69</v>
+      </c>
+      <c r="H837" t="n">
+        <v>2286.71</v>
+      </c>
+      <c r="I837" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J837" t="b">
+        <v>0</v>
+      </c>
+      <c r="K837" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2254.69 &lt;= EMA21 2286.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>TATACONSUM</t>
+        </is>
+      </c>
+      <c r="D838" t="n">
+        <v>991</v>
+      </c>
+      <c r="E838" t="n">
+        <v>1084.99</v>
+      </c>
+      <c r="F838" t="n">
+        <v>1084.99</v>
+      </c>
+      <c r="G838" t="n">
+        <v>1010.97</v>
+      </c>
+      <c r="H838" t="n">
+        <v>1032.19</v>
+      </c>
+      <c r="I838" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J838" t="b">
+        <v>0</v>
+      </c>
+      <c r="K838" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1010.97 &lt;= EMA21 1032.19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>TMCV</t>
+        </is>
+      </c>
+      <c r="D839" t="n">
+        <v>434.55</v>
+      </c>
+      <c r="E839" t="n">
+        <v>491.42</v>
+      </c>
+      <c r="F839" t="n">
+        <v>491.42</v>
+      </c>
+      <c r="G839" t="n">
+        <v>450.34</v>
+      </c>
+      <c r="H839" t="n">
+        <v>455.2</v>
+      </c>
+      <c r="I839" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J839" t="b">
+        <v>0</v>
+      </c>
+      <c r="K839" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 450.34 &lt;= EMA21 455.20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>TMPV</t>
+        </is>
+      </c>
+      <c r="D840" t="n">
+        <v>301.1</v>
+      </c>
+      <c r="E840" t="n">
+        <v>328.33</v>
+      </c>
+      <c r="F840" t="n">
+        <v>328.33</v>
+      </c>
+      <c r="G840" t="n">
+        <v>306.56</v>
+      </c>
+      <c r="H840" t="n">
+        <v>314.37</v>
+      </c>
+      <c r="I840" t="n">
+        <v>1</v>
+      </c>
+      <c r="J840" t="b">
+        <v>0</v>
+      </c>
+      <c r="K840" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 306.56 &lt;= EMA21 314.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>TATAPOWER</t>
+        </is>
+      </c>
+      <c r="D841" t="n">
+        <v>364.65</v>
+      </c>
+      <c r="E841" t="n">
+        <v>386.47</v>
+      </c>
+      <c r="F841" t="n">
+        <v>386.47</v>
+      </c>
+      <c r="G841" t="n">
+        <v>365.32</v>
+      </c>
+      <c r="H841" t="n">
+        <v>367.36</v>
+      </c>
+      <c r="I841" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="J841" t="b">
+        <v>0</v>
+      </c>
+      <c r="K841" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 365.32 &lt;= EMA21 367.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="D842" t="n">
+        <v>183</v>
+      </c>
+      <c r="E842" t="n">
+        <v>189.16</v>
+      </c>
+      <c r="F842" t="n">
+        <v>189.16</v>
+      </c>
+      <c r="G842" t="n">
+        <v>185.57</v>
+      </c>
+      <c r="H842" t="n">
+        <v>185.89</v>
+      </c>
+      <c r="I842" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J842" t="b">
+        <v>0</v>
+      </c>
+      <c r="K842" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 185.57 &lt;= EMA21 185.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>TECHM</t>
+        </is>
+      </c>
+      <c r="D843" t="n">
+        <v>1541</v>
+      </c>
+      <c r="E843" t="n">
+        <v>1656.32</v>
+      </c>
+      <c r="F843" t="n">
+        <v>1656.32</v>
+      </c>
+      <c r="G843" t="n">
+        <v>1560.35</v>
+      </c>
+      <c r="H843" t="n">
+        <v>1579.68</v>
+      </c>
+      <c r="I843" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J843" t="b">
+        <v>0</v>
+      </c>
+      <c r="K843" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1560.35 &lt;= EMA21 1579.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>TITAN</t>
+        </is>
+      </c>
+      <c r="D844" t="n">
+        <v>5009.5</v>
+      </c>
+      <c r="E844" t="n">
+        <v>5161.3</v>
+      </c>
+      <c r="F844" t="n">
+        <v>5161.3</v>
+      </c>
+      <c r="G844" t="n">
+        <v>5025.8</v>
+      </c>
+      <c r="H844" t="n">
+        <v>5022.47</v>
+      </c>
+      <c r="I844" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J844" t="b">
+        <v>0</v>
+      </c>
+      <c r="K844" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 5009.50 &lt;= Upper 5161.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>TORNTPHARM</t>
+        </is>
+      </c>
+      <c r="D845" t="n">
+        <v>4965.5</v>
+      </c>
+      <c r="E845" t="n">
+        <v>5068.18</v>
+      </c>
+      <c r="F845" t="n">
+        <v>5068.18</v>
+      </c>
+      <c r="G845" t="n">
+        <v>4944.35</v>
+      </c>
+      <c r="H845" t="n">
+        <v>4944.08</v>
+      </c>
+      <c r="I845" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J845" t="b">
+        <v>0</v>
+      </c>
+      <c r="K845" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 4965.50 &lt;= Upper 5068.18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="D846" t="n">
+        <v>2802.4</v>
+      </c>
+      <c r="E846" t="n">
+        <v>2989.58</v>
+      </c>
+      <c r="F846" t="n">
+        <v>2989.58</v>
+      </c>
+      <c r="G846" t="n">
+        <v>2830.16</v>
+      </c>
+      <c r="H846" t="n">
+        <v>2873.65</v>
+      </c>
+      <c r="I846" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J846" t="b">
+        <v>0</v>
+      </c>
+      <c r="K846" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2830.16 &lt;= EMA21 2873.65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="D847" t="n">
+        <v>11000</v>
+      </c>
+      <c r="E847" t="n">
+        <v>11899.48</v>
+      </c>
+      <c r="F847" t="n">
+        <v>11899.48</v>
+      </c>
+      <c r="G847" t="n">
+        <v>11150.11</v>
+      </c>
+      <c r="H847" t="n">
+        <v>11348.94</v>
+      </c>
+      <c r="I847" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J847" t="b">
+        <v>0</v>
+      </c>
+      <c r="K847" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11150.11 &lt;= EMA21 11348.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="D848" t="n">
+        <v>178.1</v>
+      </c>
+      <c r="E848" t="n">
+        <v>191.02</v>
+      </c>
+      <c r="F848" t="n">
+        <v>191.02</v>
+      </c>
+      <c r="G848" t="n">
+        <v>183.02</v>
+      </c>
+      <c r="H848" t="n">
+        <v>183.36</v>
+      </c>
+      <c r="I848" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J848" t="b">
+        <v>0</v>
+      </c>
+      <c r="K848" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 183.02 &lt;= EMA21 183.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>UNITDSPR</t>
+        </is>
+      </c>
+      <c r="D849" t="n">
+        <v>1395</v>
+      </c>
+      <c r="E849" t="n">
+        <v>1598.82</v>
+      </c>
+      <c r="F849" t="n">
+        <v>1598.82</v>
+      </c>
+      <c r="G849" t="n">
+        <v>1438.19</v>
+      </c>
+      <c r="H849" t="n">
+        <v>1468.95</v>
+      </c>
+      <c r="I849" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J849" t="b">
+        <v>0</v>
+      </c>
+      <c r="K849" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1438.19 &lt;= EMA21 1468.95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="D850" t="n">
+        <v>416.5</v>
+      </c>
+      <c r="E850" t="n">
+        <v>444.46</v>
+      </c>
+      <c r="F850" t="n">
+        <v>444.46</v>
+      </c>
+      <c r="G850" t="n">
+        <v>411.52</v>
+      </c>
+      <c r="H850" t="n">
+        <v>419.37</v>
+      </c>
+      <c r="I850" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="J850" t="b">
+        <v>0</v>
+      </c>
+      <c r="K850" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 411.52 &lt;= EMA21 419.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>VEDL</t>
+        </is>
+      </c>
+      <c r="D851" t="n">
+        <v>263.7</v>
+      </c>
+      <c r="E851" t="n">
+        <v>286.99</v>
+      </c>
+      <c r="F851" t="n">
+        <v>286.99</v>
+      </c>
+      <c r="G851" t="n">
+        <v>270.44</v>
+      </c>
+      <c r="H851" t="n">
+        <v>272.22</v>
+      </c>
+      <c r="I851" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J851" t="b">
+        <v>0</v>
+      </c>
+      <c r="K851" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 270.44 &lt;= EMA21 272.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="D852" t="n">
+        <v>167.4</v>
+      </c>
+      <c r="E852" t="n">
+        <v>187.56</v>
+      </c>
+      <c r="F852" t="n">
+        <v>187.56</v>
+      </c>
+      <c r="G852" t="n">
+        <v>171.75</v>
+      </c>
+      <c r="H852" t="n">
+        <v>175.66</v>
+      </c>
+      <c r="I852" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J852" t="b">
+        <v>0</v>
+      </c>
+      <c r="K852" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 171.75 &lt;= EMA21 175.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>ZYDUSLIFE</t>
+        </is>
+      </c>
+      <c r="D853" t="n">
+        <v>1119.1</v>
+      </c>
+      <c r="E853" t="n">
+        <v>1190.18</v>
+      </c>
+      <c r="F853" t="n">
+        <v>1190.18</v>
+      </c>
+      <c r="G853" t="n">
+        <v>1134.64</v>
+      </c>
+      <c r="H853" t="n">
+        <v>1138.08</v>
+      </c>
+      <c r="I853" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J853" t="b">
+        <v>0</v>
+      </c>
+      <c r="K853" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1134.64 &lt;= EMA21 1138.08)</t>
         </is>
       </c>
     </row>
@@ -33119,7 +37419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33200,10 +37500,10 @@
         <v>19685.95</v>
       </c>
       <c r="F2" t="n">
-        <v>432</v>
+        <v>426.4</v>
       </c>
       <c r="G2" t="n">
-        <v>3.14</v>
+        <v>1.8</v>
       </c>
       <c r="H2" t="n">
         <v>416.67</v>
@@ -33212,7 +37512,7 @@
         <v>436.2999877929688</v>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -33241,10 +37541,10 @@
         <v>19525</v>
       </c>
       <c r="F3" t="n">
-        <v>1768</v>
+        <v>1764.6</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.39</v>
+        <v>-0.59</v>
       </c>
       <c r="H3" t="n">
         <v>1699.9</v>
@@ -33253,7 +37553,7 @@
         <v>1780</v>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -33282,10 +37582,10 @@
         <v>19985.7</v>
       </c>
       <c r="F4" t="n">
-        <v>213.5</v>
+        <v>209.97</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.65</v>
+        <v>-2.29</v>
       </c>
       <c r="H4" t="n">
         <v>205.59</v>
@@ -33294,50 +37594,9 @@
         <v>215.2799987792969</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K4" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>CGPOWER</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>926.95</v>
-      </c>
-      <c r="D5" t="n">
-        <v>21</v>
-      </c>
-      <c r="E5" t="n">
-        <v>19465.95</v>
-      </c>
-      <c r="F5" t="n">
-        <v>914.55</v>
-      </c>
-      <c r="G5" t="n">
-        <v>-1.34</v>
-      </c>
-      <c r="H5" t="n">
-        <v>889.11</v>
-      </c>
-      <c r="I5" t="n">
-        <v>931</v>
-      </c>
-      <c r="J5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -33354,7 +37613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34235,6 +38494,57 @@
         </is>
       </c>
       <c r="M18" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>926.95</v>
+      </c>
+      <c r="E19" t="n">
+        <v>889.11</v>
+      </c>
+      <c r="F19" t="n">
+        <v>21</v>
+      </c>
+      <c r="G19" t="n">
+        <v>19465.95</v>
+      </c>
+      <c r="H19" t="n">
+        <v>-4.082</v>
+      </c>
+      <c r="I19" t="n">
+        <v>-4.382</v>
+      </c>
+      <c r="J19" t="n">
+        <v>-853</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>HARD_STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>2</v>
+      </c>
+      <c r="M19" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -34251,7 +38561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K147"/>
+  <dimension ref="A1:K148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39488,6 +43798,55 @@
       <c r="K147" t="inlineStr">
         <is>
           <t>Entry Breakout</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-09-11 19:57:31</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>0380701553</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F148" t="n">
+        <v>889.11</v>
+      </c>
+      <c r="G148" t="n">
+        <v>889.11</v>
+      </c>
+      <c r="H148" t="n">
+        <v>0</v>
+      </c>
+      <c r="I148" t="n">
+        <v>21</v>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>HARD_STOP_LOSS</t>
         </is>
       </c>
     </row>
@@ -39570,7 +43929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39983,6 +44342,39 @@
         <v>4</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>19:57:32</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>138772.28</v>
+      </c>
+      <c r="D13" t="n">
+        <v>59196.65</v>
+      </c>
+      <c r="E13" t="n">
+        <v>197968.93</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-1945.43</v>
+      </c>
+      <c r="G13" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="H13" t="n">
+        <v>18</v>
+      </c>
+      <c r="I13" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>